<commit_message>
📊 Horarios actualizados Línea 141 - 3025
</commit_message>
<xml_diff>
--- a/data/horarios-141-2026-05-17.xlsx
+++ b/data/horarios-141-2026-05-17.xlsx
@@ -419,7 +419,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E8"/>
+  <dimension ref="A1:E17"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -432,14 +432,14 @@
     <row r="2">
       <c r="A2" s="1" t="inlineStr">
         <is>
-          <t>Última actualización: 02:39:13</t>
+          <t>Última actualización: 04:59:10</t>
         </is>
       </c>
     </row>
     <row r="3">
       <c r="A3" s="1" t="inlineStr">
         <is>
-          <t>Total filas: 3</t>
+          <t>Total filas: 12</t>
         </is>
       </c>
     </row>
@@ -473,21 +473,21 @@
     <row r="6">
       <c r="A6" t="inlineStr">
         <is>
-          <t>02:39:13</t>
+          <t>04:59:10</t>
         </is>
       </c>
       <c r="B6" t="inlineStr">
         <is>
-          <t>03:02</t>
+          <t>05:17</t>
         </is>
       </c>
       <c r="C6" t="inlineStr">
         <is>
-          <t>15_ABASTO</t>
+          <t>17_ROMERO</t>
         </is>
       </c>
       <c r="D6" t="n">
-        <v>23</v>
+        <v>18</v>
       </c>
       <c r="E6" t="inlineStr">
         <is>
@@ -498,21 +498,21 @@
     <row r="7">
       <c r="A7" t="inlineStr">
         <is>
-          <t>02:39:13</t>
+          <t>04:59:10</t>
         </is>
       </c>
       <c r="B7" t="inlineStr">
         <is>
-          <t>03:48</t>
+          <t>05:22</t>
         </is>
       </c>
       <c r="C7" t="inlineStr">
         <is>
-          <t>14_ABASTO</t>
+          <t>23_HERNANDEZ</t>
         </is>
       </c>
       <c r="D7" t="n">
-        <v>69</v>
+        <v>23</v>
       </c>
       <c r="E7" t="inlineStr">
         <is>
@@ -523,23 +523,248 @@
     <row r="8">
       <c r="A8" t="inlineStr">
         <is>
-          <t>02:39:13</t>
+          <t>04:59:10</t>
         </is>
       </c>
       <c r="B8" t="inlineStr">
         <is>
-          <t>04:02</t>
+          <t>05:44</t>
         </is>
       </c>
       <c r="C8" t="inlineStr">
         <is>
-          <t>81_EL PELIGRO</t>
+          <t>14_ABASTO</t>
         </is>
       </c>
       <c r="D8" t="n">
-        <v>83</v>
+        <v>45</v>
       </c>
       <c r="E8" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" t="inlineStr">
+        <is>
+          <t>04:59:10</t>
+        </is>
+      </c>
+      <c r="B9" t="inlineStr">
+        <is>
+          <t>05:47</t>
+        </is>
+      </c>
+      <c r="C9" t="inlineStr">
+        <is>
+          <t>15_ABASTO</t>
+        </is>
+      </c>
+      <c r="D9" t="n">
+        <v>48</v>
+      </c>
+      <c r="E9" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" t="inlineStr">
+        <is>
+          <t>04:59:10</t>
+        </is>
+      </c>
+      <c r="B10" t="inlineStr">
+        <is>
+          <t>06:01</t>
+        </is>
+      </c>
+      <c r="C10" t="inlineStr">
+        <is>
+          <t>16_SANTA ANA</t>
+        </is>
+      </c>
+      <c r="D10" t="n">
+        <v>62</v>
+      </c>
+      <c r="E10" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" t="inlineStr">
+        <is>
+          <t>04:59:10</t>
+        </is>
+      </c>
+      <c r="B11" t="inlineStr">
+        <is>
+          <t>06:09</t>
+        </is>
+      </c>
+      <c r="C11" t="inlineStr">
+        <is>
+          <t>10_OLMOS</t>
+        </is>
+      </c>
+      <c r="D11" t="n">
+        <v>70</v>
+      </c>
+      <c r="E11" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="12">
+      <c r="A12" t="inlineStr">
+        <is>
+          <t>04:59:10</t>
+        </is>
+      </c>
+      <c r="B12" t="inlineStr">
+        <is>
+          <t>06:12</t>
+        </is>
+      </c>
+      <c r="C12" t="inlineStr">
+        <is>
+          <t>215A_EL PATO</t>
+        </is>
+      </c>
+      <c r="D12" t="n">
+        <v>73</v>
+      </c>
+      <c r="E12" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="13">
+      <c r="A13" t="inlineStr">
+        <is>
+          <t>04:59:10</t>
+        </is>
+      </c>
+      <c r="B13" t="inlineStr">
+        <is>
+          <t>06:30</t>
+        </is>
+      </c>
+      <c r="C13" t="inlineStr">
+        <is>
+          <t>23_HERNANDEZ</t>
+        </is>
+      </c>
+      <c r="D13" t="n">
+        <v>91</v>
+      </c>
+      <c r="E13" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="14">
+      <c r="A14" t="inlineStr">
+        <is>
+          <t>04:59:10</t>
+        </is>
+      </c>
+      <c r="B14" t="inlineStr">
+        <is>
+          <t>06:36</t>
+        </is>
+      </c>
+      <c r="C14" t="inlineStr">
+        <is>
+          <t>11_ETCHEVERRY</t>
+        </is>
+      </c>
+      <c r="D14" t="n">
+        <v>97</v>
+      </c>
+      <c r="E14" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="15">
+      <c r="A15" t="inlineStr">
+        <is>
+          <t>04:59:10</t>
+        </is>
+      </c>
+      <c r="B15" t="inlineStr">
+        <is>
+          <t>06:39</t>
+        </is>
+      </c>
+      <c r="C15" t="inlineStr">
+        <is>
+          <t>225_C ROCA-H SUR</t>
+        </is>
+      </c>
+      <c r="D15" t="n">
+        <v>100</v>
+      </c>
+      <c r="E15" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="16">
+      <c r="A16" t="inlineStr">
+        <is>
+          <t>04:59:10</t>
+        </is>
+      </c>
+      <c r="B16" t="inlineStr">
+        <is>
+          <t>06:41</t>
+        </is>
+      </c>
+      <c r="C16" t="inlineStr">
+        <is>
+          <t>17X38_ROMERO</t>
+        </is>
+      </c>
+      <c r="D16" t="n">
+        <v>102</v>
+      </c>
+      <c r="E16" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="17">
+      <c r="A17" t="inlineStr">
+        <is>
+          <t>04:59:10</t>
+        </is>
+      </c>
+      <c r="B17" t="inlineStr">
+        <is>
+          <t>06:41</t>
+        </is>
+      </c>
+      <c r="C17" t="inlineStr">
+        <is>
+          <t>16_SANTA ANA</t>
+        </is>
+      </c>
+      <c r="D17" t="n">
+        <v>102</v>
+      </c>
+      <c r="E17" t="inlineStr">
         <is>
           <t>LP1912</t>
         </is>
@@ -556,7 +781,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:A3"/>
+  <dimension ref="A1:E6"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -569,14 +794,66 @@
     <row r="2">
       <c r="A2" s="1" t="inlineStr">
         <is>
-          <t>Última actualización: 02:39:13</t>
+          <t>Última actualización: 04:59:10</t>
         </is>
       </c>
     </row>
     <row r="3">
       <c r="A3" s="1" t="inlineStr">
         <is>
-          <t>Total filas: 0</t>
+          <t>Total filas: 1</t>
+        </is>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" t="inlineStr">
+        <is>
+          <t>Hora_Scrap</t>
+        </is>
+      </c>
+      <c r="B5" t="inlineStr">
+        <is>
+          <t>Hora_Llegada</t>
+        </is>
+      </c>
+      <c r="C5" t="inlineStr">
+        <is>
+          <t>Linea</t>
+        </is>
+      </c>
+      <c r="D5" t="inlineStr">
+        <is>
+          <t>Minutos</t>
+        </is>
+      </c>
+      <c r="E5" t="inlineStr">
+        <is>
+          <t>Parada</t>
+        </is>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" t="inlineStr">
+        <is>
+          <t>04:59:10</t>
+        </is>
+      </c>
+      <c r="B6" t="inlineStr">
+        <is>
+          <t>06:12</t>
+        </is>
+      </c>
+      <c r="C6" t="inlineStr">
+        <is>
+          <t>215A_EL PATO</t>
+        </is>
+      </c>
+      <c r="D6" t="n">
+        <v>73</v>
+      </c>
+      <c r="E6" t="inlineStr">
+        <is>
+          <t>LP1912</t>
         </is>
       </c>
     </row>
@@ -604,7 +881,7 @@
     <row r="2">
       <c r="A2" s="1" t="inlineStr">
         <is>
-          <t>Última actualización: 02:39:13</t>
+          <t>Última actualización: 04:59:10</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
📊 Horarios actualizados Línea 141 - 3026
</commit_message>
<xml_diff>
--- a/data/horarios-141-2026-05-17.xlsx
+++ b/data/horarios-141-2026-05-17.xlsx
@@ -419,7 +419,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E17"/>
+  <dimension ref="A1:E21"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -432,14 +432,14 @@
     <row r="2">
       <c r="A2" s="1" t="inlineStr">
         <is>
-          <t>Última actualización: 04:59:10</t>
+          <t>Última actualización: 06:46:02</t>
         </is>
       </c>
     </row>
     <row r="3">
       <c r="A3" s="1" t="inlineStr">
         <is>
-          <t>Total filas: 12</t>
+          <t>Total filas: 16</t>
         </is>
       </c>
     </row>
@@ -473,21 +473,21 @@
     <row r="6">
       <c r="A6" t="inlineStr">
         <is>
-          <t>04:59:10</t>
+          <t>06:46:02</t>
         </is>
       </c>
       <c r="B6" t="inlineStr">
         <is>
-          <t>05:17</t>
+          <t>06:59</t>
         </is>
       </c>
       <c r="C6" t="inlineStr">
         <is>
-          <t>17_ROMERO</t>
+          <t>225_GOMEZ</t>
         </is>
       </c>
       <c r="D6" t="n">
-        <v>18</v>
+        <v>13</v>
       </c>
       <c r="E6" t="inlineStr">
         <is>
@@ -498,21 +498,21 @@
     <row r="7">
       <c r="A7" t="inlineStr">
         <is>
-          <t>04:59:10</t>
+          <t>06:46:02</t>
         </is>
       </c>
       <c r="B7" t="inlineStr">
         <is>
-          <t>05:22</t>
+          <t>07:03</t>
         </is>
       </c>
       <c r="C7" t="inlineStr">
         <is>
-          <t>23_HERNANDEZ</t>
+          <t>215A_EL PATO</t>
         </is>
       </c>
       <c r="D7" t="n">
-        <v>23</v>
+        <v>17</v>
       </c>
       <c r="E7" t="inlineStr">
         <is>
@@ -523,21 +523,21 @@
     <row r="8">
       <c r="A8" t="inlineStr">
         <is>
-          <t>04:59:10</t>
+          <t>06:46:02</t>
         </is>
       </c>
       <c r="B8" t="inlineStr">
         <is>
-          <t>05:44</t>
+          <t>07:21</t>
         </is>
       </c>
       <c r="C8" t="inlineStr">
         <is>
-          <t>14_ABASTO</t>
+          <t>16_SANTA ANA</t>
         </is>
       </c>
       <c r="D8" t="n">
-        <v>45</v>
+        <v>35</v>
       </c>
       <c r="E8" t="inlineStr">
         <is>
@@ -548,21 +548,21 @@
     <row r="9">
       <c r="A9" t="inlineStr">
         <is>
-          <t>04:59:10</t>
+          <t>06:46:02</t>
         </is>
       </c>
       <c r="B9" t="inlineStr">
         <is>
-          <t>05:47</t>
+          <t>07:27</t>
         </is>
       </c>
       <c r="C9" t="inlineStr">
         <is>
-          <t>15_ABASTO</t>
+          <t>14_ABASTO</t>
         </is>
       </c>
       <c r="D9" t="n">
-        <v>48</v>
+        <v>41</v>
       </c>
       <c r="E9" t="inlineStr">
         <is>
@@ -573,21 +573,21 @@
     <row r="10">
       <c r="A10" t="inlineStr">
         <is>
-          <t>04:59:10</t>
+          <t>06:46:02</t>
         </is>
       </c>
       <c r="B10" t="inlineStr">
         <is>
-          <t>06:01</t>
+          <t>07:27</t>
         </is>
       </c>
       <c r="C10" t="inlineStr">
         <is>
-          <t>16_SANTA ANA</t>
+          <t>23_HERNANDEZ</t>
         </is>
       </c>
       <c r="D10" t="n">
-        <v>62</v>
+        <v>41</v>
       </c>
       <c r="E10" t="inlineStr">
         <is>
@@ -598,21 +598,21 @@
     <row r="11">
       <c r="A11" t="inlineStr">
         <is>
-          <t>04:59:10</t>
+          <t>06:46:02</t>
         </is>
       </c>
       <c r="B11" t="inlineStr">
         <is>
-          <t>06:09</t>
+          <t>07:32</t>
         </is>
       </c>
       <c r="C11" t="inlineStr">
         <is>
-          <t>10_OLMOS</t>
+          <t>215C_EL PATO</t>
         </is>
       </c>
       <c r="D11" t="n">
-        <v>70</v>
+        <v>46</v>
       </c>
       <c r="E11" t="inlineStr">
         <is>
@@ -623,21 +623,21 @@
     <row r="12">
       <c r="A12" t="inlineStr">
         <is>
-          <t>04:59:10</t>
+          <t>06:46:02</t>
         </is>
       </c>
       <c r="B12" t="inlineStr">
         <is>
-          <t>06:12</t>
+          <t>07:37</t>
         </is>
       </c>
       <c r="C12" t="inlineStr">
         <is>
-          <t>215A_EL PATO</t>
+          <t>27_EL RETIRO</t>
         </is>
       </c>
       <c r="D12" t="n">
-        <v>73</v>
+        <v>51</v>
       </c>
       <c r="E12" t="inlineStr">
         <is>
@@ -648,21 +648,21 @@
     <row r="13">
       <c r="A13" t="inlineStr">
         <is>
-          <t>04:59:10</t>
+          <t>06:46:02</t>
         </is>
       </c>
       <c r="B13" t="inlineStr">
         <is>
-          <t>06:30</t>
+          <t>07:40</t>
         </is>
       </c>
       <c r="C13" t="inlineStr">
         <is>
-          <t>23_HERNANDEZ</t>
+          <t>14_ABASTO</t>
         </is>
       </c>
       <c r="D13" t="n">
-        <v>91</v>
+        <v>54</v>
       </c>
       <c r="E13" t="inlineStr">
         <is>
@@ -673,21 +673,21 @@
     <row r="14">
       <c r="A14" t="inlineStr">
         <is>
-          <t>04:59:10</t>
+          <t>06:46:02</t>
         </is>
       </c>
       <c r="B14" t="inlineStr">
         <is>
-          <t>06:36</t>
+          <t>07:44</t>
         </is>
       </c>
       <c r="C14" t="inlineStr">
         <is>
-          <t>11_ETCHEVERRY</t>
+          <t>10_OLMOS</t>
         </is>
       </c>
       <c r="D14" t="n">
-        <v>97</v>
+        <v>58</v>
       </c>
       <c r="E14" t="inlineStr">
         <is>
@@ -698,21 +698,21 @@
     <row r="15">
       <c r="A15" t="inlineStr">
         <is>
-          <t>04:59:10</t>
+          <t>06:46:02</t>
         </is>
       </c>
       <c r="B15" t="inlineStr">
         <is>
-          <t>06:39</t>
+          <t>07:52</t>
         </is>
       </c>
       <c r="C15" t="inlineStr">
         <is>
-          <t>225_C ROCA-H SUR</t>
+          <t>215A_EL PATO</t>
         </is>
       </c>
       <c r="D15" t="n">
-        <v>100</v>
+        <v>66</v>
       </c>
       <c r="E15" t="inlineStr">
         <is>
@@ -723,21 +723,21 @@
     <row r="16">
       <c r="A16" t="inlineStr">
         <is>
-          <t>04:59:10</t>
+          <t>06:46:02</t>
         </is>
       </c>
       <c r="B16" t="inlineStr">
         <is>
-          <t>06:41</t>
+          <t>08:01</t>
         </is>
       </c>
       <c r="C16" t="inlineStr">
         <is>
-          <t>17X38_ROMERO</t>
+          <t>16_SANTA ANA</t>
         </is>
       </c>
       <c r="D16" t="n">
-        <v>102</v>
+        <v>75</v>
       </c>
       <c r="E16" t="inlineStr">
         <is>
@@ -748,23 +748,123 @@
     <row r="17">
       <c r="A17" t="inlineStr">
         <is>
-          <t>04:59:10</t>
+          <t>06:46:02</t>
         </is>
       </c>
       <c r="B17" t="inlineStr">
         <is>
-          <t>06:41</t>
+          <t>08:19</t>
         </is>
       </c>
       <c r="C17" t="inlineStr">
         <is>
-          <t>16_SANTA ANA</t>
+          <t>15X38_ABASTO</t>
         </is>
       </c>
       <c r="D17" t="n">
-        <v>102</v>
+        <v>93</v>
       </c>
       <c r="E17" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="18">
+      <c r="A18" t="inlineStr">
+        <is>
+          <t>06:46:02</t>
+        </is>
+      </c>
+      <c r="B18" t="inlineStr">
+        <is>
+          <t>08:22</t>
+        </is>
+      </c>
+      <c r="C18" t="inlineStr">
+        <is>
+          <t>23_HERNANDEZ</t>
+        </is>
+      </c>
+      <c r="D18" t="n">
+        <v>96</v>
+      </c>
+      <c r="E18" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="19">
+      <c r="A19" t="inlineStr">
+        <is>
+          <t>06:46:02</t>
+        </is>
+      </c>
+      <c r="B19" t="inlineStr">
+        <is>
+          <t>08:26</t>
+        </is>
+      </c>
+      <c r="C19" t="inlineStr">
+        <is>
+          <t>11X44_ETCHEVERRY</t>
+        </is>
+      </c>
+      <c r="D19" t="n">
+        <v>100</v>
+      </c>
+      <c r="E19" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="20">
+      <c r="A20" t="inlineStr">
+        <is>
+          <t>06:46:02</t>
+        </is>
+      </c>
+      <c r="B20" t="inlineStr">
+        <is>
+          <t>08:45</t>
+        </is>
+      </c>
+      <c r="C20" t="inlineStr">
+        <is>
+          <t>215B_EL PATO</t>
+        </is>
+      </c>
+      <c r="D20" t="n">
+        <v>119</v>
+      </c>
+      <c r="E20" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="21">
+      <c r="A21" t="inlineStr">
+        <is>
+          <t>06:46:02</t>
+        </is>
+      </c>
+      <c r="B21" t="inlineStr">
+        <is>
+          <t>08:45</t>
+        </is>
+      </c>
+      <c r="C21" t="inlineStr">
+        <is>
+          <t>215C_EL PATO</t>
+        </is>
+      </c>
+      <c r="D21" t="n">
+        <v>119</v>
+      </c>
+      <c r="E21" t="inlineStr">
         <is>
           <t>LP1912</t>
         </is>
@@ -781,7 +881,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E6"/>
+  <dimension ref="A1:E10"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -794,14 +894,14 @@
     <row r="2">
       <c r="A2" s="1" t="inlineStr">
         <is>
-          <t>Última actualización: 04:59:10</t>
+          <t>Última actualización: 06:46:02</t>
         </is>
       </c>
     </row>
     <row r="3">
       <c r="A3" s="1" t="inlineStr">
         <is>
-          <t>Total filas: 1</t>
+          <t>Total filas: 5</t>
         </is>
       </c>
     </row>
@@ -835,12 +935,12 @@
     <row r="6">
       <c r="A6" t="inlineStr">
         <is>
-          <t>04:59:10</t>
+          <t>06:46:02</t>
         </is>
       </c>
       <c r="B6" t="inlineStr">
         <is>
-          <t>06:12</t>
+          <t>07:03</t>
         </is>
       </c>
       <c r="C6" t="inlineStr">
@@ -849,9 +949,109 @@
         </is>
       </c>
       <c r="D6" t="n">
-        <v>73</v>
+        <v>17</v>
       </c>
       <c r="E6" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" t="inlineStr">
+        <is>
+          <t>06:46:02</t>
+        </is>
+      </c>
+      <c r="B7" t="inlineStr">
+        <is>
+          <t>07:32</t>
+        </is>
+      </c>
+      <c r="C7" t="inlineStr">
+        <is>
+          <t>215C_EL PATO</t>
+        </is>
+      </c>
+      <c r="D7" t="n">
+        <v>46</v>
+      </c>
+      <c r="E7" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" t="inlineStr">
+        <is>
+          <t>06:46:02</t>
+        </is>
+      </c>
+      <c r="B8" t="inlineStr">
+        <is>
+          <t>07:52</t>
+        </is>
+      </c>
+      <c r="C8" t="inlineStr">
+        <is>
+          <t>215A_EL PATO</t>
+        </is>
+      </c>
+      <c r="D8" t="n">
+        <v>66</v>
+      </c>
+      <c r="E8" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" t="inlineStr">
+        <is>
+          <t>06:46:02</t>
+        </is>
+      </c>
+      <c r="B9" t="inlineStr">
+        <is>
+          <t>08:45</t>
+        </is>
+      </c>
+      <c r="C9" t="inlineStr">
+        <is>
+          <t>215B_EL PATO</t>
+        </is>
+      </c>
+      <c r="D9" t="n">
+        <v>119</v>
+      </c>
+      <c r="E9" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" t="inlineStr">
+        <is>
+          <t>06:46:02</t>
+        </is>
+      </c>
+      <c r="B10" t="inlineStr">
+        <is>
+          <t>08:45</t>
+        </is>
+      </c>
+      <c r="C10" t="inlineStr">
+        <is>
+          <t>215C_EL PATO</t>
+        </is>
+      </c>
+      <c r="D10" t="n">
+        <v>119</v>
+      </c>
+      <c r="E10" t="inlineStr">
         <is>
           <t>LP1912</t>
         </is>
@@ -868,7 +1068,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:A3"/>
+  <dimension ref="A1:E7"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -881,14 +1081,91 @@
     <row r="2">
       <c r="A2" s="1" t="inlineStr">
         <is>
-          <t>Última actualización: 04:59:10</t>
+          <t>Última actualización: 06:46:02</t>
         </is>
       </c>
     </row>
     <row r="3">
       <c r="A3" s="1" t="inlineStr">
         <is>
-          <t>Total filas: 0</t>
+          <t>Total filas: 2</t>
+        </is>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" t="inlineStr">
+        <is>
+          <t>Hora_Scrap</t>
+        </is>
+      </c>
+      <c r="B5" t="inlineStr">
+        <is>
+          <t>Hora_Llegada</t>
+        </is>
+      </c>
+      <c r="C5" t="inlineStr">
+        <is>
+          <t>Linea</t>
+        </is>
+      </c>
+      <c r="D5" t="inlineStr">
+        <is>
+          <t>Minutos</t>
+        </is>
+      </c>
+      <c r="E5" t="inlineStr">
+        <is>
+          <t>Parada</t>
+        </is>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" t="inlineStr">
+        <is>
+          <t>06:46:02</t>
+        </is>
+      </c>
+      <c r="B6" t="inlineStr">
+        <is>
+          <t>07:49</t>
+        </is>
+      </c>
+      <c r="C6" t="inlineStr">
+        <is>
+          <t>215A_LA PLATA</t>
+        </is>
+      </c>
+      <c r="D6" t="n">
+        <v>63</v>
+      </c>
+      <c r="E6" t="inlineStr">
+        <is>
+          <t>L6173</t>
+        </is>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" t="inlineStr">
+        <is>
+          <t>06:46:02</t>
+        </is>
+      </c>
+      <c r="B7" t="inlineStr">
+        <is>
+          <t>08:38</t>
+        </is>
+      </c>
+      <c r="C7" t="inlineStr">
+        <is>
+          <t>215A_LA PLATA</t>
+        </is>
+      </c>
+      <c r="D7" t="n">
+        <v>112</v>
+      </c>
+      <c r="E7" t="inlineStr">
+        <is>
+          <t>L6173</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
📊 Horarios actualizados Línea 141 - 3027
</commit_message>
<xml_diff>
--- a/data/horarios-141-2026-05-17.xlsx
+++ b/data/horarios-141-2026-05-17.xlsx
@@ -419,7 +419,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E21"/>
+  <dimension ref="A1:E34"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -432,14 +432,14 @@
     <row r="2">
       <c r="A2" s="1" t="inlineStr">
         <is>
-          <t>Última actualización: 06:46:02</t>
+          <t>Última actualización: 07:55:48</t>
         </is>
       </c>
     </row>
     <row r="3">
       <c r="A3" s="1" t="inlineStr">
         <is>
-          <t>Total filas: 16</t>
+          <t>Total filas: 29</t>
         </is>
       </c>
     </row>
@@ -723,7 +723,7 @@
     <row r="16">
       <c r="A16" t="inlineStr">
         <is>
-          <t>06:46:02</t>
+          <t>07:55:48</t>
         </is>
       </c>
       <c r="B16" t="inlineStr">
@@ -737,7 +737,7 @@
         </is>
       </c>
       <c r="D16" t="n">
-        <v>75</v>
+        <v>6</v>
       </c>
       <c r="E16" t="inlineStr">
         <is>
@@ -748,7 +748,7 @@
     <row r="17">
       <c r="A17" t="inlineStr">
         <is>
-          <t>06:46:02</t>
+          <t>07:55:48</t>
         </is>
       </c>
       <c r="B17" t="inlineStr">
@@ -762,7 +762,7 @@
         </is>
       </c>
       <c r="D17" t="n">
-        <v>93</v>
+        <v>24</v>
       </c>
       <c r="E17" t="inlineStr">
         <is>
@@ -773,12 +773,12 @@
     <row r="18">
       <c r="A18" t="inlineStr">
         <is>
-          <t>06:46:02</t>
+          <t>07:55:48</t>
         </is>
       </c>
       <c r="B18" t="inlineStr">
         <is>
-          <t>08:22</t>
+          <t>08:21</t>
         </is>
       </c>
       <c r="C18" t="inlineStr">
@@ -787,7 +787,7 @@
         </is>
       </c>
       <c r="D18" t="n">
-        <v>96</v>
+        <v>26</v>
       </c>
       <c r="E18" t="inlineStr">
         <is>
@@ -803,16 +803,16 @@
       </c>
       <c r="B19" t="inlineStr">
         <is>
-          <t>08:26</t>
+          <t>08:22</t>
         </is>
       </c>
       <c r="C19" t="inlineStr">
         <is>
-          <t>11X44_ETCHEVERRY</t>
+          <t>23_HERNANDEZ</t>
         </is>
       </c>
       <c r="D19" t="n">
-        <v>100</v>
+        <v>96</v>
       </c>
       <c r="E19" t="inlineStr">
         <is>
@@ -823,21 +823,21 @@
     <row r="20">
       <c r="A20" t="inlineStr">
         <is>
-          <t>06:46:02</t>
+          <t>07:55:48</t>
         </is>
       </c>
       <c r="B20" t="inlineStr">
         <is>
-          <t>08:45</t>
+          <t>08:25</t>
         </is>
       </c>
       <c r="C20" t="inlineStr">
         <is>
-          <t>215B_EL PATO</t>
+          <t>11X44_ETCHEVERRY</t>
         </is>
       </c>
       <c r="D20" t="n">
-        <v>119</v>
+        <v>30</v>
       </c>
       <c r="E20" t="inlineStr">
         <is>
@@ -853,18 +853,343 @@
       </c>
       <c r="B21" t="inlineStr">
         <is>
+          <t>08:26</t>
+        </is>
+      </c>
+      <c r="C21" t="inlineStr">
+        <is>
+          <t>11X44_ETCHEVERRY</t>
+        </is>
+      </c>
+      <c r="D21" t="n">
+        <v>100</v>
+      </c>
+      <c r="E21" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="22">
+      <c r="A22" t="inlineStr">
+        <is>
+          <t>07:55:48</t>
+        </is>
+      </c>
+      <c r="B22" t="inlineStr">
+        <is>
+          <t>08:42</t>
+        </is>
+      </c>
+      <c r="C22" t="inlineStr">
+        <is>
+          <t>16_SANTA ANA</t>
+        </is>
+      </c>
+      <c r="D22" t="n">
+        <v>47</v>
+      </c>
+      <c r="E22" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="23">
+      <c r="A23" t="inlineStr">
+        <is>
+          <t>07:55:48</t>
+        </is>
+      </c>
+      <c r="B23" t="inlineStr">
+        <is>
+          <t>08:44</t>
+        </is>
+      </c>
+      <c r="C23" t="inlineStr">
+        <is>
+          <t>215B_EL PATO</t>
+        </is>
+      </c>
+      <c r="D23" t="n">
+        <v>49</v>
+      </c>
+      <c r="E23" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="24">
+      <c r="A24" t="inlineStr">
+        <is>
+          <t>07:55:48</t>
+        </is>
+      </c>
+      <c r="B24" t="inlineStr">
+        <is>
+          <t>08:44</t>
+        </is>
+      </c>
+      <c r="C24" t="inlineStr">
+        <is>
+          <t>215C_EL PATO</t>
+        </is>
+      </c>
+      <c r="D24" t="n">
+        <v>49</v>
+      </c>
+      <c r="E24" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="25">
+      <c r="A25" t="inlineStr">
+        <is>
+          <t>06:46:02</t>
+        </is>
+      </c>
+      <c r="B25" t="inlineStr">
+        <is>
           <t>08:45</t>
         </is>
       </c>
-      <c r="C21" t="inlineStr">
+      <c r="C25" t="inlineStr">
         <is>
           <t>215C_EL PATO</t>
         </is>
       </c>
-      <c r="D21" t="n">
+      <c r="D25" t="n">
         <v>119</v>
       </c>
-      <c r="E21" t="inlineStr">
+      <c r="E25" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="26">
+      <c r="A26" t="inlineStr">
+        <is>
+          <t>06:46:02</t>
+        </is>
+      </c>
+      <c r="B26" t="inlineStr">
+        <is>
+          <t>08:45</t>
+        </is>
+      </c>
+      <c r="C26" t="inlineStr">
+        <is>
+          <t>215B_EL PATO</t>
+        </is>
+      </c>
+      <c r="D26" t="n">
+        <v>119</v>
+      </c>
+      <c r="E26" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="27">
+      <c r="A27" t="inlineStr">
+        <is>
+          <t>07:55:48</t>
+        </is>
+      </c>
+      <c r="B27" t="inlineStr">
+        <is>
+          <t>09:04</t>
+        </is>
+      </c>
+      <c r="C27" t="inlineStr">
+        <is>
+          <t>10_OLMOS</t>
+        </is>
+      </c>
+      <c r="D27" t="n">
+        <v>69</v>
+      </c>
+      <c r="E27" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="28">
+      <c r="A28" t="inlineStr">
+        <is>
+          <t>07:55:48</t>
+        </is>
+      </c>
+      <c r="B28" t="inlineStr">
+        <is>
+          <t>09:05</t>
+        </is>
+      </c>
+      <c r="C28" t="inlineStr">
+        <is>
+          <t>23_HERNANDEZ</t>
+        </is>
+      </c>
+      <c r="D28" t="n">
+        <v>70</v>
+      </c>
+      <c r="E28" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="29">
+      <c r="A29" t="inlineStr">
+        <is>
+          <t>07:55:48</t>
+        </is>
+      </c>
+      <c r="B29" t="inlineStr">
+        <is>
+          <t>09:06</t>
+        </is>
+      </c>
+      <c r="C29" t="inlineStr">
+        <is>
+          <t>215A_EL PATO</t>
+        </is>
+      </c>
+      <c r="D29" t="n">
+        <v>71</v>
+      </c>
+      <c r="E29" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="30">
+      <c r="A30" t="inlineStr">
+        <is>
+          <t>07:55:48</t>
+        </is>
+      </c>
+      <c r="B30" t="inlineStr">
+        <is>
+          <t>09:16</t>
+        </is>
+      </c>
+      <c r="C30" t="inlineStr">
+        <is>
+          <t>27_EL RETIRO</t>
+        </is>
+      </c>
+      <c r="D30" t="n">
+        <v>81</v>
+      </c>
+      <c r="E30" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="31">
+      <c r="A31" t="inlineStr">
+        <is>
+          <t>07:55:48</t>
+        </is>
+      </c>
+      <c r="B31" t="inlineStr">
+        <is>
+          <t>09:24</t>
+        </is>
+      </c>
+      <c r="C31" t="inlineStr">
+        <is>
+          <t>14X44_ABASTO</t>
+        </is>
+      </c>
+      <c r="D31" t="n">
+        <v>89</v>
+      </c>
+      <c r="E31" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="32">
+      <c r="A32" t="inlineStr">
+        <is>
+          <t>07:55:48</t>
+        </is>
+      </c>
+      <c r="B32" t="inlineStr">
+        <is>
+          <t>09:34</t>
+        </is>
+      </c>
+      <c r="C32" t="inlineStr">
+        <is>
+          <t>16_P MOR-SANTA ANA</t>
+        </is>
+      </c>
+      <c r="D32" t="n">
+        <v>99</v>
+      </c>
+      <c r="E32" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="33">
+      <c r="A33" t="inlineStr">
+        <is>
+          <t>07:55:48</t>
+        </is>
+      </c>
+      <c r="B33" t="inlineStr">
+        <is>
+          <t>09:35</t>
+        </is>
+      </c>
+      <c r="C33" t="inlineStr">
+        <is>
+          <t>17_ROMERO</t>
+        </is>
+      </c>
+      <c r="D33" t="n">
+        <v>100</v>
+      </c>
+      <c r="E33" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="34">
+      <c r="A34" t="inlineStr">
+        <is>
+          <t>07:55:48</t>
+        </is>
+      </c>
+      <c r="B34" t="inlineStr">
+        <is>
+          <t>09:44</t>
+        </is>
+      </c>
+      <c r="C34" t="inlineStr">
+        <is>
+          <t>11_ETCHEVERRY</t>
+        </is>
+      </c>
+      <c r="D34" t="n">
+        <v>109</v>
+      </c>
+      <c r="E34" t="inlineStr">
         <is>
           <t>LP1912</t>
         </is>
@@ -881,7 +1206,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E10"/>
+  <dimension ref="A1:E13"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -894,14 +1219,14 @@
     <row r="2">
       <c r="A2" s="1" t="inlineStr">
         <is>
-          <t>Última actualización: 06:46:02</t>
+          <t>Última actualización: 07:55:48</t>
         </is>
       </c>
     </row>
     <row r="3">
       <c r="A3" s="1" t="inlineStr">
         <is>
-          <t>Total filas: 5</t>
+          <t>Total filas: 8</t>
         </is>
       </c>
     </row>
@@ -1010,12 +1335,12 @@
     <row r="9">
       <c r="A9" t="inlineStr">
         <is>
-          <t>06:46:02</t>
+          <t>07:55:48</t>
         </is>
       </c>
       <c r="B9" t="inlineStr">
         <is>
-          <t>08:45</t>
+          <t>08:44</t>
         </is>
       </c>
       <c r="C9" t="inlineStr">
@@ -1024,7 +1349,7 @@
         </is>
       </c>
       <c r="D9" t="n">
-        <v>119</v>
+        <v>49</v>
       </c>
       <c r="E9" t="inlineStr">
         <is>
@@ -1035,23 +1360,98 @@
     <row r="10">
       <c r="A10" t="inlineStr">
         <is>
-          <t>06:46:02</t>
+          <t>07:55:48</t>
         </is>
       </c>
       <c r="B10" t="inlineStr">
         <is>
+          <t>08:44</t>
+        </is>
+      </c>
+      <c r="C10" t="inlineStr">
+        <is>
+          <t>215C_EL PATO</t>
+        </is>
+      </c>
+      <c r="D10" t="n">
+        <v>49</v>
+      </c>
+      <c r="E10" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" t="inlineStr">
+        <is>
+          <t>06:46:02</t>
+        </is>
+      </c>
+      <c r="B11" t="inlineStr">
+        <is>
           <t>08:45</t>
         </is>
       </c>
-      <c r="C10" t="inlineStr">
+      <c r="C11" t="inlineStr">
+        <is>
+          <t>215B_EL PATO</t>
+        </is>
+      </c>
+      <c r="D11" t="n">
+        <v>119</v>
+      </c>
+      <c r="E11" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="12">
+      <c r="A12" t="inlineStr">
+        <is>
+          <t>06:46:02</t>
+        </is>
+      </c>
+      <c r="B12" t="inlineStr">
+        <is>
+          <t>08:45</t>
+        </is>
+      </c>
+      <c r="C12" t="inlineStr">
         <is>
           <t>215C_EL PATO</t>
         </is>
       </c>
-      <c r="D10" t="n">
+      <c r="D12" t="n">
         <v>119</v>
       </c>
-      <c r="E10" t="inlineStr">
+      <c r="E12" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="13">
+      <c r="A13" t="inlineStr">
+        <is>
+          <t>07:55:48</t>
+        </is>
+      </c>
+      <c r="B13" t="inlineStr">
+        <is>
+          <t>09:06</t>
+        </is>
+      </c>
+      <c r="C13" t="inlineStr">
+        <is>
+          <t>215A_EL PATO</t>
+        </is>
+      </c>
+      <c r="D13" t="n">
+        <v>71</v>
+      </c>
+      <c r="E13" t="inlineStr">
         <is>
           <t>LP1912</t>
         </is>
@@ -1068,7 +1468,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E7"/>
+  <dimension ref="A1:E10"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -1081,14 +1481,14 @@
     <row r="2">
       <c r="A2" s="1" t="inlineStr">
         <is>
-          <t>Última actualización: 06:46:02</t>
+          <t>Última actualización: 07:55:48</t>
         </is>
       </c>
     </row>
     <row r="3">
       <c r="A3" s="1" t="inlineStr">
         <is>
-          <t>Total filas: 2</t>
+          <t>Total filas: 5</t>
         </is>
       </c>
     </row>
@@ -1147,23 +1547,98 @@
     <row r="7">
       <c r="A7" t="inlineStr">
         <is>
-          <t>06:46:02</t>
+          <t>07:55:48</t>
         </is>
       </c>
       <c r="B7" t="inlineStr">
         <is>
+          <t>08:37</t>
+        </is>
+      </c>
+      <c r="C7" t="inlineStr">
+        <is>
+          <t>215A_LA PLATA</t>
+        </is>
+      </c>
+      <c r="D7" t="n">
+        <v>42</v>
+      </c>
+      <c r="E7" t="inlineStr">
+        <is>
+          <t>L6173</t>
+        </is>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" t="inlineStr">
+        <is>
+          <t>06:46:02</t>
+        </is>
+      </c>
+      <c r="B8" t="inlineStr">
+        <is>
           <t>08:38</t>
         </is>
       </c>
-      <c r="C7" t="inlineStr">
+      <c r="C8" t="inlineStr">
         <is>
           <t>215A_LA PLATA</t>
         </is>
       </c>
-      <c r="D7" t="n">
+      <c r="D8" t="n">
         <v>112</v>
       </c>
-      <c r="E7" t="inlineStr">
+      <c r="E8" t="inlineStr">
+        <is>
+          <t>L6173</t>
+        </is>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" t="inlineStr">
+        <is>
+          <t>07:55:48</t>
+        </is>
+      </c>
+      <c r="B9" t="inlineStr">
+        <is>
+          <t>09:02</t>
+        </is>
+      </c>
+      <c r="C9" t="inlineStr">
+        <is>
+          <t>215C_LA PLATA</t>
+        </is>
+      </c>
+      <c r="D9" t="n">
+        <v>67</v>
+      </c>
+      <c r="E9" t="inlineStr">
+        <is>
+          <t>L6203</t>
+        </is>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" t="inlineStr">
+        <is>
+          <t>07:55:48</t>
+        </is>
+      </c>
+      <c r="B10" t="inlineStr">
+        <is>
+          <t>09:27</t>
+        </is>
+      </c>
+      <c r="C10" t="inlineStr">
+        <is>
+          <t>215A_LA PLATA</t>
+        </is>
+      </c>
+      <c r="D10" t="n">
+        <v>92</v>
+      </c>
+      <c r="E10" t="inlineStr">
         <is>
           <t>L6173</t>
         </is>

</xml_diff>

<commit_message>
📊 Horarios actualizados Línea 141 - 3028
</commit_message>
<xml_diff>
--- a/data/horarios-141-2026-05-17.xlsx
+++ b/data/horarios-141-2026-05-17.xlsx
@@ -419,7 +419,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E34"/>
+  <dimension ref="A1:E45"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -432,14 +432,14 @@
     <row r="2">
       <c r="A2" s="1" t="inlineStr">
         <is>
-          <t>Última actualización: 07:55:48</t>
+          <t>Última actualización: 08:53:32</t>
         </is>
       </c>
     </row>
     <row r="3">
       <c r="A3" s="1" t="inlineStr">
         <is>
-          <t>Total filas: 29</t>
+          <t>Total filas: 40</t>
         </is>
       </c>
     </row>
@@ -958,7 +958,7 @@
       </c>
       <c r="C25" t="inlineStr">
         <is>
-          <t>215C_EL PATO</t>
+          <t>215B_EL PATO</t>
         </is>
       </c>
       <c r="D25" t="n">
@@ -983,7 +983,7 @@
       </c>
       <c r="C26" t="inlineStr">
         <is>
-          <t>215B_EL PATO</t>
+          <t>215C_EL PATO</t>
         </is>
       </c>
       <c r="D26" t="n">
@@ -998,7 +998,7 @@
     <row r="27">
       <c r="A27" t="inlineStr">
         <is>
-          <t>07:55:48</t>
+          <t>08:53:32</t>
         </is>
       </c>
       <c r="B27" t="inlineStr">
@@ -1012,7 +1012,7 @@
         </is>
       </c>
       <c r="D27" t="n">
-        <v>69</v>
+        <v>11</v>
       </c>
       <c r="E27" t="inlineStr">
         <is>
@@ -1048,7 +1048,7 @@
     <row r="29">
       <c r="A29" t="inlineStr">
         <is>
-          <t>07:55:48</t>
+          <t>08:53:32</t>
         </is>
       </c>
       <c r="B29" t="inlineStr">
@@ -1062,7 +1062,7 @@
         </is>
       </c>
       <c r="D29" t="n">
-        <v>71</v>
+        <v>13</v>
       </c>
       <c r="E29" t="inlineStr">
         <is>
@@ -1073,21 +1073,21 @@
     <row r="30">
       <c r="A30" t="inlineStr">
         <is>
-          <t>07:55:48</t>
+          <t>08:53:32</t>
         </is>
       </c>
       <c r="B30" t="inlineStr">
         <is>
-          <t>09:16</t>
+          <t>09:11</t>
         </is>
       </c>
       <c r="C30" t="inlineStr">
         <is>
-          <t>27_EL RETIRO</t>
+          <t>23_HERNANDEZ</t>
         </is>
       </c>
       <c r="D30" t="n">
-        <v>81</v>
+        <v>18</v>
       </c>
       <c r="E30" t="inlineStr">
         <is>
@@ -1098,21 +1098,21 @@
     <row r="31">
       <c r="A31" t="inlineStr">
         <is>
-          <t>07:55:48</t>
+          <t>08:53:32</t>
         </is>
       </c>
       <c r="B31" t="inlineStr">
         <is>
-          <t>09:24</t>
+          <t>09:16</t>
         </is>
       </c>
       <c r="C31" t="inlineStr">
         <is>
-          <t>14X44_ABASTO</t>
+          <t>16_SANTA ANA</t>
         </is>
       </c>
       <c r="D31" t="n">
-        <v>89</v>
+        <v>23</v>
       </c>
       <c r="E31" t="inlineStr">
         <is>
@@ -1123,21 +1123,21 @@
     <row r="32">
       <c r="A32" t="inlineStr">
         <is>
-          <t>07:55:48</t>
+          <t>08:53:32</t>
         </is>
       </c>
       <c r="B32" t="inlineStr">
         <is>
-          <t>09:34</t>
+          <t>09:16</t>
         </is>
       </c>
       <c r="C32" t="inlineStr">
         <is>
-          <t>16_P MOR-SANTA ANA</t>
+          <t>27_EL RETIRO</t>
         </is>
       </c>
       <c r="D32" t="n">
-        <v>99</v>
+        <v>23</v>
       </c>
       <c r="E32" t="inlineStr">
         <is>
@@ -1148,21 +1148,21 @@
     <row r="33">
       <c r="A33" t="inlineStr">
         <is>
-          <t>07:55:48</t>
+          <t>08:53:32</t>
         </is>
       </c>
       <c r="B33" t="inlineStr">
         <is>
-          <t>09:35</t>
+          <t>09:24</t>
         </is>
       </c>
       <c r="C33" t="inlineStr">
         <is>
-          <t>17_ROMERO</t>
+          <t>14X44_ABASTO</t>
         </is>
       </c>
       <c r="D33" t="n">
-        <v>100</v>
+        <v>31</v>
       </c>
       <c r="E33" t="inlineStr">
         <is>
@@ -1173,23 +1173,298 @@
     <row r="34">
       <c r="A34" t="inlineStr">
         <is>
-          <t>07:55:48</t>
+          <t>08:53:32</t>
         </is>
       </c>
       <c r="B34" t="inlineStr">
         <is>
+          <t>09:34</t>
+        </is>
+      </c>
+      <c r="C34" t="inlineStr">
+        <is>
+          <t>16_P MOR-SANTA ANA</t>
+        </is>
+      </c>
+      <c r="D34" t="n">
+        <v>41</v>
+      </c>
+      <c r="E34" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="35">
+      <c r="A35" t="inlineStr">
+        <is>
+          <t>08:53:32</t>
+        </is>
+      </c>
+      <c r="B35" t="inlineStr">
+        <is>
+          <t>09:35</t>
+        </is>
+      </c>
+      <c r="C35" t="inlineStr">
+        <is>
+          <t>17_ROMERO</t>
+        </is>
+      </c>
+      <c r="D35" t="n">
+        <v>42</v>
+      </c>
+      <c r="E35" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="36">
+      <c r="A36" t="inlineStr">
+        <is>
+          <t>08:53:32</t>
+        </is>
+      </c>
+      <c r="B36" t="inlineStr">
+        <is>
           <t>09:44</t>
         </is>
       </c>
-      <c r="C34" t="inlineStr">
+      <c r="C36" t="inlineStr">
         <is>
           <t>11_ETCHEVERRY</t>
         </is>
       </c>
-      <c r="D34" t="n">
-        <v>109</v>
-      </c>
-      <c r="E34" t="inlineStr">
+      <c r="D36" t="n">
+        <v>51</v>
+      </c>
+      <c r="E36" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="37">
+      <c r="A37" t="inlineStr">
+        <is>
+          <t>08:53:32</t>
+        </is>
+      </c>
+      <c r="B37" t="inlineStr">
+        <is>
+          <t>09:51</t>
+        </is>
+      </c>
+      <c r="C37" t="inlineStr">
+        <is>
+          <t>16_SANTA ANA</t>
+        </is>
+      </c>
+      <c r="D37" t="n">
+        <v>58</v>
+      </c>
+      <c r="E37" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="38">
+      <c r="A38" t="inlineStr">
+        <is>
+          <t>08:53:32</t>
+        </is>
+      </c>
+      <c r="B38" t="inlineStr">
+        <is>
+          <t>09:55</t>
+        </is>
+      </c>
+      <c r="C38" t="inlineStr">
+        <is>
+          <t>14_ABASTO</t>
+        </is>
+      </c>
+      <c r="D38" t="n">
+        <v>62</v>
+      </c>
+      <c r="E38" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="39">
+      <c r="A39" t="inlineStr">
+        <is>
+          <t>08:53:32</t>
+        </is>
+      </c>
+      <c r="B39" t="inlineStr">
+        <is>
+          <t>09:55</t>
+        </is>
+      </c>
+      <c r="C39" t="inlineStr">
+        <is>
+          <t>215C_EL PATO</t>
+        </is>
+      </c>
+      <c r="D39" t="n">
+        <v>62</v>
+      </c>
+      <c r="E39" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="40">
+      <c r="A40" t="inlineStr">
+        <is>
+          <t>08:53:32</t>
+        </is>
+      </c>
+      <c r="B40" t="inlineStr">
+        <is>
+          <t>09:59</t>
+        </is>
+      </c>
+      <c r="C40" t="inlineStr">
+        <is>
+          <t>23_HERNANDEZ</t>
+        </is>
+      </c>
+      <c r="D40" t="n">
+        <v>66</v>
+      </c>
+      <c r="E40" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="41">
+      <c r="A41" t="inlineStr">
+        <is>
+          <t>08:53:32</t>
+        </is>
+      </c>
+      <c r="B41" t="inlineStr">
+        <is>
+          <t>10:04</t>
+        </is>
+      </c>
+      <c r="C41" t="inlineStr">
+        <is>
+          <t>10_OLMOS</t>
+        </is>
+      </c>
+      <c r="D41" t="n">
+        <v>71</v>
+      </c>
+      <c r="E41" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="42">
+      <c r="A42" t="inlineStr">
+        <is>
+          <t>08:53:32</t>
+        </is>
+      </c>
+      <c r="B42" t="inlineStr">
+        <is>
+          <t>10:15</t>
+        </is>
+      </c>
+      <c r="C42" t="inlineStr">
+        <is>
+          <t>15_ABASTO</t>
+        </is>
+      </c>
+      <c r="D42" t="n">
+        <v>82</v>
+      </c>
+      <c r="E42" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="43">
+      <c r="A43" t="inlineStr">
+        <is>
+          <t>08:53:32</t>
+        </is>
+      </c>
+      <c r="B43" t="inlineStr">
+        <is>
+          <t>10:24</t>
+        </is>
+      </c>
+      <c r="C43" t="inlineStr">
+        <is>
+          <t>14_ABASTO</t>
+        </is>
+      </c>
+      <c r="D43" t="n">
+        <v>91</v>
+      </c>
+      <c r="E43" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="44">
+      <c r="A44" t="inlineStr">
+        <is>
+          <t>08:53:32</t>
+        </is>
+      </c>
+      <c r="B44" t="inlineStr">
+        <is>
+          <t>10:34</t>
+        </is>
+      </c>
+      <c r="C44" t="inlineStr">
+        <is>
+          <t>17X38_ROMERO</t>
+        </is>
+      </c>
+      <c r="D44" t="n">
+        <v>101</v>
+      </c>
+      <c r="E44" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="45">
+      <c r="A45" t="inlineStr">
+        <is>
+          <t>08:53:32</t>
+        </is>
+      </c>
+      <c r="B45" t="inlineStr">
+        <is>
+          <t>10:44</t>
+        </is>
+      </c>
+      <c r="C45" t="inlineStr">
+        <is>
+          <t>11X44_ETCHEVERRY</t>
+        </is>
+      </c>
+      <c r="D45" t="n">
+        <v>111</v>
+      </c>
+      <c r="E45" t="inlineStr">
         <is>
           <t>LP1912</t>
         </is>
@@ -1206,7 +1481,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E13"/>
+  <dimension ref="A1:E14"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -1219,14 +1494,14 @@
     <row r="2">
       <c r="A2" s="1" t="inlineStr">
         <is>
-          <t>Última actualización: 07:55:48</t>
+          <t>Última actualización: 08:53:32</t>
         </is>
       </c>
     </row>
     <row r="3">
       <c r="A3" s="1" t="inlineStr">
         <is>
-          <t>Total filas: 8</t>
+          <t>Total filas: 9</t>
         </is>
       </c>
     </row>
@@ -1435,7 +1710,7 @@
     <row r="13">
       <c r="A13" t="inlineStr">
         <is>
-          <t>07:55:48</t>
+          <t>08:53:32</t>
         </is>
       </c>
       <c r="B13" t="inlineStr">
@@ -1449,9 +1724,34 @@
         </is>
       </c>
       <c r="D13" t="n">
-        <v>71</v>
+        <v>13</v>
       </c>
       <c r="E13" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="14">
+      <c r="A14" t="inlineStr">
+        <is>
+          <t>08:53:32</t>
+        </is>
+      </c>
+      <c r="B14" t="inlineStr">
+        <is>
+          <t>09:55</t>
+        </is>
+      </c>
+      <c r="C14" t="inlineStr">
+        <is>
+          <t>215C_EL PATO</t>
+        </is>
+      </c>
+      <c r="D14" t="n">
+        <v>62</v>
+      </c>
+      <c r="E14" t="inlineStr">
         <is>
           <t>LP1912</t>
         </is>
@@ -1468,7 +1768,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E10"/>
+  <dimension ref="A1:E15"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -1481,14 +1781,14 @@
     <row r="2">
       <c r="A2" s="1" t="inlineStr">
         <is>
-          <t>Última actualización: 07:55:48</t>
+          <t>Última actualización: 08:53:32</t>
         </is>
       </c>
     </row>
     <row r="3">
       <c r="A3" s="1" t="inlineStr">
         <is>
-          <t>Total filas: 5</t>
+          <t>Total filas: 10</t>
         </is>
       </c>
     </row>
@@ -1622,23 +1922,148 @@
     <row r="10">
       <c r="A10" t="inlineStr">
         <is>
+          <t>08:53:32</t>
+        </is>
+      </c>
+      <c r="B10" t="inlineStr">
+        <is>
+          <t>09:03</t>
+        </is>
+      </c>
+      <c r="C10" t="inlineStr">
+        <is>
+          <t>215C_LA PLATA</t>
+        </is>
+      </c>
+      <c r="D10" t="n">
+        <v>10</v>
+      </c>
+      <c r="E10" t="inlineStr">
+        <is>
+          <t>L6203</t>
+        </is>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" t="inlineStr">
+        <is>
           <t>07:55:48</t>
         </is>
       </c>
-      <c r="B10" t="inlineStr">
+      <c r="B11" t="inlineStr">
         <is>
           <t>09:27</t>
         </is>
       </c>
-      <c r="C10" t="inlineStr">
+      <c r="C11" t="inlineStr">
         <is>
           <t>215A_LA PLATA</t>
         </is>
       </c>
-      <c r="D10" t="n">
+      <c r="D11" t="n">
         <v>92</v>
       </c>
-      <c r="E10" t="inlineStr">
+      <c r="E11" t="inlineStr">
+        <is>
+          <t>L6173</t>
+        </is>
+      </c>
+    </row>
+    <row r="12">
+      <c r="A12" t="inlineStr">
+        <is>
+          <t>08:53:32</t>
+        </is>
+      </c>
+      <c r="B12" t="inlineStr">
+        <is>
+          <t>09:28</t>
+        </is>
+      </c>
+      <c r="C12" t="inlineStr">
+        <is>
+          <t>215A_LA PLATA</t>
+        </is>
+      </c>
+      <c r="D12" t="n">
+        <v>35</v>
+      </c>
+      <c r="E12" t="inlineStr">
+        <is>
+          <t>L6173</t>
+        </is>
+      </c>
+    </row>
+    <row r="13">
+      <c r="A13" t="inlineStr">
+        <is>
+          <t>08:53:32</t>
+        </is>
+      </c>
+      <c r="B13" t="inlineStr">
+        <is>
+          <t>10:18</t>
+        </is>
+      </c>
+      <c r="C13" t="inlineStr">
+        <is>
+          <t>215C_LA PLATA</t>
+        </is>
+      </c>
+      <c r="D13" t="n">
+        <v>85</v>
+      </c>
+      <c r="E13" t="inlineStr">
+        <is>
+          <t>L6203</t>
+        </is>
+      </c>
+    </row>
+    <row r="14">
+      <c r="A14" t="inlineStr">
+        <is>
+          <t>08:53:32</t>
+        </is>
+      </c>
+      <c r="B14" t="inlineStr">
+        <is>
+          <t>10:30</t>
+        </is>
+      </c>
+      <c r="C14" t="inlineStr">
+        <is>
+          <t>215B_LP-P MOR-1 Y 57</t>
+        </is>
+      </c>
+      <c r="D14" t="n">
+        <v>97</v>
+      </c>
+      <c r="E14" t="inlineStr">
+        <is>
+          <t>L6173</t>
+        </is>
+      </c>
+    </row>
+    <row r="15">
+      <c r="A15" t="inlineStr">
+        <is>
+          <t>08:53:32</t>
+        </is>
+      </c>
+      <c r="B15" t="inlineStr">
+        <is>
+          <t>10:43</t>
+        </is>
+      </c>
+      <c r="C15" t="inlineStr">
+        <is>
+          <t>215A_LA PLATA</t>
+        </is>
+      </c>
+      <c r="D15" t="n">
+        <v>110</v>
+      </c>
+      <c r="E15" t="inlineStr">
         <is>
           <t>L6173</t>
         </is>

</xml_diff>

<commit_message>
📊 Horarios actualizados Línea 141 - 3029
</commit_message>
<xml_diff>
--- a/data/horarios-141-2026-05-17.xlsx
+++ b/data/horarios-141-2026-05-17.xlsx
@@ -419,7 +419,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E45"/>
+  <dimension ref="A1:E57"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -432,14 +432,14 @@
     <row r="2">
       <c r="A2" s="1" t="inlineStr">
         <is>
-          <t>Última actualización: 08:53:32</t>
+          <t>Última actualización: 09:51:48</t>
         </is>
       </c>
     </row>
     <row r="3">
       <c r="A3" s="1" t="inlineStr">
         <is>
-          <t>Total filas: 40</t>
+          <t>Total filas: 52</t>
         </is>
       </c>
     </row>
@@ -558,7 +558,7 @@
       </c>
       <c r="C9" t="inlineStr">
         <is>
-          <t>14_ABASTO</t>
+          <t>23_HERNANDEZ</t>
         </is>
       </c>
       <c r="D9" t="n">
@@ -583,7 +583,7 @@
       </c>
       <c r="C10" t="inlineStr">
         <is>
-          <t>23_HERNANDEZ</t>
+          <t>14_ABASTO</t>
         </is>
       </c>
       <c r="D10" t="n">
@@ -908,7 +908,7 @@
       </c>
       <c r="C23" t="inlineStr">
         <is>
-          <t>215B_EL PATO</t>
+          <t>215C_EL PATO</t>
         </is>
       </c>
       <c r="D23" t="n">
@@ -933,7 +933,7 @@
       </c>
       <c r="C24" t="inlineStr">
         <is>
-          <t>215C_EL PATO</t>
+          <t>215B_EL PATO</t>
         </is>
       </c>
       <c r="D24" t="n">
@@ -1248,7 +1248,7 @@
     <row r="37">
       <c r="A37" t="inlineStr">
         <is>
-          <t>08:53:32</t>
+          <t>09:51:48</t>
         </is>
       </c>
       <c r="B37" t="inlineStr">
@@ -1262,7 +1262,7 @@
         </is>
       </c>
       <c r="D37" t="n">
-        <v>58</v>
+        <v>0</v>
       </c>
       <c r="E37" t="inlineStr">
         <is>
@@ -1273,21 +1273,21 @@
     <row r="38">
       <c r="A38" t="inlineStr">
         <is>
-          <t>08:53:32</t>
+          <t>09:51:48</t>
         </is>
       </c>
       <c r="B38" t="inlineStr">
         <is>
-          <t>09:55</t>
+          <t>09:54</t>
         </is>
       </c>
       <c r="C38" t="inlineStr">
         <is>
-          <t>14_ABASTO</t>
+          <t>215C_EL PATO</t>
         </is>
       </c>
       <c r="D38" t="n">
-        <v>62</v>
+        <v>3</v>
       </c>
       <c r="E38" t="inlineStr">
         <is>
@@ -1308,7 +1308,7 @@
       </c>
       <c r="C39" t="inlineStr">
         <is>
-          <t>215C_EL PATO</t>
+          <t>14_ABASTO</t>
         </is>
       </c>
       <c r="D39" t="n">
@@ -1328,16 +1328,16 @@
       </c>
       <c r="B40" t="inlineStr">
         <is>
-          <t>09:59</t>
+          <t>09:55</t>
         </is>
       </c>
       <c r="C40" t="inlineStr">
         <is>
-          <t>23_HERNANDEZ</t>
+          <t>215C_EL PATO</t>
         </is>
       </c>
       <c r="D40" t="n">
-        <v>66</v>
+        <v>62</v>
       </c>
       <c r="E40" t="inlineStr">
         <is>
@@ -1353,16 +1353,16 @@
       </c>
       <c r="B41" t="inlineStr">
         <is>
-          <t>10:04</t>
+          <t>09:59</t>
         </is>
       </c>
       <c r="C41" t="inlineStr">
         <is>
-          <t>10_OLMOS</t>
+          <t>23_HERNANDEZ</t>
         </is>
       </c>
       <c r="D41" t="n">
-        <v>71</v>
+        <v>66</v>
       </c>
       <c r="E41" t="inlineStr">
         <is>
@@ -1373,21 +1373,21 @@
     <row r="42">
       <c r="A42" t="inlineStr">
         <is>
-          <t>08:53:32</t>
+          <t>09:51:48</t>
         </is>
       </c>
       <c r="B42" t="inlineStr">
         <is>
-          <t>10:15</t>
+          <t>10:01</t>
         </is>
       </c>
       <c r="C42" t="inlineStr">
         <is>
-          <t>15_ABASTO</t>
+          <t>23_HERNANDEZ</t>
         </is>
       </c>
       <c r="D42" t="n">
-        <v>82</v>
+        <v>10</v>
       </c>
       <c r="E42" t="inlineStr">
         <is>
@@ -1398,21 +1398,21 @@
     <row r="43">
       <c r="A43" t="inlineStr">
         <is>
-          <t>08:53:32</t>
+          <t>09:51:48</t>
         </is>
       </c>
       <c r="B43" t="inlineStr">
         <is>
-          <t>10:24</t>
+          <t>10:04</t>
         </is>
       </c>
       <c r="C43" t="inlineStr">
         <is>
-          <t>14_ABASTO</t>
+          <t>10_OLMOS</t>
         </is>
       </c>
       <c r="D43" t="n">
-        <v>91</v>
+        <v>13</v>
       </c>
       <c r="E43" t="inlineStr">
         <is>
@@ -1423,21 +1423,21 @@
     <row r="44">
       <c r="A44" t="inlineStr">
         <is>
-          <t>08:53:32</t>
+          <t>09:51:48</t>
         </is>
       </c>
       <c r="B44" t="inlineStr">
         <is>
-          <t>10:34</t>
+          <t>10:15</t>
         </is>
       </c>
       <c r="C44" t="inlineStr">
         <is>
-          <t>17X38_ROMERO</t>
+          <t>15_ABASTO</t>
         </is>
       </c>
       <c r="D44" t="n">
-        <v>101</v>
+        <v>24</v>
       </c>
       <c r="E44" t="inlineStr">
         <is>
@@ -1448,23 +1448,323 @@
     <row r="45">
       <c r="A45" t="inlineStr">
         <is>
-          <t>08:53:32</t>
+          <t>09:51:48</t>
         </is>
       </c>
       <c r="B45" t="inlineStr">
         <is>
+          <t>10:24</t>
+        </is>
+      </c>
+      <c r="C45" t="inlineStr">
+        <is>
+          <t>14_ABASTO</t>
+        </is>
+      </c>
+      <c r="D45" t="n">
+        <v>33</v>
+      </c>
+      <c r="E45" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="46">
+      <c r="A46" t="inlineStr">
+        <is>
+          <t>09:51:48</t>
+        </is>
+      </c>
+      <c r="B46" t="inlineStr">
+        <is>
+          <t>10:34</t>
+        </is>
+      </c>
+      <c r="C46" t="inlineStr">
+        <is>
+          <t>17X38_ROMERO</t>
+        </is>
+      </c>
+      <c r="D46" t="n">
+        <v>43</v>
+      </c>
+      <c r="E46" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="47">
+      <c r="A47" t="inlineStr">
+        <is>
+          <t>09:51:48</t>
+        </is>
+      </c>
+      <c r="B47" t="inlineStr">
+        <is>
           <t>10:44</t>
         </is>
       </c>
-      <c r="C45" t="inlineStr">
+      <c r="C47" t="inlineStr">
         <is>
           <t>11X44_ETCHEVERRY</t>
         </is>
       </c>
-      <c r="D45" t="n">
-        <v>111</v>
-      </c>
-      <c r="E45" t="inlineStr">
+      <c r="D47" t="n">
+        <v>53</v>
+      </c>
+      <c r="E47" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="48">
+      <c r="A48" t="inlineStr">
+        <is>
+          <t>09:51:48</t>
+        </is>
+      </c>
+      <c r="B48" t="inlineStr">
+        <is>
+          <t>10:47</t>
+        </is>
+      </c>
+      <c r="C48" t="inlineStr">
+        <is>
+          <t>23_HERNANDEZ</t>
+        </is>
+      </c>
+      <c r="D48" t="n">
+        <v>56</v>
+      </c>
+      <c r="E48" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="49">
+      <c r="A49" t="inlineStr">
+        <is>
+          <t>09:51:48</t>
+        </is>
+      </c>
+      <c r="B49" t="inlineStr">
+        <is>
+          <t>10:53</t>
+        </is>
+      </c>
+      <c r="C49" t="inlineStr">
+        <is>
+          <t>27_EL RETIRO</t>
+        </is>
+      </c>
+      <c r="D49" t="n">
+        <v>62</v>
+      </c>
+      <c r="E49" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="50">
+      <c r="A50" t="inlineStr">
+        <is>
+          <t>09:51:48</t>
+        </is>
+      </c>
+      <c r="B50" t="inlineStr">
+        <is>
+          <t>10:55</t>
+        </is>
+      </c>
+      <c r="C50" t="inlineStr">
+        <is>
+          <t>81_EL PELIGRO</t>
+        </is>
+      </c>
+      <c r="D50" t="n">
+        <v>64</v>
+      </c>
+      <c r="E50" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="51">
+      <c r="A51" t="inlineStr">
+        <is>
+          <t>09:51:48</t>
+        </is>
+      </c>
+      <c r="B51" t="inlineStr">
+        <is>
+          <t>11:01</t>
+        </is>
+      </c>
+      <c r="C51" t="inlineStr">
+        <is>
+          <t>16_SANTA ANA</t>
+        </is>
+      </c>
+      <c r="D51" t="n">
+        <v>70</v>
+      </c>
+      <c r="E51" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="52">
+      <c r="A52" t="inlineStr">
+        <is>
+          <t>09:51:48</t>
+        </is>
+      </c>
+      <c r="B52" t="inlineStr">
+        <is>
+          <t>11:04</t>
+        </is>
+      </c>
+      <c r="C52" t="inlineStr">
+        <is>
+          <t>14_ABASTO</t>
+        </is>
+      </c>
+      <c r="D52" t="n">
+        <v>73</v>
+      </c>
+      <c r="E52" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="53">
+      <c r="A53" t="inlineStr">
+        <is>
+          <t>09:51:48</t>
+        </is>
+      </c>
+      <c r="B53" t="inlineStr">
+        <is>
+          <t>11:08</t>
+        </is>
+      </c>
+      <c r="C53" t="inlineStr">
+        <is>
+          <t>225_C ROCA-H SUR</t>
+        </is>
+      </c>
+      <c r="D53" t="n">
+        <v>77</v>
+      </c>
+      <c r="E53" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="54">
+      <c r="A54" t="inlineStr">
+        <is>
+          <t>09:51:48</t>
+        </is>
+      </c>
+      <c r="B54" t="inlineStr">
+        <is>
+          <t>11:11</t>
+        </is>
+      </c>
+      <c r="C54" t="inlineStr">
+        <is>
+          <t>17_ROMERO</t>
+        </is>
+      </c>
+      <c r="D54" t="n">
+        <v>80</v>
+      </c>
+      <c r="E54" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="55">
+      <c r="A55" t="inlineStr">
+        <is>
+          <t>09:51:48</t>
+        </is>
+      </c>
+      <c r="B55" t="inlineStr">
+        <is>
+          <t>11:24</t>
+        </is>
+      </c>
+      <c r="C55" t="inlineStr">
+        <is>
+          <t>10_OLMOS</t>
+        </is>
+      </c>
+      <c r="D55" t="n">
+        <v>93</v>
+      </c>
+      <c r="E55" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="56">
+      <c r="A56" t="inlineStr">
+        <is>
+          <t>09:51:48</t>
+        </is>
+      </c>
+      <c r="B56" t="inlineStr">
+        <is>
+          <t>11:34</t>
+        </is>
+      </c>
+      <c r="C56" t="inlineStr">
+        <is>
+          <t>215C_EL PATO</t>
+        </is>
+      </c>
+      <c r="D56" t="n">
+        <v>103</v>
+      </c>
+      <c r="E56" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="57">
+      <c r="A57" t="inlineStr">
+        <is>
+          <t>09:51:48</t>
+        </is>
+      </c>
+      <c r="B57" t="inlineStr">
+        <is>
+          <t>11:44</t>
+        </is>
+      </c>
+      <c r="C57" t="inlineStr">
+        <is>
+          <t>215B_EL PATO</t>
+        </is>
+      </c>
+      <c r="D57" t="n">
+        <v>113</v>
+      </c>
+      <c r="E57" t="inlineStr">
         <is>
           <t>LP1912</t>
         </is>
@@ -1481,7 +1781,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E14"/>
+  <dimension ref="A1:E17"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -1494,14 +1794,14 @@
     <row r="2">
       <c r="A2" s="1" t="inlineStr">
         <is>
-          <t>Última actualización: 08:53:32</t>
+          <t>Última actualización: 09:51:48</t>
         </is>
       </c>
     </row>
     <row r="3">
       <c r="A3" s="1" t="inlineStr">
         <is>
-          <t>Total filas: 9</t>
+          <t>Total filas: 12</t>
         </is>
       </c>
     </row>
@@ -1735,23 +2035,98 @@
     <row r="14">
       <c r="A14" t="inlineStr">
         <is>
+          <t>09:51:48</t>
+        </is>
+      </c>
+      <c r="B14" t="inlineStr">
+        <is>
+          <t>09:54</t>
+        </is>
+      </c>
+      <c r="C14" t="inlineStr">
+        <is>
+          <t>215C_EL PATO</t>
+        </is>
+      </c>
+      <c r="D14" t="n">
+        <v>3</v>
+      </c>
+      <c r="E14" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="15">
+      <c r="A15" t="inlineStr">
+        <is>
           <t>08:53:32</t>
         </is>
       </c>
-      <c r="B14" t="inlineStr">
+      <c r="B15" t="inlineStr">
         <is>
           <t>09:55</t>
         </is>
       </c>
-      <c r="C14" t="inlineStr">
+      <c r="C15" t="inlineStr">
         <is>
           <t>215C_EL PATO</t>
         </is>
       </c>
-      <c r="D14" t="n">
+      <c r="D15" t="n">
         <v>62</v>
       </c>
-      <c r="E14" t="inlineStr">
+      <c r="E15" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="16">
+      <c r="A16" t="inlineStr">
+        <is>
+          <t>09:51:48</t>
+        </is>
+      </c>
+      <c r="B16" t="inlineStr">
+        <is>
+          <t>11:34</t>
+        </is>
+      </c>
+      <c r="C16" t="inlineStr">
+        <is>
+          <t>215C_EL PATO</t>
+        </is>
+      </c>
+      <c r="D16" t="n">
+        <v>103</v>
+      </c>
+      <c r="E16" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="17">
+      <c r="A17" t="inlineStr">
+        <is>
+          <t>09:51:48</t>
+        </is>
+      </c>
+      <c r="B17" t="inlineStr">
+        <is>
+          <t>11:44</t>
+        </is>
+      </c>
+      <c r="C17" t="inlineStr">
+        <is>
+          <t>215B_EL PATO</t>
+        </is>
+      </c>
+      <c r="D17" t="n">
+        <v>113</v>
+      </c>
+      <c r="E17" t="inlineStr">
         <is>
           <t>LP1912</t>
         </is>
@@ -1768,7 +2143,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E15"/>
+  <dimension ref="A1:E19"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -1781,14 +2156,14 @@
     <row r="2">
       <c r="A2" s="1" t="inlineStr">
         <is>
-          <t>Última actualización: 08:53:32</t>
+          <t>Última actualización: 09:51:48</t>
         </is>
       </c>
     </row>
     <row r="3">
       <c r="A3" s="1" t="inlineStr">
         <is>
-          <t>Total filas: 10</t>
+          <t>Total filas: 14</t>
         </is>
       </c>
     </row>
@@ -1997,12 +2372,12 @@
     <row r="13">
       <c r="A13" t="inlineStr">
         <is>
-          <t>08:53:32</t>
+          <t>09:51:48</t>
         </is>
       </c>
       <c r="B13" t="inlineStr">
         <is>
-          <t>10:18</t>
+          <t>10:17</t>
         </is>
       </c>
       <c r="C13" t="inlineStr">
@@ -2011,7 +2386,7 @@
         </is>
       </c>
       <c r="D13" t="n">
-        <v>85</v>
+        <v>26</v>
       </c>
       <c r="E13" t="inlineStr">
         <is>
@@ -2027,45 +2402,145 @@
       </c>
       <c r="B14" t="inlineStr">
         <is>
-          <t>10:30</t>
+          <t>10:18</t>
         </is>
       </c>
       <c r="C14" t="inlineStr">
         <is>
-          <t>215B_LP-P MOR-1 Y 57</t>
+          <t>215C_LA PLATA</t>
         </is>
       </c>
       <c r="D14" t="n">
-        <v>97</v>
+        <v>85</v>
       </c>
       <c r="E14" t="inlineStr">
         <is>
-          <t>L6173</t>
+          <t>L6203</t>
         </is>
       </c>
     </row>
     <row r="15">
       <c r="A15" t="inlineStr">
         <is>
+          <t>09:51:48</t>
+        </is>
+      </c>
+      <c r="B15" t="inlineStr">
+        <is>
+          <t>10:29</t>
+        </is>
+      </c>
+      <c r="C15" t="inlineStr">
+        <is>
+          <t>215B_LP-P MOR-1 Y 57</t>
+        </is>
+      </c>
+      <c r="D15" t="n">
+        <v>38</v>
+      </c>
+      <c r="E15" t="inlineStr">
+        <is>
+          <t>L6173</t>
+        </is>
+      </c>
+    </row>
+    <row r="16">
+      <c r="A16" t="inlineStr">
+        <is>
           <t>08:53:32</t>
         </is>
       </c>
-      <c r="B15" t="inlineStr">
+      <c r="B16" t="inlineStr">
+        <is>
+          <t>10:30</t>
+        </is>
+      </c>
+      <c r="C16" t="inlineStr">
+        <is>
+          <t>215B_LP-P MOR-1 Y 57</t>
+        </is>
+      </c>
+      <c r="D16" t="n">
+        <v>97</v>
+      </c>
+      <c r="E16" t="inlineStr">
+        <is>
+          <t>L6173</t>
+        </is>
+      </c>
+    </row>
+    <row r="17">
+      <c r="A17" t="inlineStr">
+        <is>
+          <t>09:51:48</t>
+        </is>
+      </c>
+      <c r="B17" t="inlineStr">
+        <is>
+          <t>10:42</t>
+        </is>
+      </c>
+      <c r="C17" t="inlineStr">
+        <is>
+          <t>215A_LA PLATA</t>
+        </is>
+      </c>
+      <c r="D17" t="n">
+        <v>51</v>
+      </c>
+      <c r="E17" t="inlineStr">
+        <is>
+          <t>L6173</t>
+        </is>
+      </c>
+    </row>
+    <row r="18">
+      <c r="A18" t="inlineStr">
+        <is>
+          <t>08:53:32</t>
+        </is>
+      </c>
+      <c r="B18" t="inlineStr">
         <is>
           <t>10:43</t>
         </is>
       </c>
-      <c r="C15" t="inlineStr">
+      <c r="C18" t="inlineStr">
         <is>
           <t>215A_LA PLATA</t>
         </is>
       </c>
-      <c r="D15" t="n">
+      <c r="D18" t="n">
         <v>110</v>
       </c>
-      <c r="E15" t="inlineStr">
+      <c r="E18" t="inlineStr">
         <is>
           <t>L6173</t>
+        </is>
+      </c>
+    </row>
+    <row r="19">
+      <c r="A19" t="inlineStr">
+        <is>
+          <t>09:51:48</t>
+        </is>
+      </c>
+      <c r="B19" t="inlineStr">
+        <is>
+          <t>11:22</t>
+        </is>
+      </c>
+      <c r="C19" t="inlineStr">
+        <is>
+          <t>215C_LA PLATA</t>
+        </is>
+      </c>
+      <c r="D19" t="n">
+        <v>91</v>
+      </c>
+      <c r="E19" t="inlineStr">
+        <is>
+          <t>L6203</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
📊 Horarios actualizados Línea 141 - 3030
</commit_message>
<xml_diff>
--- a/data/horarios-141-2026-05-17.xlsx
+++ b/data/horarios-141-2026-05-17.xlsx
@@ -419,7 +419,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E57"/>
+  <dimension ref="A1:E73"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -432,14 +432,14 @@
     <row r="2">
       <c r="A2" s="1" t="inlineStr">
         <is>
-          <t>Última actualización: 09:51:48</t>
+          <t>Última actualización: 11:19:53</t>
         </is>
       </c>
     </row>
     <row r="3">
       <c r="A3" s="1" t="inlineStr">
         <is>
-          <t>Total filas: 52</t>
+          <t>Total filas: 68</t>
         </is>
       </c>
     </row>
@@ -558,7 +558,7 @@
       </c>
       <c r="C9" t="inlineStr">
         <is>
-          <t>23_HERNANDEZ</t>
+          <t>14_ABASTO</t>
         </is>
       </c>
       <c r="D9" t="n">
@@ -583,7 +583,7 @@
       </c>
       <c r="C10" t="inlineStr">
         <is>
-          <t>14_ABASTO</t>
+          <t>23_HERNANDEZ</t>
         </is>
       </c>
       <c r="D10" t="n">
@@ -908,7 +908,7 @@
       </c>
       <c r="C23" t="inlineStr">
         <is>
-          <t>215C_EL PATO</t>
+          <t>215B_EL PATO</t>
         </is>
       </c>
       <c r="D23" t="n">
@@ -933,7 +933,7 @@
       </c>
       <c r="C24" t="inlineStr">
         <is>
-          <t>215B_EL PATO</t>
+          <t>215C_EL PATO</t>
         </is>
       </c>
       <c r="D24" t="n">
@@ -1698,12 +1698,12 @@
     <row r="55">
       <c r="A55" t="inlineStr">
         <is>
-          <t>09:51:48</t>
+          <t>11:19:53</t>
         </is>
       </c>
       <c r="B55" t="inlineStr">
         <is>
-          <t>11:24</t>
+          <t>11:23</t>
         </is>
       </c>
       <c r="C55" t="inlineStr">
@@ -1712,7 +1712,7 @@
         </is>
       </c>
       <c r="D55" t="n">
-        <v>93</v>
+        <v>4</v>
       </c>
       <c r="E55" t="inlineStr">
         <is>
@@ -1728,16 +1728,16 @@
       </c>
       <c r="B56" t="inlineStr">
         <is>
-          <t>11:34</t>
+          <t>11:24</t>
         </is>
       </c>
       <c r="C56" t="inlineStr">
         <is>
-          <t>215C_EL PATO</t>
+          <t>10_OLMOS</t>
         </is>
       </c>
       <c r="D56" t="n">
-        <v>103</v>
+        <v>93</v>
       </c>
       <c r="E56" t="inlineStr">
         <is>
@@ -1748,23 +1748,423 @@
     <row r="57">
       <c r="A57" t="inlineStr">
         <is>
-          <t>09:51:48</t>
+          <t>11:19:53</t>
         </is>
       </c>
       <c r="B57" t="inlineStr">
         <is>
+          <t>11:34</t>
+        </is>
+      </c>
+      <c r="C57" t="inlineStr">
+        <is>
+          <t>215C_EL PATO</t>
+        </is>
+      </c>
+      <c r="D57" t="n">
+        <v>15</v>
+      </c>
+      <c r="E57" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="58">
+      <c r="A58" t="inlineStr">
+        <is>
+          <t>11:19:53</t>
+        </is>
+      </c>
+      <c r="B58" t="inlineStr">
+        <is>
+          <t>11:36</t>
+        </is>
+      </c>
+      <c r="C58" t="inlineStr">
+        <is>
+          <t>16_SANTA ANA</t>
+        </is>
+      </c>
+      <c r="D58" t="n">
+        <v>17</v>
+      </c>
+      <c r="E58" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="59">
+      <c r="A59" t="inlineStr">
+        <is>
+          <t>11:19:53</t>
+        </is>
+      </c>
+      <c r="B59" t="inlineStr">
+        <is>
+          <t>11:41</t>
+        </is>
+      </c>
+      <c r="C59" t="inlineStr">
+        <is>
+          <t>23_HERNANDEZ</t>
+        </is>
+      </c>
+      <c r="D59" t="n">
+        <v>22</v>
+      </c>
+      <c r="E59" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="60">
+      <c r="A60" t="inlineStr">
+        <is>
+          <t>11:19:53</t>
+        </is>
+      </c>
+      <c r="B60" t="inlineStr">
+        <is>
           <t>11:44</t>
         </is>
       </c>
-      <c r="C57" t="inlineStr">
+      <c r="C60" t="inlineStr">
         <is>
           <t>215B_EL PATO</t>
         </is>
       </c>
-      <c r="D57" t="n">
-        <v>113</v>
-      </c>
-      <c r="E57" t="inlineStr">
+      <c r="D60" t="n">
+        <v>25</v>
+      </c>
+      <c r="E60" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="61">
+      <c r="A61" t="inlineStr">
+        <is>
+          <t>11:19:53</t>
+        </is>
+      </c>
+      <c r="B61" t="inlineStr">
+        <is>
+          <t>11:54</t>
+        </is>
+      </c>
+      <c r="C61" t="inlineStr">
+        <is>
+          <t>16_P MOR-SANTA ANA</t>
+        </is>
+      </c>
+      <c r="D61" t="n">
+        <v>35</v>
+      </c>
+      <c r="E61" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="62">
+      <c r="A62" t="inlineStr">
+        <is>
+          <t>11:19:53</t>
+        </is>
+      </c>
+      <c r="B62" t="inlineStr">
+        <is>
+          <t>11:55</t>
+        </is>
+      </c>
+      <c r="C62" t="inlineStr">
+        <is>
+          <t>17_ROMERO</t>
+        </is>
+      </c>
+      <c r="D62" t="n">
+        <v>36</v>
+      </c>
+      <c r="E62" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="63">
+      <c r="A63" t="inlineStr">
+        <is>
+          <t>11:19:53</t>
+        </is>
+      </c>
+      <c r="B63" t="inlineStr">
+        <is>
+          <t>12:03</t>
+        </is>
+      </c>
+      <c r="C63" t="inlineStr">
+        <is>
+          <t>225_GOMEZ</t>
+        </is>
+      </c>
+      <c r="D63" t="n">
+        <v>44</v>
+      </c>
+      <c r="E63" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="64">
+      <c r="A64" t="inlineStr">
+        <is>
+          <t>11:19:53</t>
+        </is>
+      </c>
+      <c r="B64" t="inlineStr">
+        <is>
+          <t>12:15</t>
+        </is>
+      </c>
+      <c r="C64" t="inlineStr">
+        <is>
+          <t>15_ABASTO</t>
+        </is>
+      </c>
+      <c r="D64" t="n">
+        <v>56</v>
+      </c>
+      <c r="E64" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="65">
+      <c r="A65" t="inlineStr">
+        <is>
+          <t>11:19:53</t>
+        </is>
+      </c>
+      <c r="B65" t="inlineStr">
+        <is>
+          <t>12:24</t>
+        </is>
+      </c>
+      <c r="C65" t="inlineStr">
+        <is>
+          <t>11_ETCHEVERRY</t>
+        </is>
+      </c>
+      <c r="D65" t="n">
+        <v>65</v>
+      </c>
+      <c r="E65" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="66">
+      <c r="A66" t="inlineStr">
+        <is>
+          <t>11:19:53</t>
+        </is>
+      </c>
+      <c r="B66" t="inlineStr">
+        <is>
+          <t>12:31</t>
+        </is>
+      </c>
+      <c r="C66" t="inlineStr">
+        <is>
+          <t>23_HERNANDEZ</t>
+        </is>
+      </c>
+      <c r="D66" t="n">
+        <v>72</v>
+      </c>
+      <c r="E66" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="67">
+      <c r="A67" t="inlineStr">
+        <is>
+          <t>11:19:53</t>
+        </is>
+      </c>
+      <c r="B67" t="inlineStr">
+        <is>
+          <t>12:34</t>
+        </is>
+      </c>
+      <c r="C67" t="inlineStr">
+        <is>
+          <t>27_EL RETIRO</t>
+        </is>
+      </c>
+      <c r="D67" t="n">
+        <v>75</v>
+      </c>
+      <c r="E67" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="68">
+      <c r="A68" t="inlineStr">
+        <is>
+          <t>11:19:53</t>
+        </is>
+      </c>
+      <c r="B68" t="inlineStr">
+        <is>
+          <t>12:34</t>
+        </is>
+      </c>
+      <c r="C68" t="inlineStr">
+        <is>
+          <t>17X38_ROMERO</t>
+        </is>
+      </c>
+      <c r="D68" t="n">
+        <v>75</v>
+      </c>
+      <c r="E68" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="69">
+      <c r="A69" t="inlineStr">
+        <is>
+          <t>11:19:53</t>
+        </is>
+      </c>
+      <c r="B69" t="inlineStr">
+        <is>
+          <t>12:43</t>
+        </is>
+      </c>
+      <c r="C69" t="inlineStr">
+        <is>
+          <t>14X44_ABASTO</t>
+        </is>
+      </c>
+      <c r="D69" t="n">
+        <v>84</v>
+      </c>
+      <c r="E69" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="70">
+      <c r="A70" t="inlineStr">
+        <is>
+          <t>11:19:53</t>
+        </is>
+      </c>
+      <c r="B70" t="inlineStr">
+        <is>
+          <t>12:46</t>
+        </is>
+      </c>
+      <c r="C70" t="inlineStr">
+        <is>
+          <t>16_SANTA ANA</t>
+        </is>
+      </c>
+      <c r="D70" t="n">
+        <v>87</v>
+      </c>
+      <c r="E70" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="71">
+      <c r="A71" t="inlineStr">
+        <is>
+          <t>11:19:53</t>
+        </is>
+      </c>
+      <c r="B71" t="inlineStr">
+        <is>
+          <t>12:54</t>
+        </is>
+      </c>
+      <c r="C71" t="inlineStr">
+        <is>
+          <t>215C_EL PATO</t>
+        </is>
+      </c>
+      <c r="D71" t="n">
+        <v>95</v>
+      </c>
+      <c r="E71" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="72">
+      <c r="A72" t="inlineStr">
+        <is>
+          <t>11:19:53</t>
+        </is>
+      </c>
+      <c r="B72" t="inlineStr">
+        <is>
+          <t>13:04</t>
+        </is>
+      </c>
+      <c r="C72" t="inlineStr">
+        <is>
+          <t>11_ETCHEVERRY</t>
+        </is>
+      </c>
+      <c r="D72" t="n">
+        <v>105</v>
+      </c>
+      <c r="E72" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="73">
+      <c r="A73" t="inlineStr">
+        <is>
+          <t>11:19:53</t>
+        </is>
+      </c>
+      <c r="B73" t="inlineStr">
+        <is>
+          <t>13:15</t>
+        </is>
+      </c>
+      <c r="C73" t="inlineStr">
+        <is>
+          <t>15_ABASTO</t>
+        </is>
+      </c>
+      <c r="D73" t="n">
+        <v>116</v>
+      </c>
+      <c r="E73" t="inlineStr">
         <is>
           <t>LP1912</t>
         </is>
@@ -1781,7 +2181,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E17"/>
+  <dimension ref="A1:E18"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -1794,14 +2194,14 @@
     <row r="2">
       <c r="A2" s="1" t="inlineStr">
         <is>
-          <t>Última actualización: 09:51:48</t>
+          <t>Última actualización: 11:19:53</t>
         </is>
       </c>
     </row>
     <row r="3">
       <c r="A3" s="1" t="inlineStr">
         <is>
-          <t>Total filas: 12</t>
+          <t>Total filas: 13</t>
         </is>
       </c>
     </row>
@@ -2085,7 +2485,7 @@
     <row r="16">
       <c r="A16" t="inlineStr">
         <is>
-          <t>09:51:48</t>
+          <t>11:19:53</t>
         </is>
       </c>
       <c r="B16" t="inlineStr">
@@ -2099,7 +2499,7 @@
         </is>
       </c>
       <c r="D16" t="n">
-        <v>103</v>
+        <v>15</v>
       </c>
       <c r="E16" t="inlineStr">
         <is>
@@ -2110,7 +2510,7 @@
     <row r="17">
       <c r="A17" t="inlineStr">
         <is>
-          <t>09:51:48</t>
+          <t>11:19:53</t>
         </is>
       </c>
       <c r="B17" t="inlineStr">
@@ -2124,9 +2524,34 @@
         </is>
       </c>
       <c r="D17" t="n">
-        <v>113</v>
+        <v>25</v>
       </c>
       <c r="E17" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="18">
+      <c r="A18" t="inlineStr">
+        <is>
+          <t>11:19:53</t>
+        </is>
+      </c>
+      <c r="B18" t="inlineStr">
+        <is>
+          <t>12:54</t>
+        </is>
+      </c>
+      <c r="C18" t="inlineStr">
+        <is>
+          <t>215C_EL PATO</t>
+        </is>
+      </c>
+      <c r="D18" t="n">
+        <v>95</v>
+      </c>
+      <c r="E18" t="inlineStr">
         <is>
           <t>LP1912</t>
         </is>
@@ -2143,7 +2568,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E19"/>
+  <dimension ref="A1:E20"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -2156,14 +2581,14 @@
     <row r="2">
       <c r="A2" s="1" t="inlineStr">
         <is>
-          <t>Última actualización: 09:51:48</t>
+          <t>Última actualización: 11:19:53</t>
         </is>
       </c>
     </row>
     <row r="3">
       <c r="A3" s="1" t="inlineStr">
         <is>
-          <t>Total filas: 14</t>
+          <t>Total filas: 15</t>
         </is>
       </c>
     </row>
@@ -2522,23 +2947,48 @@
     <row r="19">
       <c r="A19" t="inlineStr">
         <is>
+          <t>11:19:53</t>
+        </is>
+      </c>
+      <c r="B19" t="inlineStr">
+        <is>
+          <t>11:20</t>
+        </is>
+      </c>
+      <c r="C19" t="inlineStr">
+        <is>
+          <t>215C_LA PLATA</t>
+        </is>
+      </c>
+      <c r="D19" t="n">
+        <v>1</v>
+      </c>
+      <c r="E19" t="inlineStr">
+        <is>
+          <t>L6203</t>
+        </is>
+      </c>
+    </row>
+    <row r="20">
+      <c r="A20" t="inlineStr">
+        <is>
           <t>09:51:48</t>
         </is>
       </c>
-      <c r="B19" t="inlineStr">
+      <c r="B20" t="inlineStr">
         <is>
           <t>11:22</t>
         </is>
       </c>
-      <c r="C19" t="inlineStr">
+      <c r="C20" t="inlineStr">
         <is>
           <t>215C_LA PLATA</t>
         </is>
       </c>
-      <c r="D19" t="n">
+      <c r="D20" t="n">
         <v>91</v>
       </c>
-      <c r="E19" t="inlineStr">
+      <c r="E20" t="inlineStr">
         <is>
           <t>L6203</t>
         </is>

</xml_diff>

<commit_message>
📊 Horarios actualizados Línea 141 - 3031
</commit_message>
<xml_diff>
--- a/data/horarios-141-2026-05-17.xlsx
+++ b/data/horarios-141-2026-05-17.xlsx
@@ -419,7 +419,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E73"/>
+  <dimension ref="A1:E89"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -432,14 +432,14 @@
     <row r="2">
       <c r="A2" s="1" t="inlineStr">
         <is>
-          <t>Última actualización: 11:19:53</t>
+          <t>Última actualización: 12:31:04</t>
         </is>
       </c>
     </row>
     <row r="3">
       <c r="A3" s="1" t="inlineStr">
         <is>
-          <t>Total filas: 68</t>
+          <t>Total filas: 84</t>
         </is>
       </c>
     </row>
@@ -558,7 +558,7 @@
       </c>
       <c r="C9" t="inlineStr">
         <is>
-          <t>14_ABASTO</t>
+          <t>23_HERNANDEZ</t>
         </is>
       </c>
       <c r="D9" t="n">
@@ -583,7 +583,7 @@
       </c>
       <c r="C10" t="inlineStr">
         <is>
-          <t>23_HERNANDEZ</t>
+          <t>14_ABASTO</t>
         </is>
       </c>
       <c r="D10" t="n">
@@ -908,7 +908,7 @@
       </c>
       <c r="C23" t="inlineStr">
         <is>
-          <t>215B_EL PATO</t>
+          <t>215C_EL PATO</t>
         </is>
       </c>
       <c r="D23" t="n">
@@ -933,7 +933,7 @@
       </c>
       <c r="C24" t="inlineStr">
         <is>
-          <t>215C_EL PATO</t>
+          <t>215B_EL PATO</t>
         </is>
       </c>
       <c r="D24" t="n">
@@ -958,7 +958,7 @@
       </c>
       <c r="C25" t="inlineStr">
         <is>
-          <t>215B_EL PATO</t>
+          <t>215C_EL PATO</t>
         </is>
       </c>
       <c r="D25" t="n">
@@ -983,7 +983,7 @@
       </c>
       <c r="C26" t="inlineStr">
         <is>
-          <t>215C_EL PATO</t>
+          <t>215B_EL PATO</t>
         </is>
       </c>
       <c r="D26" t="n">
@@ -1108,7 +1108,7 @@
       </c>
       <c r="C31" t="inlineStr">
         <is>
-          <t>16_SANTA ANA</t>
+          <t>27_EL RETIRO</t>
         </is>
       </c>
       <c r="D31" t="n">
@@ -1133,7 +1133,7 @@
       </c>
       <c r="C32" t="inlineStr">
         <is>
-          <t>27_EL RETIRO</t>
+          <t>16_SANTA ANA</t>
         </is>
       </c>
       <c r="D32" t="n">
@@ -1998,21 +1998,21 @@
     <row r="67">
       <c r="A67" t="inlineStr">
         <is>
-          <t>11:19:53</t>
+          <t>12:31:04</t>
         </is>
       </c>
       <c r="B67" t="inlineStr">
         <is>
-          <t>12:34</t>
+          <t>12:33</t>
         </is>
       </c>
       <c r="C67" t="inlineStr">
         <is>
-          <t>27_EL RETIRO</t>
+          <t>23_HERNANDEZ</t>
         </is>
       </c>
       <c r="D67" t="n">
-        <v>75</v>
+        <v>2</v>
       </c>
       <c r="E67" t="inlineStr">
         <is>
@@ -2033,7 +2033,7 @@
       </c>
       <c r="C68" t="inlineStr">
         <is>
-          <t>17X38_ROMERO</t>
+          <t>27_EL RETIRO</t>
         </is>
       </c>
       <c r="D68" t="n">
@@ -2048,21 +2048,21 @@
     <row r="69">
       <c r="A69" t="inlineStr">
         <is>
-          <t>11:19:53</t>
+          <t>12:31:04</t>
         </is>
       </c>
       <c r="B69" t="inlineStr">
         <is>
-          <t>12:43</t>
+          <t>12:34</t>
         </is>
       </c>
       <c r="C69" t="inlineStr">
         <is>
-          <t>14X44_ABASTO</t>
+          <t>17X38_ROMERO</t>
         </is>
       </c>
       <c r="D69" t="n">
-        <v>84</v>
+        <v>3</v>
       </c>
       <c r="E69" t="inlineStr">
         <is>
@@ -2073,21 +2073,21 @@
     <row r="70">
       <c r="A70" t="inlineStr">
         <is>
-          <t>11:19:53</t>
+          <t>12:31:04</t>
         </is>
       </c>
       <c r="B70" t="inlineStr">
         <is>
-          <t>12:46</t>
+          <t>12:37</t>
         </is>
       </c>
       <c r="C70" t="inlineStr">
         <is>
-          <t>16_SANTA ANA</t>
+          <t>27_EL RETIRO</t>
         </is>
       </c>
       <c r="D70" t="n">
-        <v>87</v>
+        <v>6</v>
       </c>
       <c r="E70" t="inlineStr">
         <is>
@@ -2103,16 +2103,16 @@
       </c>
       <c r="B71" t="inlineStr">
         <is>
-          <t>12:54</t>
+          <t>12:43</t>
         </is>
       </c>
       <c r="C71" t="inlineStr">
         <is>
-          <t>215C_EL PATO</t>
+          <t>14X44_ABASTO</t>
         </is>
       </c>
       <c r="D71" t="n">
-        <v>95</v>
+        <v>84</v>
       </c>
       <c r="E71" t="inlineStr">
         <is>
@@ -2123,21 +2123,21 @@
     <row r="72">
       <c r="A72" t="inlineStr">
         <is>
-          <t>11:19:53</t>
+          <t>12:31:04</t>
         </is>
       </c>
       <c r="B72" t="inlineStr">
         <is>
-          <t>13:04</t>
+          <t>12:44</t>
         </is>
       </c>
       <c r="C72" t="inlineStr">
         <is>
-          <t>11_ETCHEVERRY</t>
+          <t>14X44_ABASTO</t>
         </is>
       </c>
       <c r="D72" t="n">
-        <v>105</v>
+        <v>13</v>
       </c>
       <c r="E72" t="inlineStr">
         <is>
@@ -2148,23 +2148,423 @@
     <row r="73">
       <c r="A73" t="inlineStr">
         <is>
+          <t>12:31:04</t>
+        </is>
+      </c>
+      <c r="B73" t="inlineStr">
+        <is>
+          <t>12:46</t>
+        </is>
+      </c>
+      <c r="C73" t="inlineStr">
+        <is>
+          <t>16_SANTA ANA</t>
+        </is>
+      </c>
+      <c r="D73" t="n">
+        <v>15</v>
+      </c>
+      <c r="E73" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="74">
+      <c r="A74" t="inlineStr">
+        <is>
           <t>11:19:53</t>
         </is>
       </c>
-      <c r="B73" t="inlineStr">
+      <c r="B74" t="inlineStr">
+        <is>
+          <t>12:54</t>
+        </is>
+      </c>
+      <c r="C74" t="inlineStr">
+        <is>
+          <t>215C_EL PATO</t>
+        </is>
+      </c>
+      <c r="D74" t="n">
+        <v>95</v>
+      </c>
+      <c r="E74" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="75">
+      <c r="A75" t="inlineStr">
+        <is>
+          <t>12:31:04</t>
+        </is>
+      </c>
+      <c r="B75" t="inlineStr">
+        <is>
+          <t>12:55</t>
+        </is>
+      </c>
+      <c r="C75" t="inlineStr">
+        <is>
+          <t>215C_EL PATO</t>
+        </is>
+      </c>
+      <c r="D75" t="n">
+        <v>24</v>
+      </c>
+      <c r="E75" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="76">
+      <c r="A76" t="inlineStr">
+        <is>
+          <t>11:19:53</t>
+        </is>
+      </c>
+      <c r="B76" t="inlineStr">
+        <is>
+          <t>13:04</t>
+        </is>
+      </c>
+      <c r="C76" t="inlineStr">
+        <is>
+          <t>11_ETCHEVERRY</t>
+        </is>
+      </c>
+      <c r="D76" t="n">
+        <v>105</v>
+      </c>
+      <c r="E76" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="77">
+      <c r="A77" t="inlineStr">
+        <is>
+          <t>12:31:04</t>
+        </is>
+      </c>
+      <c r="B77" t="inlineStr">
+        <is>
+          <t>13:05</t>
+        </is>
+      </c>
+      <c r="C77" t="inlineStr">
+        <is>
+          <t>11_ETCHEVERRY</t>
+        </is>
+      </c>
+      <c r="D77" t="n">
+        <v>34</v>
+      </c>
+      <c r="E77" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="78">
+      <c r="A78" t="inlineStr">
+        <is>
+          <t>12:31:04</t>
+        </is>
+      </c>
+      <c r="B78" t="inlineStr">
         <is>
           <t>13:15</t>
         </is>
       </c>
-      <c r="C73" t="inlineStr">
+      <c r="C78" t="inlineStr">
         <is>
           <t>15_ABASTO</t>
         </is>
       </c>
-      <c r="D73" t="n">
-        <v>116</v>
-      </c>
-      <c r="E73" t="inlineStr">
+      <c r="D78" t="n">
+        <v>44</v>
+      </c>
+      <c r="E78" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="79">
+      <c r="A79" t="inlineStr">
+        <is>
+          <t>12:31:04</t>
+        </is>
+      </c>
+      <c r="B79" t="inlineStr">
+        <is>
+          <t>13:22</t>
+        </is>
+      </c>
+      <c r="C79" t="inlineStr">
+        <is>
+          <t>23_HERNANDEZ</t>
+        </is>
+      </c>
+      <c r="D79" t="n">
+        <v>51</v>
+      </c>
+      <c r="E79" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="80">
+      <c r="A80" t="inlineStr">
+        <is>
+          <t>12:31:04</t>
+        </is>
+      </c>
+      <c r="B80" t="inlineStr">
+        <is>
+          <t>13:24</t>
+        </is>
+      </c>
+      <c r="C80" t="inlineStr">
+        <is>
+          <t>10_OLMOS</t>
+        </is>
+      </c>
+      <c r="D80" t="n">
+        <v>53</v>
+      </c>
+      <c r="E80" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="81">
+      <c r="A81" t="inlineStr">
+        <is>
+          <t>12:31:04</t>
+        </is>
+      </c>
+      <c r="B81" t="inlineStr">
+        <is>
+          <t>13:32</t>
+        </is>
+      </c>
+      <c r="C81" t="inlineStr">
+        <is>
+          <t>215A_EL PATO</t>
+        </is>
+      </c>
+      <c r="D81" t="n">
+        <v>61</v>
+      </c>
+      <c r="E81" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="82">
+      <c r="A82" t="inlineStr">
+        <is>
+          <t>12:31:04</t>
+        </is>
+      </c>
+      <c r="B82" t="inlineStr">
+        <is>
+          <t>13:45</t>
+        </is>
+      </c>
+      <c r="C82" t="inlineStr">
+        <is>
+          <t>14_ABASTO</t>
+        </is>
+      </c>
+      <c r="D82" t="n">
+        <v>74</v>
+      </c>
+      <c r="E82" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="83">
+      <c r="A83" t="inlineStr">
+        <is>
+          <t>12:31:04</t>
+        </is>
+      </c>
+      <c r="B83" t="inlineStr">
+        <is>
+          <t>13:55</t>
+        </is>
+      </c>
+      <c r="C83" t="inlineStr">
+        <is>
+          <t>17_ROMERO</t>
+        </is>
+      </c>
+      <c r="D83" t="n">
+        <v>84</v>
+      </c>
+      <c r="E83" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="84">
+      <c r="A84" t="inlineStr">
+        <is>
+          <t>12:31:04</t>
+        </is>
+      </c>
+      <c r="B84" t="inlineStr">
+        <is>
+          <t>13:56</t>
+        </is>
+      </c>
+      <c r="C84" t="inlineStr">
+        <is>
+          <t>16_SANTA ANA</t>
+        </is>
+      </c>
+      <c r="D84" t="n">
+        <v>85</v>
+      </c>
+      <c r="E84" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="85">
+      <c r="A85" t="inlineStr">
+        <is>
+          <t>12:31:04</t>
+        </is>
+      </c>
+      <c r="B85" t="inlineStr">
+        <is>
+          <t>14:04</t>
+        </is>
+      </c>
+      <c r="C85" t="inlineStr">
+        <is>
+          <t>225_GOMEZ</t>
+        </is>
+      </c>
+      <c r="D85" t="n">
+        <v>93</v>
+      </c>
+      <c r="E85" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="86">
+      <c r="A86" t="inlineStr">
+        <is>
+          <t>12:31:04</t>
+        </is>
+      </c>
+      <c r="B86" t="inlineStr">
+        <is>
+          <t>14:14</t>
+        </is>
+      </c>
+      <c r="C86" t="inlineStr">
+        <is>
+          <t>16_P MOR-SANTA ANA</t>
+        </is>
+      </c>
+      <c r="D86" t="n">
+        <v>103</v>
+      </c>
+      <c r="E86" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="87">
+      <c r="A87" t="inlineStr">
+        <is>
+          <t>12:31:04</t>
+        </is>
+      </c>
+      <c r="B87" t="inlineStr">
+        <is>
+          <t>14:14</t>
+        </is>
+      </c>
+      <c r="C87" t="inlineStr">
+        <is>
+          <t>15X38_ABASTO</t>
+        </is>
+      </c>
+      <c r="D87" t="n">
+        <v>103</v>
+      </c>
+      <c r="E87" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="88">
+      <c r="A88" t="inlineStr">
+        <is>
+          <t>12:31:04</t>
+        </is>
+      </c>
+      <c r="B88" t="inlineStr">
+        <is>
+          <t>14:17</t>
+        </is>
+      </c>
+      <c r="C88" t="inlineStr">
+        <is>
+          <t>27_EL RETIRO</t>
+        </is>
+      </c>
+      <c r="D88" t="n">
+        <v>106</v>
+      </c>
+      <c r="E88" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="89">
+      <c r="A89" t="inlineStr">
+        <is>
+          <t>12:31:04</t>
+        </is>
+      </c>
+      <c r="B89" t="inlineStr">
+        <is>
+          <t>14:25</t>
+        </is>
+      </c>
+      <c r="C89" t="inlineStr">
+        <is>
+          <t>11_ETCHEVERRY</t>
+        </is>
+      </c>
+      <c r="D89" t="n">
+        <v>114</v>
+      </c>
+      <c r="E89" t="inlineStr">
         <is>
           <t>LP1912</t>
         </is>
@@ -2181,7 +2581,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E18"/>
+  <dimension ref="A1:E20"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -2194,14 +2594,14 @@
     <row r="2">
       <c r="A2" s="1" t="inlineStr">
         <is>
-          <t>Última actualización: 11:19:53</t>
+          <t>Última actualización: 12:31:04</t>
         </is>
       </c>
     </row>
     <row r="3">
       <c r="A3" s="1" t="inlineStr">
         <is>
-          <t>Total filas: 13</t>
+          <t>Total filas: 15</t>
         </is>
       </c>
     </row>
@@ -2552,6 +2952,56 @@
         <v>95</v>
       </c>
       <c r="E18" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="19">
+      <c r="A19" t="inlineStr">
+        <is>
+          <t>12:31:04</t>
+        </is>
+      </c>
+      <c r="B19" t="inlineStr">
+        <is>
+          <t>12:55</t>
+        </is>
+      </c>
+      <c r="C19" t="inlineStr">
+        <is>
+          <t>215C_EL PATO</t>
+        </is>
+      </c>
+      <c r="D19" t="n">
+        <v>24</v>
+      </c>
+      <c r="E19" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="20">
+      <c r="A20" t="inlineStr">
+        <is>
+          <t>12:31:04</t>
+        </is>
+      </c>
+      <c r="B20" t="inlineStr">
+        <is>
+          <t>13:32</t>
+        </is>
+      </c>
+      <c r="C20" t="inlineStr">
+        <is>
+          <t>215A_EL PATO</t>
+        </is>
+      </c>
+      <c r="D20" t="n">
+        <v>61</v>
+      </c>
+      <c r="E20" t="inlineStr">
         <is>
           <t>LP1912</t>
         </is>
@@ -2568,7 +3018,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E20"/>
+  <dimension ref="A1:E22"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -2581,14 +3031,14 @@
     <row r="2">
       <c r="A2" s="1" t="inlineStr">
         <is>
-          <t>Última actualización: 11:19:53</t>
+          <t>Última actualización: 12:31:04</t>
         </is>
       </c>
     </row>
     <row r="3">
       <c r="A3" s="1" t="inlineStr">
         <is>
-          <t>Total filas: 15</t>
+          <t>Total filas: 17</t>
         </is>
       </c>
     </row>
@@ -2991,6 +3441,56 @@
       <c r="E20" t="inlineStr">
         <is>
           <t>L6203</t>
+        </is>
+      </c>
+    </row>
+    <row r="21">
+      <c r="A21" t="inlineStr">
+        <is>
+          <t>12:31:04</t>
+        </is>
+      </c>
+      <c r="B21" t="inlineStr">
+        <is>
+          <t>13:23</t>
+        </is>
+      </c>
+      <c r="C21" t="inlineStr">
+        <is>
+          <t>215C_LA PLATA</t>
+        </is>
+      </c>
+      <c r="D21" t="n">
+        <v>52</v>
+      </c>
+      <c r="E21" t="inlineStr">
+        <is>
+          <t>L6203</t>
+        </is>
+      </c>
+    </row>
+    <row r="22">
+      <c r="A22" t="inlineStr">
+        <is>
+          <t>12:31:04</t>
+        </is>
+      </c>
+      <c r="B22" t="inlineStr">
+        <is>
+          <t>13:50</t>
+        </is>
+      </c>
+      <c r="C22" t="inlineStr">
+        <is>
+          <t>215B_LP-P MOR-1 Y 57</t>
+        </is>
+      </c>
+      <c r="D22" t="n">
+        <v>79</v>
+      </c>
+      <c r="E22" t="inlineStr">
+        <is>
+          <t>L6173</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
📊 Horarios actualizados Línea 141 - 3032
</commit_message>
<xml_diff>
--- a/data/horarios-141-2026-05-17.xlsx
+++ b/data/horarios-141-2026-05-17.xlsx
@@ -419,7 +419,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E89"/>
+  <dimension ref="A1:E98"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -432,14 +432,14 @@
     <row r="2">
       <c r="A2" s="1" t="inlineStr">
         <is>
-          <t>Última actualización: 12:31:04</t>
+          <t>Última actualización: 13:33:07</t>
         </is>
       </c>
     </row>
     <row r="3">
       <c r="A3" s="1" t="inlineStr">
         <is>
-          <t>Total filas: 84</t>
+          <t>Total filas: 93</t>
         </is>
       </c>
     </row>
@@ -558,7 +558,7 @@
       </c>
       <c r="C9" t="inlineStr">
         <is>
-          <t>23_HERNANDEZ</t>
+          <t>14_ABASTO</t>
         </is>
       </c>
       <c r="D9" t="n">
@@ -583,7 +583,7 @@
       </c>
       <c r="C10" t="inlineStr">
         <is>
-          <t>14_ABASTO</t>
+          <t>23_HERNANDEZ</t>
         </is>
       </c>
       <c r="D10" t="n">
@@ -958,7 +958,7 @@
       </c>
       <c r="C25" t="inlineStr">
         <is>
-          <t>215C_EL PATO</t>
+          <t>215B_EL PATO</t>
         </is>
       </c>
       <c r="D25" t="n">
@@ -983,7 +983,7 @@
       </c>
       <c r="C26" t="inlineStr">
         <is>
-          <t>215B_EL PATO</t>
+          <t>215C_EL PATO</t>
         </is>
       </c>
       <c r="D26" t="n">
@@ -1108,7 +1108,7 @@
       </c>
       <c r="C31" t="inlineStr">
         <is>
-          <t>27_EL RETIRO</t>
+          <t>16_SANTA ANA</t>
         </is>
       </c>
       <c r="D31" t="n">
@@ -1133,7 +1133,7 @@
       </c>
       <c r="C32" t="inlineStr">
         <is>
-          <t>16_SANTA ANA</t>
+          <t>27_EL RETIRO</t>
         </is>
       </c>
       <c r="D32" t="n">
@@ -1308,7 +1308,7 @@
       </c>
       <c r="C39" t="inlineStr">
         <is>
-          <t>14_ABASTO</t>
+          <t>215C_EL PATO</t>
         </is>
       </c>
       <c r="D39" t="n">
@@ -1333,7 +1333,7 @@
       </c>
       <c r="C40" t="inlineStr">
         <is>
-          <t>215C_EL PATO</t>
+          <t>14_ABASTO</t>
         </is>
       </c>
       <c r="D40" t="n">
@@ -2373,7 +2373,7 @@
     <row r="82">
       <c r="A82" t="inlineStr">
         <is>
-          <t>12:31:04</t>
+          <t>13:33:07</t>
         </is>
       </c>
       <c r="B82" t="inlineStr">
@@ -2387,7 +2387,7 @@
         </is>
       </c>
       <c r="D82" t="n">
-        <v>74</v>
+        <v>12</v>
       </c>
       <c r="E82" t="inlineStr">
         <is>
@@ -2398,7 +2398,7 @@
     <row r="83">
       <c r="A83" t="inlineStr">
         <is>
-          <t>12:31:04</t>
+          <t>13:33:07</t>
         </is>
       </c>
       <c r="B83" t="inlineStr">
@@ -2412,7 +2412,7 @@
         </is>
       </c>
       <c r="D83" t="n">
-        <v>84</v>
+        <v>22</v>
       </c>
       <c r="E83" t="inlineStr">
         <is>
@@ -2423,7 +2423,7 @@
     <row r="84">
       <c r="A84" t="inlineStr">
         <is>
-          <t>12:31:04</t>
+          <t>13:33:07</t>
         </is>
       </c>
       <c r="B84" t="inlineStr">
@@ -2437,7 +2437,7 @@
         </is>
       </c>
       <c r="D84" t="n">
-        <v>85</v>
+        <v>23</v>
       </c>
       <c r="E84" t="inlineStr">
         <is>
@@ -2448,7 +2448,7 @@
     <row r="85">
       <c r="A85" t="inlineStr">
         <is>
-          <t>12:31:04</t>
+          <t>13:33:07</t>
         </is>
       </c>
       <c r="B85" t="inlineStr">
@@ -2462,7 +2462,7 @@
         </is>
       </c>
       <c r="D85" t="n">
-        <v>93</v>
+        <v>31</v>
       </c>
       <c r="E85" t="inlineStr">
         <is>
@@ -2473,21 +2473,21 @@
     <row r="86">
       <c r="A86" t="inlineStr">
         <is>
-          <t>12:31:04</t>
+          <t>13:33:07</t>
         </is>
       </c>
       <c r="B86" t="inlineStr">
         <is>
-          <t>14:14</t>
+          <t>14:12</t>
         </is>
       </c>
       <c r="C86" t="inlineStr">
         <is>
-          <t>16_P MOR-SANTA ANA</t>
+          <t>23_HERNANDEZ</t>
         </is>
       </c>
       <c r="D86" t="n">
-        <v>103</v>
+        <v>39</v>
       </c>
       <c r="E86" t="inlineStr">
         <is>
@@ -2498,7 +2498,7 @@
     <row r="87">
       <c r="A87" t="inlineStr">
         <is>
-          <t>12:31:04</t>
+          <t>13:33:07</t>
         </is>
       </c>
       <c r="B87" t="inlineStr">
@@ -2508,11 +2508,11 @@
       </c>
       <c r="C87" t="inlineStr">
         <is>
-          <t>15X38_ABASTO</t>
+          <t>16_P MOR-SANTA ANA</t>
         </is>
       </c>
       <c r="D87" t="n">
-        <v>103</v>
+        <v>41</v>
       </c>
       <c r="E87" t="inlineStr">
         <is>
@@ -2523,21 +2523,21 @@
     <row r="88">
       <c r="A88" t="inlineStr">
         <is>
-          <t>12:31:04</t>
+          <t>13:33:07</t>
         </is>
       </c>
       <c r="B88" t="inlineStr">
         <is>
-          <t>14:17</t>
+          <t>14:14</t>
         </is>
       </c>
       <c r="C88" t="inlineStr">
         <is>
-          <t>27_EL RETIRO</t>
+          <t>15X38_ABASTO</t>
         </is>
       </c>
       <c r="D88" t="n">
-        <v>106</v>
+        <v>41</v>
       </c>
       <c r="E88" t="inlineStr">
         <is>
@@ -2548,23 +2548,248 @@
     <row r="89">
       <c r="A89" t="inlineStr">
         <is>
-          <t>12:31:04</t>
+          <t>13:33:07</t>
         </is>
       </c>
       <c r="B89" t="inlineStr">
         <is>
+          <t>14:17</t>
+        </is>
+      </c>
+      <c r="C89" t="inlineStr">
+        <is>
+          <t>27_EL RETIRO</t>
+        </is>
+      </c>
+      <c r="D89" t="n">
+        <v>44</v>
+      </c>
+      <c r="E89" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="90">
+      <c r="A90" t="inlineStr">
+        <is>
+          <t>13:33:07</t>
+        </is>
+      </c>
+      <c r="B90" t="inlineStr">
+        <is>
           <t>14:25</t>
         </is>
       </c>
-      <c r="C89" t="inlineStr">
+      <c r="C90" t="inlineStr">
         <is>
           <t>11_ETCHEVERRY</t>
         </is>
       </c>
-      <c r="D89" t="n">
-        <v>114</v>
-      </c>
-      <c r="E89" t="inlineStr">
+      <c r="D90" t="n">
+        <v>52</v>
+      </c>
+      <c r="E90" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="91">
+      <c r="A91" t="inlineStr">
+        <is>
+          <t>13:33:07</t>
+        </is>
+      </c>
+      <c r="B91" t="inlineStr">
+        <is>
+          <t>14:31</t>
+        </is>
+      </c>
+      <c r="C91" t="inlineStr">
+        <is>
+          <t>16_SANTA ANA</t>
+        </is>
+      </c>
+      <c r="D91" t="n">
+        <v>58</v>
+      </c>
+      <c r="E91" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="92">
+      <c r="A92" t="inlineStr">
+        <is>
+          <t>13:33:07</t>
+        </is>
+      </c>
+      <c r="B92" t="inlineStr">
+        <is>
+          <t>14:35</t>
+        </is>
+      </c>
+      <c r="C92" t="inlineStr">
+        <is>
+          <t>215C_EL PATO</t>
+        </is>
+      </c>
+      <c r="D92" t="n">
+        <v>62</v>
+      </c>
+      <c r="E92" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="93">
+      <c r="A93" t="inlineStr">
+        <is>
+          <t>13:33:07</t>
+        </is>
+      </c>
+      <c r="B93" t="inlineStr">
+        <is>
+          <t>14:44</t>
+        </is>
+      </c>
+      <c r="C93" t="inlineStr">
+        <is>
+          <t>10_OLMOS</t>
+        </is>
+      </c>
+      <c r="D93" t="n">
+        <v>71</v>
+      </c>
+      <c r="E93" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="94">
+      <c r="A94" t="inlineStr">
+        <is>
+          <t>13:33:07</t>
+        </is>
+      </c>
+      <c r="B94" t="inlineStr">
+        <is>
+          <t>14:55</t>
+        </is>
+      </c>
+      <c r="C94" t="inlineStr">
+        <is>
+          <t>215_EL PELIGRO</t>
+        </is>
+      </c>
+      <c r="D94" t="n">
+        <v>82</v>
+      </c>
+      <c r="E94" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="95">
+      <c r="A95" t="inlineStr">
+        <is>
+          <t>13:33:07</t>
+        </is>
+      </c>
+      <c r="B95" t="inlineStr">
+        <is>
+          <t>15:02</t>
+        </is>
+      </c>
+      <c r="C95" t="inlineStr">
+        <is>
+          <t>23_HERNANDEZ</t>
+        </is>
+      </c>
+      <c r="D95" t="n">
+        <v>89</v>
+      </c>
+      <c r="E95" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="96">
+      <c r="A96" t="inlineStr">
+        <is>
+          <t>13:33:07</t>
+        </is>
+      </c>
+      <c r="B96" t="inlineStr">
+        <is>
+          <t>15:05</t>
+        </is>
+      </c>
+      <c r="C96" t="inlineStr">
+        <is>
+          <t>215B_EL PATO</t>
+        </is>
+      </c>
+      <c r="D96" t="n">
+        <v>92</v>
+      </c>
+      <c r="E96" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="97">
+      <c r="A97" t="inlineStr">
+        <is>
+          <t>13:33:07</t>
+        </is>
+      </c>
+      <c r="B97" t="inlineStr">
+        <is>
+          <t>15:24</t>
+        </is>
+      </c>
+      <c r="C97" t="inlineStr">
+        <is>
+          <t>11X44_ETCHEVERRY</t>
+        </is>
+      </c>
+      <c r="D97" t="n">
+        <v>111</v>
+      </c>
+      <c r="E97" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="98">
+      <c r="A98" t="inlineStr">
+        <is>
+          <t>13:33:07</t>
+        </is>
+      </c>
+      <c r="B98" t="inlineStr">
+        <is>
+          <t>15:29</t>
+        </is>
+      </c>
+      <c r="C98" t="inlineStr">
+        <is>
+          <t>17_ROMERO</t>
+        </is>
+      </c>
+      <c r="D98" t="n">
+        <v>116</v>
+      </c>
+      <c r="E98" t="inlineStr">
         <is>
           <t>LP1912</t>
         </is>
@@ -2581,7 +2806,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E20"/>
+  <dimension ref="A1:E23"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -2594,14 +2819,14 @@
     <row r="2">
       <c r="A2" s="1" t="inlineStr">
         <is>
-          <t>Última actualización: 12:31:04</t>
+          <t>Última actualización: 13:33:07</t>
         </is>
       </c>
     </row>
     <row r="3">
       <c r="A3" s="1" t="inlineStr">
         <is>
-          <t>Total filas: 15</t>
+          <t>Total filas: 18</t>
         </is>
       </c>
     </row>
@@ -3002,6 +3227,81 @@
         <v>61</v>
       </c>
       <c r="E20" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="21">
+      <c r="A21" t="inlineStr">
+        <is>
+          <t>13:33:07</t>
+        </is>
+      </c>
+      <c r="B21" t="inlineStr">
+        <is>
+          <t>14:35</t>
+        </is>
+      </c>
+      <c r="C21" t="inlineStr">
+        <is>
+          <t>215C_EL PATO</t>
+        </is>
+      </c>
+      <c r="D21" t="n">
+        <v>62</v>
+      </c>
+      <c r="E21" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="22">
+      <c r="A22" t="inlineStr">
+        <is>
+          <t>13:33:07</t>
+        </is>
+      </c>
+      <c r="B22" t="inlineStr">
+        <is>
+          <t>14:55</t>
+        </is>
+      </c>
+      <c r="C22" t="inlineStr">
+        <is>
+          <t>215_EL PELIGRO</t>
+        </is>
+      </c>
+      <c r="D22" t="n">
+        <v>82</v>
+      </c>
+      <c r="E22" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="23">
+      <c r="A23" t="inlineStr">
+        <is>
+          <t>13:33:07</t>
+        </is>
+      </c>
+      <c r="B23" t="inlineStr">
+        <is>
+          <t>15:05</t>
+        </is>
+      </c>
+      <c r="C23" t="inlineStr">
+        <is>
+          <t>215B_EL PATO</t>
+        </is>
+      </c>
+      <c r="D23" t="n">
+        <v>92</v>
+      </c>
+      <c r="E23" t="inlineStr">
         <is>
           <t>LP1912</t>
         </is>
@@ -3018,7 +3318,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E22"/>
+  <dimension ref="A1:E24"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -3031,14 +3331,14 @@
     <row r="2">
       <c r="A2" s="1" t="inlineStr">
         <is>
-          <t>Última actualización: 12:31:04</t>
+          <t>Última actualización: 13:33:07</t>
         </is>
       </c>
     </row>
     <row r="3">
       <c r="A3" s="1" t="inlineStr">
         <is>
-          <t>Total filas: 17</t>
+          <t>Total filas: 19</t>
         </is>
       </c>
     </row>
@@ -3472,7 +3772,7 @@
     <row r="22">
       <c r="A22" t="inlineStr">
         <is>
-          <t>12:31:04</t>
+          <t>13:33:07</t>
         </is>
       </c>
       <c r="B22" t="inlineStr">
@@ -3486,9 +3786,59 @@
         </is>
       </c>
       <c r="D22" t="n">
-        <v>79</v>
+        <v>17</v>
       </c>
       <c r="E22" t="inlineStr">
+        <is>
+          <t>L6173</t>
+        </is>
+      </c>
+    </row>
+    <row r="23">
+      <c r="A23" t="inlineStr">
+        <is>
+          <t>13:33:07</t>
+        </is>
+      </c>
+      <c r="B23" t="inlineStr">
+        <is>
+          <t>14:43</t>
+        </is>
+      </c>
+      <c r="C23" t="inlineStr">
+        <is>
+          <t>215C_LA PLATA</t>
+        </is>
+      </c>
+      <c r="D23" t="n">
+        <v>70</v>
+      </c>
+      <c r="E23" t="inlineStr">
+        <is>
+          <t>L6203</t>
+        </is>
+      </c>
+    </row>
+    <row r="24">
+      <c r="A24" t="inlineStr">
+        <is>
+          <t>13:33:07</t>
+        </is>
+      </c>
+      <c r="B24" t="inlineStr">
+        <is>
+          <t>15:23</t>
+        </is>
+      </c>
+      <c r="C24" t="inlineStr">
+        <is>
+          <t>215A_LA PLATA</t>
+        </is>
+      </c>
+      <c r="D24" t="n">
+        <v>110</v>
+      </c>
+      <c r="E24" t="inlineStr">
         <is>
           <t>L6173</t>
         </is>

</xml_diff>

<commit_message>
📊 Horarios actualizados Línea 141 - 3033
</commit_message>
<xml_diff>
--- a/data/horarios-141-2026-05-17.xlsx
+++ b/data/horarios-141-2026-05-17.xlsx
@@ -419,7 +419,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E98"/>
+  <dimension ref="A1:E110"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -432,14 +432,14 @@
     <row r="2">
       <c r="A2" s="1" t="inlineStr">
         <is>
-          <t>Última actualización: 13:33:07</t>
+          <t>Última actualización: 14:35:05</t>
         </is>
       </c>
     </row>
     <row r="3">
       <c r="A3" s="1" t="inlineStr">
         <is>
-          <t>Total filas: 93</t>
+          <t>Total filas: 105</t>
         </is>
       </c>
     </row>
@@ -958,7 +958,7 @@
       </c>
       <c r="C25" t="inlineStr">
         <is>
-          <t>215B_EL PATO</t>
+          <t>215C_EL PATO</t>
         </is>
       </c>
       <c r="D25" t="n">
@@ -983,7 +983,7 @@
       </c>
       <c r="C26" t="inlineStr">
         <is>
-          <t>215C_EL PATO</t>
+          <t>215B_EL PATO</t>
         </is>
       </c>
       <c r="D26" t="n">
@@ -2508,7 +2508,7 @@
       </c>
       <c r="C87" t="inlineStr">
         <is>
-          <t>16_P MOR-SANTA ANA</t>
+          <t>15X38_ABASTO</t>
         </is>
       </c>
       <c r="D87" t="n">
@@ -2533,7 +2533,7 @@
       </c>
       <c r="C88" t="inlineStr">
         <is>
-          <t>15X38_ABASTO</t>
+          <t>16_P MOR-SANTA ANA</t>
         </is>
       </c>
       <c r="D88" t="n">
@@ -2623,7 +2623,7 @@
     <row r="92">
       <c r="A92" t="inlineStr">
         <is>
-          <t>13:33:07</t>
+          <t>14:35:05</t>
         </is>
       </c>
       <c r="B92" t="inlineStr">
@@ -2637,7 +2637,7 @@
         </is>
       </c>
       <c r="D92" t="n">
-        <v>62</v>
+        <v>0</v>
       </c>
       <c r="E92" t="inlineStr">
         <is>
@@ -2648,7 +2648,7 @@
     <row r="93">
       <c r="A93" t="inlineStr">
         <is>
-          <t>13:33:07</t>
+          <t>14:35:05</t>
         </is>
       </c>
       <c r="B93" t="inlineStr">
@@ -2662,7 +2662,7 @@
         </is>
       </c>
       <c r="D93" t="n">
-        <v>71</v>
+        <v>9</v>
       </c>
       <c r="E93" t="inlineStr">
         <is>
@@ -2673,7 +2673,7 @@
     <row r="94">
       <c r="A94" t="inlineStr">
         <is>
-          <t>13:33:07</t>
+          <t>14:35:05</t>
         </is>
       </c>
       <c r="B94" t="inlineStr">
@@ -2687,7 +2687,7 @@
         </is>
       </c>
       <c r="D94" t="n">
-        <v>82</v>
+        <v>20</v>
       </c>
       <c r="E94" t="inlineStr">
         <is>
@@ -2698,7 +2698,7 @@
     <row r="95">
       <c r="A95" t="inlineStr">
         <is>
-          <t>13:33:07</t>
+          <t>14:35:05</t>
         </is>
       </c>
       <c r="B95" t="inlineStr">
@@ -2712,7 +2712,7 @@
         </is>
       </c>
       <c r="D95" t="n">
-        <v>89</v>
+        <v>27</v>
       </c>
       <c r="E95" t="inlineStr">
         <is>
@@ -2723,7 +2723,7 @@
     <row r="96">
       <c r="A96" t="inlineStr">
         <is>
-          <t>13:33:07</t>
+          <t>14:35:05</t>
         </is>
       </c>
       <c r="B96" t="inlineStr">
@@ -2737,7 +2737,7 @@
         </is>
       </c>
       <c r="D96" t="n">
-        <v>92</v>
+        <v>30</v>
       </c>
       <c r="E96" t="inlineStr">
         <is>
@@ -2748,21 +2748,21 @@
     <row r="97">
       <c r="A97" t="inlineStr">
         <is>
-          <t>13:33:07</t>
+          <t>14:35:05</t>
         </is>
       </c>
       <c r="B97" t="inlineStr">
         <is>
-          <t>15:24</t>
+          <t>15:06</t>
         </is>
       </c>
       <c r="C97" t="inlineStr">
         <is>
-          <t>11X44_ETCHEVERRY</t>
+          <t>16_SANTA ANA</t>
         </is>
       </c>
       <c r="D97" t="n">
-        <v>111</v>
+        <v>31</v>
       </c>
       <c r="E97" t="inlineStr">
         <is>
@@ -2773,23 +2773,323 @@
     <row r="98">
       <c r="A98" t="inlineStr">
         <is>
+          <t>14:35:05</t>
+        </is>
+      </c>
+      <c r="B98" t="inlineStr">
+        <is>
+          <t>15:15</t>
+        </is>
+      </c>
+      <c r="C98" t="inlineStr">
+        <is>
+          <t>17_ROMERO</t>
+        </is>
+      </c>
+      <c r="D98" t="n">
+        <v>40</v>
+      </c>
+      <c r="E98" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="99">
+      <c r="A99" t="inlineStr">
+        <is>
+          <t>14:35:05</t>
+        </is>
+      </c>
+      <c r="B99" t="inlineStr">
+        <is>
+          <t>15:24</t>
+        </is>
+      </c>
+      <c r="C99" t="inlineStr">
+        <is>
+          <t>11X44_ETCHEVERRY</t>
+        </is>
+      </c>
+      <c r="D99" t="n">
+        <v>49</v>
+      </c>
+      <c r="E99" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="100">
+      <c r="A100" t="inlineStr">
+        <is>
           <t>13:33:07</t>
         </is>
       </c>
-      <c r="B98" t="inlineStr">
+      <c r="B100" t="inlineStr">
         <is>
           <t>15:29</t>
         </is>
       </c>
-      <c r="C98" t="inlineStr">
+      <c r="C100" t="inlineStr">
         <is>
           <t>17_ROMERO</t>
         </is>
       </c>
-      <c r="D98" t="n">
+      <c r="D100" t="n">
         <v>116</v>
       </c>
-      <c r="E98" t="inlineStr">
+      <c r="E100" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="101">
+      <c r="A101" t="inlineStr">
+        <is>
+          <t>14:35:05</t>
+        </is>
+      </c>
+      <c r="B101" t="inlineStr">
+        <is>
+          <t>15:35</t>
+        </is>
+      </c>
+      <c r="C101" t="inlineStr">
+        <is>
+          <t>215C_EL PATO</t>
+        </is>
+      </c>
+      <c r="D101" t="n">
+        <v>60</v>
+      </c>
+      <c r="E101" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="102">
+      <c r="A102" t="inlineStr">
+        <is>
+          <t>14:35:05</t>
+        </is>
+      </c>
+      <c r="B102" t="inlineStr">
+        <is>
+          <t>15:41</t>
+        </is>
+      </c>
+      <c r="C102" t="inlineStr">
+        <is>
+          <t>16_SANTA ANA</t>
+        </is>
+      </c>
+      <c r="D102" t="n">
+        <v>66</v>
+      </c>
+      <c r="E102" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="103">
+      <c r="A103" t="inlineStr">
+        <is>
+          <t>14:35:05</t>
+        </is>
+      </c>
+      <c r="B103" t="inlineStr">
+        <is>
+          <t>15:45</t>
+        </is>
+      </c>
+      <c r="C103" t="inlineStr">
+        <is>
+          <t>11_ETCHEVERRY</t>
+        </is>
+      </c>
+      <c r="D103" t="n">
+        <v>70</v>
+      </c>
+      <c r="E103" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="104">
+      <c r="A104" t="inlineStr">
+        <is>
+          <t>14:35:05</t>
+        </is>
+      </c>
+      <c r="B104" t="inlineStr">
+        <is>
+          <t>15:48</t>
+        </is>
+      </c>
+      <c r="C104" t="inlineStr">
+        <is>
+          <t>23_HERNANDEZ</t>
+        </is>
+      </c>
+      <c r="D104" t="n">
+        <v>73</v>
+      </c>
+      <c r="E104" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="105">
+      <c r="A105" t="inlineStr">
+        <is>
+          <t>14:35:05</t>
+        </is>
+      </c>
+      <c r="B105" t="inlineStr">
+        <is>
+          <t>15:55</t>
+        </is>
+      </c>
+      <c r="C105" t="inlineStr">
+        <is>
+          <t>15_ABASTO</t>
+        </is>
+      </c>
+      <c r="D105" t="n">
+        <v>80</v>
+      </c>
+      <c r="E105" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="106">
+      <c r="A106" t="inlineStr">
+        <is>
+          <t>14:35:05</t>
+        </is>
+      </c>
+      <c r="B106" t="inlineStr">
+        <is>
+          <t>15:57</t>
+        </is>
+      </c>
+      <c r="C106" t="inlineStr">
+        <is>
+          <t>27_EL RETIRO</t>
+        </is>
+      </c>
+      <c r="D106" t="n">
+        <v>82</v>
+      </c>
+      <c r="E106" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="107">
+      <c r="A107" t="inlineStr">
+        <is>
+          <t>14:35:05</t>
+        </is>
+      </c>
+      <c r="B107" t="inlineStr">
+        <is>
+          <t>16:04</t>
+        </is>
+      </c>
+      <c r="C107" t="inlineStr">
+        <is>
+          <t>10_OLMOS</t>
+        </is>
+      </c>
+      <c r="D107" t="n">
+        <v>89</v>
+      </c>
+      <c r="E107" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="108">
+      <c r="A108" t="inlineStr">
+        <is>
+          <t>14:35:05</t>
+        </is>
+      </c>
+      <c r="B108" t="inlineStr">
+        <is>
+          <t>16:14</t>
+        </is>
+      </c>
+      <c r="C108" t="inlineStr">
+        <is>
+          <t>17X38_ROMERO</t>
+        </is>
+      </c>
+      <c r="D108" t="n">
+        <v>99</v>
+      </c>
+      <c r="E108" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="109">
+      <c r="A109" t="inlineStr">
+        <is>
+          <t>14:35:05</t>
+        </is>
+      </c>
+      <c r="B109" t="inlineStr">
+        <is>
+          <t>16:25</t>
+        </is>
+      </c>
+      <c r="C109" t="inlineStr">
+        <is>
+          <t>14_ABASTO</t>
+        </is>
+      </c>
+      <c r="D109" t="n">
+        <v>110</v>
+      </c>
+      <c r="E109" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="110">
+      <c r="A110" t="inlineStr">
+        <is>
+          <t>14:35:05</t>
+        </is>
+      </c>
+      <c r="B110" t="inlineStr">
+        <is>
+          <t>16:34</t>
+        </is>
+      </c>
+      <c r="C110" t="inlineStr">
+        <is>
+          <t>16_P MOR-SANTA ANA</t>
+        </is>
+      </c>
+      <c r="D110" t="n">
+        <v>119</v>
+      </c>
+      <c r="E110" t="inlineStr">
         <is>
           <t>LP1912</t>
         </is>
@@ -2806,7 +3106,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E23"/>
+  <dimension ref="A1:E24"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -2819,14 +3119,14 @@
     <row r="2">
       <c r="A2" s="1" t="inlineStr">
         <is>
-          <t>Última actualización: 13:33:07</t>
+          <t>Última actualización: 14:35:05</t>
         </is>
       </c>
     </row>
     <row r="3">
       <c r="A3" s="1" t="inlineStr">
         <is>
-          <t>Total filas: 18</t>
+          <t>Total filas: 19</t>
         </is>
       </c>
     </row>
@@ -3235,7 +3535,7 @@
     <row r="21">
       <c r="A21" t="inlineStr">
         <is>
-          <t>13:33:07</t>
+          <t>14:35:05</t>
         </is>
       </c>
       <c r="B21" t="inlineStr">
@@ -3249,7 +3549,7 @@
         </is>
       </c>
       <c r="D21" t="n">
-        <v>62</v>
+        <v>0</v>
       </c>
       <c r="E21" t="inlineStr">
         <is>
@@ -3260,7 +3560,7 @@
     <row r="22">
       <c r="A22" t="inlineStr">
         <is>
-          <t>13:33:07</t>
+          <t>14:35:05</t>
         </is>
       </c>
       <c r="B22" t="inlineStr">
@@ -3274,7 +3574,7 @@
         </is>
       </c>
       <c r="D22" t="n">
-        <v>82</v>
+        <v>20</v>
       </c>
       <c r="E22" t="inlineStr">
         <is>
@@ -3285,7 +3585,7 @@
     <row r="23">
       <c r="A23" t="inlineStr">
         <is>
-          <t>13:33:07</t>
+          <t>14:35:05</t>
         </is>
       </c>
       <c r="B23" t="inlineStr">
@@ -3299,9 +3599,34 @@
         </is>
       </c>
       <c r="D23" t="n">
-        <v>92</v>
+        <v>30</v>
       </c>
       <c r="E23" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="24">
+      <c r="A24" t="inlineStr">
+        <is>
+          <t>14:35:05</t>
+        </is>
+      </c>
+      <c r="B24" t="inlineStr">
+        <is>
+          <t>15:35</t>
+        </is>
+      </c>
+      <c r="C24" t="inlineStr">
+        <is>
+          <t>215C_EL PATO</t>
+        </is>
+      </c>
+      <c r="D24" t="n">
+        <v>60</v>
+      </c>
+      <c r="E24" t="inlineStr">
         <is>
           <t>LP1912</t>
         </is>
@@ -3318,7 +3643,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E24"/>
+  <dimension ref="A1:E26"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -3331,14 +3656,14 @@
     <row r="2">
       <c r="A2" s="1" t="inlineStr">
         <is>
-          <t>Última actualización: 13:33:07</t>
+          <t>Última actualización: 14:35:05</t>
         </is>
       </c>
     </row>
     <row r="3">
       <c r="A3" s="1" t="inlineStr">
         <is>
-          <t>Total filas: 19</t>
+          <t>Total filas: 21</t>
         </is>
       </c>
     </row>
@@ -3797,7 +4122,7 @@
     <row r="23">
       <c r="A23" t="inlineStr">
         <is>
-          <t>13:33:07</t>
+          <t>14:35:05</t>
         </is>
       </c>
       <c r="B23" t="inlineStr">
@@ -3811,7 +4136,7 @@
         </is>
       </c>
       <c r="D23" t="n">
-        <v>70</v>
+        <v>8</v>
       </c>
       <c r="E23" t="inlineStr">
         <is>
@@ -3822,7 +4147,7 @@
     <row r="24">
       <c r="A24" t="inlineStr">
         <is>
-          <t>13:33:07</t>
+          <t>14:35:05</t>
         </is>
       </c>
       <c r="B24" t="inlineStr">
@@ -3836,9 +4161,59 @@
         </is>
       </c>
       <c r="D24" t="n">
-        <v>110</v>
+        <v>48</v>
       </c>
       <c r="E24" t="inlineStr">
+        <is>
+          <t>L6173</t>
+        </is>
+      </c>
+    </row>
+    <row r="25">
+      <c r="A25" t="inlineStr">
+        <is>
+          <t>14:35:05</t>
+        </is>
+      </c>
+      <c r="B25" t="inlineStr">
+        <is>
+          <t>16:03</t>
+        </is>
+      </c>
+      <c r="C25" t="inlineStr">
+        <is>
+          <t>215C_LA PLATA</t>
+        </is>
+      </c>
+      <c r="D25" t="n">
+        <v>88</v>
+      </c>
+      <c r="E25" t="inlineStr">
+        <is>
+          <t>L6203</t>
+        </is>
+      </c>
+    </row>
+    <row r="26">
+      <c r="A26" t="inlineStr">
+        <is>
+          <t>14:35:05</t>
+        </is>
+      </c>
+      <c r="B26" t="inlineStr">
+        <is>
+          <t>16:30</t>
+        </is>
+      </c>
+      <c r="C26" t="inlineStr">
+        <is>
+          <t>215B_LP-P MOR-40 Y 115</t>
+        </is>
+      </c>
+      <c r="D26" t="n">
+        <v>115</v>
+      </c>
+      <c r="E26" t="inlineStr">
         <is>
           <t>L6173</t>
         </is>

</xml_diff>

<commit_message>
📊 Horarios actualizados Línea 141 - 3034
</commit_message>
<xml_diff>
--- a/data/horarios-141-2026-05-17.xlsx
+++ b/data/horarios-141-2026-05-17.xlsx
@@ -419,7 +419,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E110"/>
+  <dimension ref="A1:E122"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -432,14 +432,14 @@
     <row r="2">
       <c r="A2" s="1" t="inlineStr">
         <is>
-          <t>Última actualización: 14:35:05</t>
+          <t>Última actualización: 15:38:14</t>
         </is>
       </c>
     </row>
     <row r="3">
       <c r="A3" s="1" t="inlineStr">
         <is>
-          <t>Total filas: 105</t>
+          <t>Total filas: 117</t>
         </is>
       </c>
     </row>
@@ -958,7 +958,7 @@
       </c>
       <c r="C25" t="inlineStr">
         <is>
-          <t>215C_EL PATO</t>
+          <t>215B_EL PATO</t>
         </is>
       </c>
       <c r="D25" t="n">
@@ -983,7 +983,7 @@
       </c>
       <c r="C26" t="inlineStr">
         <is>
-          <t>215B_EL PATO</t>
+          <t>215C_EL PATO</t>
         </is>
       </c>
       <c r="D26" t="n">
@@ -1108,7 +1108,7 @@
       </c>
       <c r="C31" t="inlineStr">
         <is>
-          <t>16_SANTA ANA</t>
+          <t>27_EL RETIRO</t>
         </is>
       </c>
       <c r="D31" t="n">
@@ -1133,7 +1133,7 @@
       </c>
       <c r="C32" t="inlineStr">
         <is>
-          <t>27_EL RETIRO</t>
+          <t>16_SANTA ANA</t>
         </is>
       </c>
       <c r="D32" t="n">
@@ -2873,7 +2873,7 @@
     <row r="102">
       <c r="A102" t="inlineStr">
         <is>
-          <t>14:35:05</t>
+          <t>15:38:14</t>
         </is>
       </c>
       <c r="B102" t="inlineStr">
@@ -2887,7 +2887,7 @@
         </is>
       </c>
       <c r="D102" t="n">
-        <v>66</v>
+        <v>3</v>
       </c>
       <c r="E102" t="inlineStr">
         <is>
@@ -2898,7 +2898,7 @@
     <row r="103">
       <c r="A103" t="inlineStr">
         <is>
-          <t>14:35:05</t>
+          <t>15:38:14</t>
         </is>
       </c>
       <c r="B103" t="inlineStr">
@@ -2912,7 +2912,7 @@
         </is>
       </c>
       <c r="D103" t="n">
-        <v>70</v>
+        <v>7</v>
       </c>
       <c r="E103" t="inlineStr">
         <is>
@@ -2948,21 +2948,21 @@
     <row r="105">
       <c r="A105" t="inlineStr">
         <is>
-          <t>14:35:05</t>
+          <t>15:38:14</t>
         </is>
       </c>
       <c r="B105" t="inlineStr">
         <is>
-          <t>15:55</t>
+          <t>15:51</t>
         </is>
       </c>
       <c r="C105" t="inlineStr">
         <is>
-          <t>15_ABASTO</t>
+          <t>23_HERNANDEZ</t>
         </is>
       </c>
       <c r="D105" t="n">
-        <v>80</v>
+        <v>13</v>
       </c>
       <c r="E105" t="inlineStr">
         <is>
@@ -2973,21 +2973,21 @@
     <row r="106">
       <c r="A106" t="inlineStr">
         <is>
-          <t>14:35:05</t>
+          <t>15:38:14</t>
         </is>
       </c>
       <c r="B106" t="inlineStr">
         <is>
-          <t>15:57</t>
+          <t>15:55</t>
         </is>
       </c>
       <c r="C106" t="inlineStr">
         <is>
-          <t>27_EL RETIRO</t>
+          <t>15_ABASTO</t>
         </is>
       </c>
       <c r="D106" t="n">
-        <v>82</v>
+        <v>17</v>
       </c>
       <c r="E106" t="inlineStr">
         <is>
@@ -2998,21 +2998,21 @@
     <row r="107">
       <c r="A107" t="inlineStr">
         <is>
-          <t>14:35:05</t>
+          <t>15:38:14</t>
         </is>
       </c>
       <c r="B107" t="inlineStr">
         <is>
-          <t>16:04</t>
+          <t>15:57</t>
         </is>
       </c>
       <c r="C107" t="inlineStr">
         <is>
-          <t>10_OLMOS</t>
+          <t>27_EL RETIRO</t>
         </is>
       </c>
       <c r="D107" t="n">
-        <v>89</v>
+        <v>19</v>
       </c>
       <c r="E107" t="inlineStr">
         <is>
@@ -3023,21 +3023,21 @@
     <row r="108">
       <c r="A108" t="inlineStr">
         <is>
-          <t>14:35:05</t>
+          <t>15:38:14</t>
         </is>
       </c>
       <c r="B108" t="inlineStr">
         <is>
-          <t>16:14</t>
+          <t>16:04</t>
         </is>
       </c>
       <c r="C108" t="inlineStr">
         <is>
-          <t>17X38_ROMERO</t>
+          <t>10_OLMOS</t>
         </is>
       </c>
       <c r="D108" t="n">
-        <v>99</v>
+        <v>26</v>
       </c>
       <c r="E108" t="inlineStr">
         <is>
@@ -3048,21 +3048,21 @@
     <row r="109">
       <c r="A109" t="inlineStr">
         <is>
-          <t>14:35:05</t>
+          <t>15:38:14</t>
         </is>
       </c>
       <c r="B109" t="inlineStr">
         <is>
-          <t>16:25</t>
+          <t>16:14</t>
         </is>
       </c>
       <c r="C109" t="inlineStr">
         <is>
-          <t>14_ABASTO</t>
+          <t>17X38_ROMERO</t>
         </is>
       </c>
       <c r="D109" t="n">
-        <v>110</v>
+        <v>36</v>
       </c>
       <c r="E109" t="inlineStr">
         <is>
@@ -3073,23 +3073,323 @@
     <row r="110">
       <c r="A110" t="inlineStr">
         <is>
+          <t>15:38:14</t>
+        </is>
+      </c>
+      <c r="B110" t="inlineStr">
+        <is>
+          <t>16:24</t>
+        </is>
+      </c>
+      <c r="C110" t="inlineStr">
+        <is>
+          <t>14_ABASTO</t>
+        </is>
+      </c>
+      <c r="D110" t="n">
+        <v>46</v>
+      </c>
+      <c r="E110" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="111">
+      <c r="A111" t="inlineStr">
+        <is>
           <t>14:35:05</t>
         </is>
       </c>
-      <c r="B110" t="inlineStr">
+      <c r="B111" t="inlineStr">
+        <is>
+          <t>16:25</t>
+        </is>
+      </c>
+      <c r="C111" t="inlineStr">
+        <is>
+          <t>14_ABASTO</t>
+        </is>
+      </c>
+      <c r="D111" t="n">
+        <v>110</v>
+      </c>
+      <c r="E111" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="112">
+      <c r="A112" t="inlineStr">
+        <is>
+          <t>15:38:14</t>
+        </is>
+      </c>
+      <c r="B112" t="inlineStr">
         <is>
           <t>16:34</t>
         </is>
       </c>
-      <c r="C110" t="inlineStr">
+      <c r="C112" t="inlineStr">
         <is>
           <t>16_P MOR-SANTA ANA</t>
         </is>
       </c>
-      <c r="D110" t="n">
+      <c r="D112" t="n">
+        <v>56</v>
+      </c>
+      <c r="E112" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="113">
+      <c r="A113" t="inlineStr">
+        <is>
+          <t>15:38:14</t>
+        </is>
+      </c>
+      <c r="B113" t="inlineStr">
+        <is>
+          <t>16:35</t>
+        </is>
+      </c>
+      <c r="C113" t="inlineStr">
+        <is>
+          <t>83_ALUAR</t>
+        </is>
+      </c>
+      <c r="D113" t="n">
+        <v>57</v>
+      </c>
+      <c r="E113" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="114">
+      <c r="A114" t="inlineStr">
+        <is>
+          <t>15:38:14</t>
+        </is>
+      </c>
+      <c r="B114" t="inlineStr">
+        <is>
+          <t>16:44</t>
+        </is>
+      </c>
+      <c r="C114" t="inlineStr">
+        <is>
+          <t>225_GOMEZ</t>
+        </is>
+      </c>
+      <c r="D114" t="n">
+        <v>66</v>
+      </c>
+      <c r="E114" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="115">
+      <c r="A115" t="inlineStr">
+        <is>
+          <t>15:38:14</t>
+        </is>
+      </c>
+      <c r="B115" t="inlineStr">
+        <is>
+          <t>16:51</t>
+        </is>
+      </c>
+      <c r="C115" t="inlineStr">
+        <is>
+          <t>16_SANTA ANA</t>
+        </is>
+      </c>
+      <c r="D115" t="n">
+        <v>73</v>
+      </c>
+      <c r="E115" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="116">
+      <c r="A116" t="inlineStr">
+        <is>
+          <t>15:38:14</t>
+        </is>
+      </c>
+      <c r="B116" t="inlineStr">
+        <is>
+          <t>16:55</t>
+        </is>
+      </c>
+      <c r="C116" t="inlineStr">
+        <is>
+          <t>15_ABASTO</t>
+        </is>
+      </c>
+      <c r="D116" t="n">
+        <v>77</v>
+      </c>
+      <c r="E116" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="117">
+      <c r="A117" t="inlineStr">
+        <is>
+          <t>15:38:14</t>
+        </is>
+      </c>
+      <c r="B117" t="inlineStr">
+        <is>
+          <t>17:05</t>
+        </is>
+      </c>
+      <c r="C117" t="inlineStr">
+        <is>
+          <t>11_ETCHEVERRY</t>
+        </is>
+      </c>
+      <c r="D117" t="n">
+        <v>87</v>
+      </c>
+      <c r="E117" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="118">
+      <c r="A118" t="inlineStr">
+        <is>
+          <t>15:38:14</t>
+        </is>
+      </c>
+      <c r="B118" t="inlineStr">
+        <is>
+          <t>17:15</t>
+        </is>
+      </c>
+      <c r="C118" t="inlineStr">
+        <is>
+          <t>215C_EL PATO</t>
+        </is>
+      </c>
+      <c r="D118" t="n">
+        <v>97</v>
+      </c>
+      <c r="E118" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="119">
+      <c r="A119" t="inlineStr">
+        <is>
+          <t>15:38:14</t>
+        </is>
+      </c>
+      <c r="B119" t="inlineStr">
+        <is>
+          <t>17:24</t>
+        </is>
+      </c>
+      <c r="C119" t="inlineStr">
+        <is>
+          <t>10_OLMOS</t>
+        </is>
+      </c>
+      <c r="D119" t="n">
+        <v>106</v>
+      </c>
+      <c r="E119" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="120">
+      <c r="A120" t="inlineStr">
+        <is>
+          <t>15:38:14</t>
+        </is>
+      </c>
+      <c r="B120" t="inlineStr">
+        <is>
+          <t>17:31</t>
+        </is>
+      </c>
+      <c r="C120" t="inlineStr">
+        <is>
+          <t>23_HERNANDEZ</t>
+        </is>
+      </c>
+      <c r="D120" t="n">
+        <v>113</v>
+      </c>
+      <c r="E120" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="121">
+      <c r="A121" t="inlineStr">
+        <is>
+          <t>15:38:14</t>
+        </is>
+      </c>
+      <c r="B121" t="inlineStr">
+        <is>
+          <t>17:35</t>
+        </is>
+      </c>
+      <c r="C121" t="inlineStr">
+        <is>
+          <t>17_ROMERO</t>
+        </is>
+      </c>
+      <c r="D121" t="n">
+        <v>117</v>
+      </c>
+      <c r="E121" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="122">
+      <c r="A122" t="inlineStr">
+        <is>
+          <t>15:38:14</t>
+        </is>
+      </c>
+      <c r="B122" t="inlineStr">
+        <is>
+          <t>17:37</t>
+        </is>
+      </c>
+      <c r="C122" t="inlineStr">
+        <is>
+          <t>27_EL RETIRO</t>
+        </is>
+      </c>
+      <c r="D122" t="n">
         <v>119</v>
       </c>
-      <c r="E110" t="inlineStr">
+      <c r="E122" t="inlineStr">
         <is>
           <t>LP1912</t>
         </is>
@@ -3106,7 +3406,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E24"/>
+  <dimension ref="A1:E25"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -3119,14 +3419,14 @@
     <row r="2">
       <c r="A2" s="1" t="inlineStr">
         <is>
-          <t>Última actualización: 14:35:05</t>
+          <t>Última actualización: 15:38:14</t>
         </is>
       </c>
     </row>
     <row r="3">
       <c r="A3" s="1" t="inlineStr">
         <is>
-          <t>Total filas: 19</t>
+          <t>Total filas: 20</t>
         </is>
       </c>
     </row>
@@ -3627,6 +3927,31 @@
         <v>60</v>
       </c>
       <c r="E24" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="25">
+      <c r="A25" t="inlineStr">
+        <is>
+          <t>15:38:14</t>
+        </is>
+      </c>
+      <c r="B25" t="inlineStr">
+        <is>
+          <t>17:15</t>
+        </is>
+      </c>
+      <c r="C25" t="inlineStr">
+        <is>
+          <t>215C_EL PATO</t>
+        </is>
+      </c>
+      <c r="D25" t="n">
+        <v>97</v>
+      </c>
+      <c r="E25" t="inlineStr">
         <is>
           <t>LP1912</t>
         </is>
@@ -3643,7 +3968,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E26"/>
+  <dimension ref="A1:E27"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -3656,14 +3981,14 @@
     <row r="2">
       <c r="A2" s="1" t="inlineStr">
         <is>
-          <t>Última actualización: 14:35:05</t>
+          <t>Última actualización: 15:38:14</t>
         </is>
       </c>
     </row>
     <row r="3">
       <c r="A3" s="1" t="inlineStr">
         <is>
-          <t>Total filas: 21</t>
+          <t>Total filas: 22</t>
         </is>
       </c>
     </row>
@@ -4172,7 +4497,7 @@
     <row r="25">
       <c r="A25" t="inlineStr">
         <is>
-          <t>14:35:05</t>
+          <t>15:38:14</t>
         </is>
       </c>
       <c r="B25" t="inlineStr">
@@ -4186,7 +4511,7 @@
         </is>
       </c>
       <c r="D25" t="n">
-        <v>88</v>
+        <v>25</v>
       </c>
       <c r="E25" t="inlineStr">
         <is>
@@ -4197,7 +4522,7 @@
     <row r="26">
       <c r="A26" t="inlineStr">
         <is>
-          <t>14:35:05</t>
+          <t>15:38:14</t>
         </is>
       </c>
       <c r="B26" t="inlineStr">
@@ -4211,11 +4536,36 @@
         </is>
       </c>
       <c r="D26" t="n">
-        <v>115</v>
+        <v>52</v>
       </c>
       <c r="E26" t="inlineStr">
         <is>
           <t>L6173</t>
+        </is>
+      </c>
+    </row>
+    <row r="27">
+      <c r="A27" t="inlineStr">
+        <is>
+          <t>15:38:14</t>
+        </is>
+      </c>
+      <c r="B27" t="inlineStr">
+        <is>
+          <t>17:23</t>
+        </is>
+      </c>
+      <c r="C27" t="inlineStr">
+        <is>
+          <t>215C_LA PLATA</t>
+        </is>
+      </c>
+      <c r="D27" t="n">
+        <v>105</v>
+      </c>
+      <c r="E27" t="inlineStr">
+        <is>
+          <t>L6203</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
📊 Horarios actualizados Línea 141 - 3035
</commit_message>
<xml_diff>
--- a/data/horarios-141-2026-05-17.xlsx
+++ b/data/horarios-141-2026-05-17.xlsx
@@ -419,7 +419,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E122"/>
+  <dimension ref="A1:E138"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -432,14 +432,14 @@
     <row r="2">
       <c r="A2" s="1" t="inlineStr">
         <is>
-          <t>Última actualización: 15:38:14</t>
+          <t>Última actualización: 16:46:59</t>
         </is>
       </c>
     </row>
     <row r="3">
       <c r="A3" s="1" t="inlineStr">
         <is>
-          <t>Total filas: 117</t>
+          <t>Total filas: 133</t>
         </is>
       </c>
     </row>
@@ -958,7 +958,7 @@
       </c>
       <c r="C25" t="inlineStr">
         <is>
-          <t>215B_EL PATO</t>
+          <t>215C_EL PATO</t>
         </is>
       </c>
       <c r="D25" t="n">
@@ -983,7 +983,7 @@
       </c>
       <c r="C26" t="inlineStr">
         <is>
-          <t>215C_EL PATO</t>
+          <t>215B_EL PATO</t>
         </is>
       </c>
       <c r="D26" t="n">
@@ -1108,7 +1108,7 @@
       </c>
       <c r="C31" t="inlineStr">
         <is>
-          <t>27_EL RETIRO</t>
+          <t>16_SANTA ANA</t>
         </is>
       </c>
       <c r="D31" t="n">
@@ -1133,7 +1133,7 @@
       </c>
       <c r="C32" t="inlineStr">
         <is>
-          <t>16_SANTA ANA</t>
+          <t>27_EL RETIRO</t>
         </is>
       </c>
       <c r="D32" t="n">
@@ -3198,12 +3198,12 @@
     <row r="115">
       <c r="A115" t="inlineStr">
         <is>
-          <t>15:38:14</t>
+          <t>16:46:59</t>
         </is>
       </c>
       <c r="B115" t="inlineStr">
         <is>
-          <t>16:51</t>
+          <t>16:50</t>
         </is>
       </c>
       <c r="C115" t="inlineStr">
@@ -3212,7 +3212,7 @@
         </is>
       </c>
       <c r="D115" t="n">
-        <v>73</v>
+        <v>4</v>
       </c>
       <c r="E115" t="inlineStr">
         <is>
@@ -3228,16 +3228,16 @@
       </c>
       <c r="B116" t="inlineStr">
         <is>
-          <t>16:55</t>
+          <t>16:51</t>
         </is>
       </c>
       <c r="C116" t="inlineStr">
         <is>
-          <t>15_ABASTO</t>
+          <t>16_SANTA ANA</t>
         </is>
       </c>
       <c r="D116" t="n">
-        <v>77</v>
+        <v>73</v>
       </c>
       <c r="E116" t="inlineStr">
         <is>
@@ -3248,21 +3248,21 @@
     <row r="117">
       <c r="A117" t="inlineStr">
         <is>
-          <t>15:38:14</t>
+          <t>16:46:59</t>
         </is>
       </c>
       <c r="B117" t="inlineStr">
         <is>
-          <t>17:05</t>
+          <t>16:54</t>
         </is>
       </c>
       <c r="C117" t="inlineStr">
         <is>
-          <t>11_ETCHEVERRY</t>
+          <t>15_ABASTO</t>
         </is>
       </c>
       <c r="D117" t="n">
-        <v>87</v>
+        <v>8</v>
       </c>
       <c r="E117" t="inlineStr">
         <is>
@@ -3278,16 +3278,16 @@
       </c>
       <c r="B118" t="inlineStr">
         <is>
-          <t>17:15</t>
+          <t>16:55</t>
         </is>
       </c>
       <c r="C118" t="inlineStr">
         <is>
-          <t>215C_EL PATO</t>
+          <t>15_ABASTO</t>
         </is>
       </c>
       <c r="D118" t="n">
-        <v>97</v>
+        <v>77</v>
       </c>
       <c r="E118" t="inlineStr">
         <is>
@@ -3298,21 +3298,21 @@
     <row r="119">
       <c r="A119" t="inlineStr">
         <is>
-          <t>15:38:14</t>
+          <t>16:46:59</t>
         </is>
       </c>
       <c r="B119" t="inlineStr">
         <is>
-          <t>17:24</t>
+          <t>17:04</t>
         </is>
       </c>
       <c r="C119" t="inlineStr">
         <is>
-          <t>10_OLMOS</t>
+          <t>11_ETCHEVERRY</t>
         </is>
       </c>
       <c r="D119" t="n">
-        <v>106</v>
+        <v>18</v>
       </c>
       <c r="E119" t="inlineStr">
         <is>
@@ -3328,16 +3328,16 @@
       </c>
       <c r="B120" t="inlineStr">
         <is>
-          <t>17:31</t>
+          <t>17:05</t>
         </is>
       </c>
       <c r="C120" t="inlineStr">
         <is>
-          <t>23_HERNANDEZ</t>
+          <t>11_ETCHEVERRY</t>
         </is>
       </c>
       <c r="D120" t="n">
-        <v>113</v>
+        <v>87</v>
       </c>
       <c r="E120" t="inlineStr">
         <is>
@@ -3348,21 +3348,21 @@
     <row r="121">
       <c r="A121" t="inlineStr">
         <is>
-          <t>15:38:14</t>
+          <t>16:46:59</t>
         </is>
       </c>
       <c r="B121" t="inlineStr">
         <is>
-          <t>17:35</t>
+          <t>17:14</t>
         </is>
       </c>
       <c r="C121" t="inlineStr">
         <is>
-          <t>17_ROMERO</t>
+          <t>215C_EL PATO</t>
         </is>
       </c>
       <c r="D121" t="n">
-        <v>117</v>
+        <v>28</v>
       </c>
       <c r="E121" t="inlineStr">
         <is>
@@ -3378,18 +3378,418 @@
       </c>
       <c r="B122" t="inlineStr">
         <is>
+          <t>17:15</t>
+        </is>
+      </c>
+      <c r="C122" t="inlineStr">
+        <is>
+          <t>215C_EL PATO</t>
+        </is>
+      </c>
+      <c r="D122" t="n">
+        <v>97</v>
+      </c>
+      <c r="E122" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="123">
+      <c r="A123" t="inlineStr">
+        <is>
+          <t>16:46:59</t>
+        </is>
+      </c>
+      <c r="B123" t="inlineStr">
+        <is>
+          <t>17:23</t>
+        </is>
+      </c>
+      <c r="C123" t="inlineStr">
+        <is>
+          <t>10_OLMOS</t>
+        </is>
+      </c>
+      <c r="D123" t="n">
+        <v>37</v>
+      </c>
+      <c r="E123" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="124">
+      <c r="A124" t="inlineStr">
+        <is>
+          <t>15:38:14</t>
+        </is>
+      </c>
+      <c r="B124" t="inlineStr">
+        <is>
+          <t>17:24</t>
+        </is>
+      </c>
+      <c r="C124" t="inlineStr">
+        <is>
+          <t>10_OLMOS</t>
+        </is>
+      </c>
+      <c r="D124" t="n">
+        <v>106</v>
+      </c>
+      <c r="E124" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="125">
+      <c r="A125" t="inlineStr">
+        <is>
+          <t>16:46:59</t>
+        </is>
+      </c>
+      <c r="B125" t="inlineStr">
+        <is>
+          <t>17:31</t>
+        </is>
+      </c>
+      <c r="C125" t="inlineStr">
+        <is>
+          <t>23_HERNANDEZ</t>
+        </is>
+      </c>
+      <c r="D125" t="n">
+        <v>45</v>
+      </c>
+      <c r="E125" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="126">
+      <c r="A126" t="inlineStr">
+        <is>
+          <t>16:46:59</t>
+        </is>
+      </c>
+      <c r="B126" t="inlineStr">
+        <is>
+          <t>17:34</t>
+        </is>
+      </c>
+      <c r="C126" t="inlineStr">
+        <is>
+          <t>17_ROMERO</t>
+        </is>
+      </c>
+      <c r="D126" t="n">
+        <v>48</v>
+      </c>
+      <c r="E126" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="127">
+      <c r="A127" t="inlineStr">
+        <is>
+          <t>15:38:14</t>
+        </is>
+      </c>
+      <c r="B127" t="inlineStr">
+        <is>
+          <t>17:35</t>
+        </is>
+      </c>
+      <c r="C127" t="inlineStr">
+        <is>
+          <t>17_ROMERO</t>
+        </is>
+      </c>
+      <c r="D127" t="n">
+        <v>117</v>
+      </c>
+      <c r="E127" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="128">
+      <c r="A128" t="inlineStr">
+        <is>
+          <t>16:46:59</t>
+        </is>
+      </c>
+      <c r="B128" t="inlineStr">
+        <is>
+          <t>17:36</t>
+        </is>
+      </c>
+      <c r="C128" t="inlineStr">
+        <is>
+          <t>27_EL RETIRO</t>
+        </is>
+      </c>
+      <c r="D128" t="n">
+        <v>50</v>
+      </c>
+      <c r="E128" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="129">
+      <c r="A129" t="inlineStr">
+        <is>
+          <t>15:38:14</t>
+        </is>
+      </c>
+      <c r="B129" t="inlineStr">
+        <is>
           <t>17:37</t>
         </is>
       </c>
-      <c r="C122" t="inlineStr">
+      <c r="C129" t="inlineStr">
         <is>
           <t>27_EL RETIRO</t>
         </is>
       </c>
-      <c r="D122" t="n">
+      <c r="D129" t="n">
         <v>119</v>
       </c>
-      <c r="E122" t="inlineStr">
+      <c r="E129" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="130">
+      <c r="A130" t="inlineStr">
+        <is>
+          <t>16:46:59</t>
+        </is>
+      </c>
+      <c r="B130" t="inlineStr">
+        <is>
+          <t>17:44</t>
+        </is>
+      </c>
+      <c r="C130" t="inlineStr">
+        <is>
+          <t>215B_EL PATO</t>
+        </is>
+      </c>
+      <c r="D130" t="n">
+        <v>58</v>
+      </c>
+      <c r="E130" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="131">
+      <c r="A131" t="inlineStr">
+        <is>
+          <t>16:46:59</t>
+        </is>
+      </c>
+      <c r="B131" t="inlineStr">
+        <is>
+          <t>17:54</t>
+        </is>
+      </c>
+      <c r="C131" t="inlineStr">
+        <is>
+          <t>215_EL PELIGRO</t>
+        </is>
+      </c>
+      <c r="D131" t="n">
+        <v>68</v>
+      </c>
+      <c r="E131" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="132">
+      <c r="A132" t="inlineStr">
+        <is>
+          <t>16:46:59</t>
+        </is>
+      </c>
+      <c r="B132" t="inlineStr">
+        <is>
+          <t>18:03</t>
+        </is>
+      </c>
+      <c r="C132" t="inlineStr">
+        <is>
+          <t>11X44_ETCHEVERRY</t>
+        </is>
+      </c>
+      <c r="D132" t="n">
+        <v>77</v>
+      </c>
+      <c r="E132" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="133">
+      <c r="A133" t="inlineStr">
+        <is>
+          <t>16:46:59</t>
+        </is>
+      </c>
+      <c r="B133" t="inlineStr">
+        <is>
+          <t>18:14</t>
+        </is>
+      </c>
+      <c r="C133" t="inlineStr">
+        <is>
+          <t>215C_EL PATO</t>
+        </is>
+      </c>
+      <c r="D133" t="n">
+        <v>88</v>
+      </c>
+      <c r="E133" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="134">
+      <c r="A134" t="inlineStr">
+        <is>
+          <t>16:46:59</t>
+        </is>
+      </c>
+      <c r="B134" t="inlineStr">
+        <is>
+          <t>18:19</t>
+        </is>
+      </c>
+      <c r="C134" t="inlineStr">
+        <is>
+          <t>23_HERNANDEZ</t>
+        </is>
+      </c>
+      <c r="D134" t="n">
+        <v>93</v>
+      </c>
+      <c r="E134" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="135">
+      <c r="A135" t="inlineStr">
+        <is>
+          <t>16:46:59</t>
+        </is>
+      </c>
+      <c r="B135" t="inlineStr">
+        <is>
+          <t>18:24</t>
+        </is>
+      </c>
+      <c r="C135" t="inlineStr">
+        <is>
+          <t>14_ABASTO</t>
+        </is>
+      </c>
+      <c r="D135" t="n">
+        <v>98</v>
+      </c>
+      <c r="E135" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="136">
+      <c r="A136" t="inlineStr">
+        <is>
+          <t>16:46:59</t>
+        </is>
+      </c>
+      <c r="B136" t="inlineStr">
+        <is>
+          <t>18:33</t>
+        </is>
+      </c>
+      <c r="C136" t="inlineStr">
+        <is>
+          <t>15X38_ABASTO</t>
+        </is>
+      </c>
+      <c r="D136" t="n">
+        <v>107</v>
+      </c>
+      <c r="E136" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="137">
+      <c r="A137" t="inlineStr">
+        <is>
+          <t>16:46:59</t>
+        </is>
+      </c>
+      <c r="B137" t="inlineStr">
+        <is>
+          <t>18:35</t>
+        </is>
+      </c>
+      <c r="C137" t="inlineStr">
+        <is>
+          <t>16_SANTA ANA</t>
+        </is>
+      </c>
+      <c r="D137" t="n">
+        <v>109</v>
+      </c>
+      <c r="E137" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="138">
+      <c r="A138" t="inlineStr">
+        <is>
+          <t>16:46:59</t>
+        </is>
+      </c>
+      <c r="B138" t="inlineStr">
+        <is>
+          <t>18:43</t>
+        </is>
+      </c>
+      <c r="C138" t="inlineStr">
+        <is>
+          <t>10_OLMOS</t>
+        </is>
+      </c>
+      <c r="D138" t="n">
+        <v>117</v>
+      </c>
+      <c r="E138" t="inlineStr">
         <is>
           <t>LP1912</t>
         </is>
@@ -3406,7 +3806,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E25"/>
+  <dimension ref="A1:E29"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -3419,14 +3819,14 @@
     <row r="2">
       <c r="A2" s="1" t="inlineStr">
         <is>
-          <t>Última actualización: 15:38:14</t>
+          <t>Última actualización: 16:46:59</t>
         </is>
       </c>
     </row>
     <row r="3">
       <c r="A3" s="1" t="inlineStr">
         <is>
-          <t>Total filas: 20</t>
+          <t>Total filas: 24</t>
         </is>
       </c>
     </row>
@@ -3935,23 +4335,123 @@
     <row r="25">
       <c r="A25" t="inlineStr">
         <is>
+          <t>16:46:59</t>
+        </is>
+      </c>
+      <c r="B25" t="inlineStr">
+        <is>
+          <t>17:14</t>
+        </is>
+      </c>
+      <c r="C25" t="inlineStr">
+        <is>
+          <t>215C_EL PATO</t>
+        </is>
+      </c>
+      <c r="D25" t="n">
+        <v>28</v>
+      </c>
+      <c r="E25" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="26">
+      <c r="A26" t="inlineStr">
+        <is>
           <t>15:38:14</t>
         </is>
       </c>
-      <c r="B25" t="inlineStr">
+      <c r="B26" t="inlineStr">
         <is>
           <t>17:15</t>
         </is>
       </c>
-      <c r="C25" t="inlineStr">
+      <c r="C26" t="inlineStr">
         <is>
           <t>215C_EL PATO</t>
         </is>
       </c>
-      <c r="D25" t="n">
+      <c r="D26" t="n">
         <v>97</v>
       </c>
-      <c r="E25" t="inlineStr">
+      <c r="E26" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="27">
+      <c r="A27" t="inlineStr">
+        <is>
+          <t>16:46:59</t>
+        </is>
+      </c>
+      <c r="B27" t="inlineStr">
+        <is>
+          <t>17:44</t>
+        </is>
+      </c>
+      <c r="C27" t="inlineStr">
+        <is>
+          <t>215B_EL PATO</t>
+        </is>
+      </c>
+      <c r="D27" t="n">
+        <v>58</v>
+      </c>
+      <c r="E27" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="28">
+      <c r="A28" t="inlineStr">
+        <is>
+          <t>16:46:59</t>
+        </is>
+      </c>
+      <c r="B28" t="inlineStr">
+        <is>
+          <t>17:54</t>
+        </is>
+      </c>
+      <c r="C28" t="inlineStr">
+        <is>
+          <t>215_EL PELIGRO</t>
+        </is>
+      </c>
+      <c r="D28" t="n">
+        <v>68</v>
+      </c>
+      <c r="E28" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="29">
+      <c r="A29" t="inlineStr">
+        <is>
+          <t>16:46:59</t>
+        </is>
+      </c>
+      <c r="B29" t="inlineStr">
+        <is>
+          <t>18:14</t>
+        </is>
+      </c>
+      <c r="C29" t="inlineStr">
+        <is>
+          <t>215C_EL PATO</t>
+        </is>
+      </c>
+      <c r="D29" t="n">
+        <v>88</v>
+      </c>
+      <c r="E29" t="inlineStr">
         <is>
           <t>LP1912</t>
         </is>
@@ -3968,7 +4468,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E27"/>
+  <dimension ref="A1:E29"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -3981,14 +4481,14 @@
     <row r="2">
       <c r="A2" s="1" t="inlineStr">
         <is>
-          <t>Última actualización: 15:38:14</t>
+          <t>Última actualización: 16:46:59</t>
         </is>
       </c>
     </row>
     <row r="3">
       <c r="A3" s="1" t="inlineStr">
         <is>
-          <t>Total filas: 22</t>
+          <t>Total filas: 24</t>
         </is>
       </c>
     </row>
@@ -4547,23 +5047,73 @@
     <row r="27">
       <c r="A27" t="inlineStr">
         <is>
+          <t>16:46:59</t>
+        </is>
+      </c>
+      <c r="B27" t="inlineStr">
+        <is>
+          <t>17:22</t>
+        </is>
+      </c>
+      <c r="C27" t="inlineStr">
+        <is>
+          <t>215C_LA PLATA</t>
+        </is>
+      </c>
+      <c r="D27" t="n">
+        <v>36</v>
+      </c>
+      <c r="E27" t="inlineStr">
+        <is>
+          <t>L6203</t>
+        </is>
+      </c>
+    </row>
+    <row r="28">
+      <c r="A28" t="inlineStr">
+        <is>
           <t>15:38:14</t>
         </is>
       </c>
-      <c r="B27" t="inlineStr">
+      <c r="B28" t="inlineStr">
         <is>
           <t>17:23</t>
         </is>
       </c>
-      <c r="C27" t="inlineStr">
+      <c r="C28" t="inlineStr">
         <is>
           <t>215C_LA PLATA</t>
         </is>
       </c>
-      <c r="D27" t="n">
+      <c r="D28" t="n">
         <v>105</v>
       </c>
-      <c r="E27" t="inlineStr">
+      <c r="E28" t="inlineStr">
+        <is>
+          <t>L6203</t>
+        </is>
+      </c>
+    </row>
+    <row r="29">
+      <c r="A29" t="inlineStr">
+        <is>
+          <t>16:46:59</t>
+        </is>
+      </c>
+      <c r="B29" t="inlineStr">
+        <is>
+          <t>18:44</t>
+        </is>
+      </c>
+      <c r="C29" t="inlineStr">
+        <is>
+          <t>215C_LA PLATA</t>
+        </is>
+      </c>
+      <c r="D29" t="n">
+        <v>118</v>
+      </c>
+      <c r="E29" t="inlineStr">
         <is>
           <t>L6203</t>
         </is>

</xml_diff>

<commit_message>
📊 Horarios actualizados Línea 141 - 3036
</commit_message>
<xml_diff>
--- a/data/horarios-141-2026-05-17.xlsx
+++ b/data/horarios-141-2026-05-17.xlsx
@@ -419,7 +419,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E138"/>
+  <dimension ref="A1:E155"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -432,14 +432,14 @@
     <row r="2">
       <c r="A2" s="1" t="inlineStr">
         <is>
-          <t>Última actualización: 16:46:59</t>
+          <t>Última actualización: 17:34:04</t>
         </is>
       </c>
     </row>
     <row r="3">
       <c r="A3" s="1" t="inlineStr">
         <is>
-          <t>Total filas: 133</t>
+          <t>Total filas: 150</t>
         </is>
       </c>
     </row>
@@ -558,7 +558,7 @@
       </c>
       <c r="C9" t="inlineStr">
         <is>
-          <t>14_ABASTO</t>
+          <t>23_HERNANDEZ</t>
         </is>
       </c>
       <c r="D9" t="n">
@@ -583,7 +583,7 @@
       </c>
       <c r="C10" t="inlineStr">
         <is>
-          <t>23_HERNANDEZ</t>
+          <t>14_ABASTO</t>
         </is>
       </c>
       <c r="D10" t="n">
@@ -908,7 +908,7 @@
       </c>
       <c r="C23" t="inlineStr">
         <is>
-          <t>215C_EL PATO</t>
+          <t>215B_EL PATO</t>
         </is>
       </c>
       <c r="D23" t="n">
@@ -933,7 +933,7 @@
       </c>
       <c r="C24" t="inlineStr">
         <is>
-          <t>215B_EL PATO</t>
+          <t>215C_EL PATO</t>
         </is>
       </c>
       <c r="D24" t="n">
@@ -958,7 +958,7 @@
       </c>
       <c r="C25" t="inlineStr">
         <is>
-          <t>215C_EL PATO</t>
+          <t>215B_EL PATO</t>
         </is>
       </c>
       <c r="D25" t="n">
@@ -983,7 +983,7 @@
       </c>
       <c r="C26" t="inlineStr">
         <is>
-          <t>215B_EL PATO</t>
+          <t>215C_EL PATO</t>
         </is>
       </c>
       <c r="D26" t="n">
@@ -1308,7 +1308,7 @@
       </c>
       <c r="C39" t="inlineStr">
         <is>
-          <t>215C_EL PATO</t>
+          <t>14_ABASTO</t>
         </is>
       </c>
       <c r="D39" t="n">
@@ -1333,7 +1333,7 @@
       </c>
       <c r="C40" t="inlineStr">
         <is>
-          <t>14_ABASTO</t>
+          <t>215C_EL PATO</t>
         </is>
       </c>
       <c r="D40" t="n">
@@ -2508,7 +2508,7 @@
       </c>
       <c r="C87" t="inlineStr">
         <is>
-          <t>15X38_ABASTO</t>
+          <t>16_P MOR-SANTA ANA</t>
         </is>
       </c>
       <c r="D87" t="n">
@@ -2533,7 +2533,7 @@
       </c>
       <c r="C88" t="inlineStr">
         <is>
-          <t>16_P MOR-SANTA ANA</t>
+          <t>15X38_ABASTO</t>
         </is>
       </c>
       <c r="D88" t="n">
@@ -3498,7 +3498,7 @@
     <row r="127">
       <c r="A127" t="inlineStr">
         <is>
-          <t>15:38:14</t>
+          <t>17:34:04</t>
         </is>
       </c>
       <c r="B127" t="inlineStr">
@@ -3512,7 +3512,7 @@
         </is>
       </c>
       <c r="D127" t="n">
-        <v>117</v>
+        <v>1</v>
       </c>
       <c r="E127" t="inlineStr">
         <is>
@@ -3548,7 +3548,7 @@
     <row r="129">
       <c r="A129" t="inlineStr">
         <is>
-          <t>15:38:14</t>
+          <t>17:34:04</t>
         </is>
       </c>
       <c r="B129" t="inlineStr">
@@ -3562,7 +3562,7 @@
         </is>
       </c>
       <c r="D129" t="n">
-        <v>119</v>
+        <v>3</v>
       </c>
       <c r="E129" t="inlineStr">
         <is>
@@ -3598,21 +3598,21 @@
     <row r="131">
       <c r="A131" t="inlineStr">
         <is>
-          <t>16:46:59</t>
+          <t>17:34:04</t>
         </is>
       </c>
       <c r="B131" t="inlineStr">
         <is>
-          <t>17:54</t>
+          <t>17:45</t>
         </is>
       </c>
       <c r="C131" t="inlineStr">
         <is>
-          <t>215_EL PELIGRO</t>
+          <t>215B_EL PATO</t>
         </is>
       </c>
       <c r="D131" t="n">
-        <v>68</v>
+        <v>11</v>
       </c>
       <c r="E131" t="inlineStr">
         <is>
@@ -3628,16 +3628,16 @@
       </c>
       <c r="B132" t="inlineStr">
         <is>
-          <t>18:03</t>
+          <t>17:54</t>
         </is>
       </c>
       <c r="C132" t="inlineStr">
         <is>
-          <t>11X44_ETCHEVERRY</t>
+          <t>215_EL PELIGRO</t>
         </is>
       </c>
       <c r="D132" t="n">
-        <v>77</v>
+        <v>68</v>
       </c>
       <c r="E132" t="inlineStr">
         <is>
@@ -3648,21 +3648,21 @@
     <row r="133">
       <c r="A133" t="inlineStr">
         <is>
-          <t>16:46:59</t>
+          <t>17:34:04</t>
         </is>
       </c>
       <c r="B133" t="inlineStr">
         <is>
-          <t>18:14</t>
+          <t>17:55</t>
         </is>
       </c>
       <c r="C133" t="inlineStr">
         <is>
-          <t>215C_EL PATO</t>
+          <t>215_EL PELIGRO</t>
         </is>
       </c>
       <c r="D133" t="n">
-        <v>88</v>
+        <v>21</v>
       </c>
       <c r="E133" t="inlineStr">
         <is>
@@ -3678,16 +3678,16 @@
       </c>
       <c r="B134" t="inlineStr">
         <is>
-          <t>18:19</t>
+          <t>18:03</t>
         </is>
       </c>
       <c r="C134" t="inlineStr">
         <is>
-          <t>23_HERNANDEZ</t>
+          <t>11X44_ETCHEVERRY</t>
         </is>
       </c>
       <c r="D134" t="n">
-        <v>93</v>
+        <v>77</v>
       </c>
       <c r="E134" t="inlineStr">
         <is>
@@ -3703,16 +3703,16 @@
       </c>
       <c r="B135" t="inlineStr">
         <is>
-          <t>18:24</t>
+          <t>18:14</t>
         </is>
       </c>
       <c r="C135" t="inlineStr">
         <is>
-          <t>14_ABASTO</t>
+          <t>215C_EL PATO</t>
         </is>
       </c>
       <c r="D135" t="n">
-        <v>98</v>
+        <v>88</v>
       </c>
       <c r="E135" t="inlineStr">
         <is>
@@ -3723,21 +3723,21 @@
     <row r="136">
       <c r="A136" t="inlineStr">
         <is>
-          <t>16:46:59</t>
+          <t>17:34:04</t>
         </is>
       </c>
       <c r="B136" t="inlineStr">
         <is>
-          <t>18:33</t>
+          <t>18:15</t>
         </is>
       </c>
       <c r="C136" t="inlineStr">
         <is>
-          <t>15X38_ABASTO</t>
+          <t>215C_EL PATO</t>
         </is>
       </c>
       <c r="D136" t="n">
-        <v>107</v>
+        <v>41</v>
       </c>
       <c r="E136" t="inlineStr">
         <is>
@@ -3753,16 +3753,16 @@
       </c>
       <c r="B137" t="inlineStr">
         <is>
-          <t>18:35</t>
+          <t>18:19</t>
         </is>
       </c>
       <c r="C137" t="inlineStr">
         <is>
-          <t>16_SANTA ANA</t>
+          <t>23_HERNANDEZ</t>
         </is>
       </c>
       <c r="D137" t="n">
-        <v>109</v>
+        <v>93</v>
       </c>
       <c r="E137" t="inlineStr">
         <is>
@@ -3773,23 +3773,448 @@
     <row r="138">
       <c r="A138" t="inlineStr">
         <is>
+          <t>17:34:04</t>
+        </is>
+      </c>
+      <c r="B138" t="inlineStr">
+        <is>
+          <t>18:22</t>
+        </is>
+      </c>
+      <c r="C138" t="inlineStr">
+        <is>
+          <t>23_HERNANDEZ</t>
+        </is>
+      </c>
+      <c r="D138" t="n">
+        <v>48</v>
+      </c>
+      <c r="E138" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="139">
+      <c r="A139" t="inlineStr">
+        <is>
+          <t>17:34:04</t>
+        </is>
+      </c>
+      <c r="B139" t="inlineStr">
+        <is>
+          <t>18:23</t>
+        </is>
+      </c>
+      <c r="C139" t="inlineStr">
+        <is>
+          <t>11X44_ETCHEVERRY</t>
+        </is>
+      </c>
+      <c r="D139" t="n">
+        <v>49</v>
+      </c>
+      <c r="E139" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="140">
+      <c r="A140" t="inlineStr">
+        <is>
           <t>16:46:59</t>
         </is>
       </c>
-      <c r="B138" t="inlineStr">
+      <c r="B140" t="inlineStr">
+        <is>
+          <t>18:24</t>
+        </is>
+      </c>
+      <c r="C140" t="inlineStr">
+        <is>
+          <t>14_ABASTO</t>
+        </is>
+      </c>
+      <c r="D140" t="n">
+        <v>98</v>
+      </c>
+      <c r="E140" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="141">
+      <c r="A141" t="inlineStr">
+        <is>
+          <t>17:34:04</t>
+        </is>
+      </c>
+      <c r="B141" t="inlineStr">
+        <is>
+          <t>18:25</t>
+        </is>
+      </c>
+      <c r="C141" t="inlineStr">
+        <is>
+          <t>14_ABASTO</t>
+        </is>
+      </c>
+      <c r="D141" t="n">
+        <v>51</v>
+      </c>
+      <c r="E141" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="142">
+      <c r="A142" t="inlineStr">
+        <is>
+          <t>16:46:59</t>
+        </is>
+      </c>
+      <c r="B142" t="inlineStr">
+        <is>
+          <t>18:33</t>
+        </is>
+      </c>
+      <c r="C142" t="inlineStr">
+        <is>
+          <t>15X38_ABASTO</t>
+        </is>
+      </c>
+      <c r="D142" t="n">
+        <v>107</v>
+      </c>
+      <c r="E142" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="143">
+      <c r="A143" t="inlineStr">
+        <is>
+          <t>17:34:04</t>
+        </is>
+      </c>
+      <c r="B143" t="inlineStr">
+        <is>
+          <t>18:34</t>
+        </is>
+      </c>
+      <c r="C143" t="inlineStr">
+        <is>
+          <t>15X38_ABASTO</t>
+        </is>
+      </c>
+      <c r="D143" t="n">
+        <v>60</v>
+      </c>
+      <c r="E143" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="144">
+      <c r="A144" t="inlineStr">
+        <is>
+          <t>16:46:59</t>
+        </is>
+      </c>
+      <c r="B144" t="inlineStr">
+        <is>
+          <t>18:35</t>
+        </is>
+      </c>
+      <c r="C144" t="inlineStr">
+        <is>
+          <t>16_SANTA ANA</t>
+        </is>
+      </c>
+      <c r="D144" t="n">
+        <v>109</v>
+      </c>
+      <c r="E144" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="145">
+      <c r="A145" t="inlineStr">
+        <is>
+          <t>17:34:04</t>
+        </is>
+      </c>
+      <c r="B145" t="inlineStr">
+        <is>
+          <t>18:36</t>
+        </is>
+      </c>
+      <c r="C145" t="inlineStr">
+        <is>
+          <t>16_SANTA ANA</t>
+        </is>
+      </c>
+      <c r="D145" t="n">
+        <v>62</v>
+      </c>
+      <c r="E145" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="146">
+      <c r="A146" t="inlineStr">
+        <is>
+          <t>16:46:59</t>
+        </is>
+      </c>
+      <c r="B146" t="inlineStr">
         <is>
           <t>18:43</t>
         </is>
       </c>
-      <c r="C138" t="inlineStr">
+      <c r="C146" t="inlineStr">
         <is>
           <t>10_OLMOS</t>
         </is>
       </c>
-      <c r="D138" t="n">
+      <c r="D146" t="n">
         <v>117</v>
       </c>
-      <c r="E138" t="inlineStr">
+      <c r="E146" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="147">
+      <c r="A147" t="inlineStr">
+        <is>
+          <t>17:34:04</t>
+        </is>
+      </c>
+      <c r="B147" t="inlineStr">
+        <is>
+          <t>18:44</t>
+        </is>
+      </c>
+      <c r="C147" t="inlineStr">
+        <is>
+          <t>10_OLMOS</t>
+        </is>
+      </c>
+      <c r="D147" t="n">
+        <v>70</v>
+      </c>
+      <c r="E147" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="148">
+      <c r="A148" t="inlineStr">
+        <is>
+          <t>17:34:04</t>
+        </is>
+      </c>
+      <c r="B148" t="inlineStr">
+        <is>
+          <t>18:54</t>
+        </is>
+      </c>
+      <c r="C148" t="inlineStr">
+        <is>
+          <t>16_P MOR-SANTA ANA</t>
+        </is>
+      </c>
+      <c r="D148" t="n">
+        <v>80</v>
+      </c>
+      <c r="E148" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="149">
+      <c r="A149" t="inlineStr">
+        <is>
+          <t>17:34:04</t>
+        </is>
+      </c>
+      <c r="B149" t="inlineStr">
+        <is>
+          <t>19:00</t>
+        </is>
+      </c>
+      <c r="C149" t="inlineStr">
+        <is>
+          <t>215_EL PELIGRO</t>
+        </is>
+      </c>
+      <c r="D149" t="n">
+        <v>86</v>
+      </c>
+      <c r="E149" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="150">
+      <c r="A150" t="inlineStr">
+        <is>
+          <t>17:34:04</t>
+        </is>
+      </c>
+      <c r="B150" t="inlineStr">
+        <is>
+          <t>19:05</t>
+        </is>
+      </c>
+      <c r="C150" t="inlineStr">
+        <is>
+          <t>14_ABASTO</t>
+        </is>
+      </c>
+      <c r="D150" t="n">
+        <v>91</v>
+      </c>
+      <c r="E150" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="151">
+      <c r="A151" t="inlineStr">
+        <is>
+          <t>17:34:04</t>
+        </is>
+      </c>
+      <c r="B151" t="inlineStr">
+        <is>
+          <t>19:12</t>
+        </is>
+      </c>
+      <c r="C151" t="inlineStr">
+        <is>
+          <t>23_HERNANDEZ</t>
+        </is>
+      </c>
+      <c r="D151" t="n">
+        <v>98</v>
+      </c>
+      <c r="E151" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="152">
+      <c r="A152" t="inlineStr">
+        <is>
+          <t>17:34:04</t>
+        </is>
+      </c>
+      <c r="B152" t="inlineStr">
+        <is>
+          <t>19:16</t>
+        </is>
+      </c>
+      <c r="C152" t="inlineStr">
+        <is>
+          <t>16_SANTA ANA</t>
+        </is>
+      </c>
+      <c r="D152" t="n">
+        <v>102</v>
+      </c>
+      <c r="E152" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="153">
+      <c r="A153" t="inlineStr">
+        <is>
+          <t>17:34:04</t>
+        </is>
+      </c>
+      <c r="B153" t="inlineStr">
+        <is>
+          <t>19:17</t>
+        </is>
+      </c>
+      <c r="C153" t="inlineStr">
+        <is>
+          <t>27_EL RETIRO</t>
+        </is>
+      </c>
+      <c r="D153" t="n">
+        <v>103</v>
+      </c>
+      <c r="E153" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="154">
+      <c r="A154" t="inlineStr">
+        <is>
+          <t>17:34:04</t>
+        </is>
+      </c>
+      <c r="B154" t="inlineStr">
+        <is>
+          <t>19:24</t>
+        </is>
+      </c>
+      <c r="C154" t="inlineStr">
+        <is>
+          <t>11X44_ETCHEVERRY</t>
+        </is>
+      </c>
+      <c r="D154" t="n">
+        <v>110</v>
+      </c>
+      <c r="E154" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="155">
+      <c r="A155" t="inlineStr">
+        <is>
+          <t>17:34:04</t>
+        </is>
+      </c>
+      <c r="B155" t="inlineStr">
+        <is>
+          <t>19:25</t>
+        </is>
+      </c>
+      <c r="C155" t="inlineStr">
+        <is>
+          <t>215C_EL PATO</t>
+        </is>
+      </c>
+      <c r="D155" t="n">
+        <v>111</v>
+      </c>
+      <c r="E155" t="inlineStr">
         <is>
           <t>LP1912</t>
         </is>
@@ -3806,7 +4231,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E29"/>
+  <dimension ref="A1:E34"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -3819,14 +4244,14 @@
     <row r="2">
       <c r="A2" s="1" t="inlineStr">
         <is>
-          <t>Última actualización: 16:46:59</t>
+          <t>Última actualización: 17:34:04</t>
         </is>
       </c>
     </row>
     <row r="3">
       <c r="A3" s="1" t="inlineStr">
         <is>
-          <t>Total filas: 24</t>
+          <t>Total filas: 29</t>
         </is>
       </c>
     </row>
@@ -4410,21 +4835,21 @@
     <row r="28">
       <c r="A28" t="inlineStr">
         <is>
-          <t>16:46:59</t>
+          <t>17:34:04</t>
         </is>
       </c>
       <c r="B28" t="inlineStr">
         <is>
-          <t>17:54</t>
+          <t>17:45</t>
         </is>
       </c>
       <c r="C28" t="inlineStr">
         <is>
-          <t>215_EL PELIGRO</t>
+          <t>215B_EL PATO</t>
         </is>
       </c>
       <c r="D28" t="n">
-        <v>68</v>
+        <v>11</v>
       </c>
       <c r="E28" t="inlineStr">
         <is>
@@ -4440,18 +4865,143 @@
       </c>
       <c r="B29" t="inlineStr">
         <is>
+          <t>17:54</t>
+        </is>
+      </c>
+      <c r="C29" t="inlineStr">
+        <is>
+          <t>215_EL PELIGRO</t>
+        </is>
+      </c>
+      <c r="D29" t="n">
+        <v>68</v>
+      </c>
+      <c r="E29" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="30">
+      <c r="A30" t="inlineStr">
+        <is>
+          <t>17:34:04</t>
+        </is>
+      </c>
+      <c r="B30" t="inlineStr">
+        <is>
+          <t>17:55</t>
+        </is>
+      </c>
+      <c r="C30" t="inlineStr">
+        <is>
+          <t>215_EL PELIGRO</t>
+        </is>
+      </c>
+      <c r="D30" t="n">
+        <v>21</v>
+      </c>
+      <c r="E30" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="31">
+      <c r="A31" t="inlineStr">
+        <is>
+          <t>16:46:59</t>
+        </is>
+      </c>
+      <c r="B31" t="inlineStr">
+        <is>
           <t>18:14</t>
         </is>
       </c>
-      <c r="C29" t="inlineStr">
+      <c r="C31" t="inlineStr">
         <is>
           <t>215C_EL PATO</t>
         </is>
       </c>
-      <c r="D29" t="n">
+      <c r="D31" t="n">
         <v>88</v>
       </c>
-      <c r="E29" t="inlineStr">
+      <c r="E31" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="32">
+      <c r="A32" t="inlineStr">
+        <is>
+          <t>17:34:04</t>
+        </is>
+      </c>
+      <c r="B32" t="inlineStr">
+        <is>
+          <t>18:15</t>
+        </is>
+      </c>
+      <c r="C32" t="inlineStr">
+        <is>
+          <t>215C_EL PATO</t>
+        </is>
+      </c>
+      <c r="D32" t="n">
+        <v>41</v>
+      </c>
+      <c r="E32" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="33">
+      <c r="A33" t="inlineStr">
+        <is>
+          <t>17:34:04</t>
+        </is>
+      </c>
+      <c r="B33" t="inlineStr">
+        <is>
+          <t>19:00</t>
+        </is>
+      </c>
+      <c r="C33" t="inlineStr">
+        <is>
+          <t>215_EL PELIGRO</t>
+        </is>
+      </c>
+      <c r="D33" t="n">
+        <v>86</v>
+      </c>
+      <c r="E33" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="34">
+      <c r="A34" t="inlineStr">
+        <is>
+          <t>17:34:04</t>
+        </is>
+      </c>
+      <c r="B34" t="inlineStr">
+        <is>
+          <t>19:25</t>
+        </is>
+      </c>
+      <c r="C34" t="inlineStr">
+        <is>
+          <t>215C_EL PATO</t>
+        </is>
+      </c>
+      <c r="D34" t="n">
+        <v>111</v>
+      </c>
+      <c r="E34" t="inlineStr">
         <is>
           <t>LP1912</t>
         </is>
@@ -4468,7 +5018,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E29"/>
+  <dimension ref="A1:E31"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -4481,14 +5031,14 @@
     <row r="2">
       <c r="A2" s="1" t="inlineStr">
         <is>
-          <t>Última actualización: 16:46:59</t>
+          <t>Última actualización: 17:34:04</t>
         </is>
       </c>
     </row>
     <row r="3">
       <c r="A3" s="1" t="inlineStr">
         <is>
-          <t>Total filas: 24</t>
+          <t>Total filas: 26</t>
         </is>
       </c>
     </row>
@@ -5116,6 +5666,56 @@
       <c r="E29" t="inlineStr">
         <is>
           <t>L6203</t>
+        </is>
+      </c>
+    </row>
+    <row r="30">
+      <c r="A30" t="inlineStr">
+        <is>
+          <t>17:34:04</t>
+        </is>
+      </c>
+      <c r="B30" t="inlineStr">
+        <is>
+          <t>18:45</t>
+        </is>
+      </c>
+      <c r="C30" t="inlineStr">
+        <is>
+          <t>215C_LA PLATA</t>
+        </is>
+      </c>
+      <c r="D30" t="n">
+        <v>71</v>
+      </c>
+      <c r="E30" t="inlineStr">
+        <is>
+          <t>L6203</t>
+        </is>
+      </c>
+    </row>
+    <row r="31">
+      <c r="A31" t="inlineStr">
+        <is>
+          <t>17:34:04</t>
+        </is>
+      </c>
+      <c r="B31" t="inlineStr">
+        <is>
+          <t>19:15</t>
+        </is>
+      </c>
+      <c r="C31" t="inlineStr">
+        <is>
+          <t>215B_LP-P MOR-1 Y 57</t>
+        </is>
+      </c>
+      <c r="D31" t="n">
+        <v>101</v>
+      </c>
+      <c r="E31" t="inlineStr">
+        <is>
+          <t>L6173</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
📊 Horarios actualizados Línea 141 - 3037
</commit_message>
<xml_diff>
--- a/data/horarios-141-2026-05-17.xlsx
+++ b/data/horarios-141-2026-05-17.xlsx
@@ -419,7 +419,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E155"/>
+  <dimension ref="A1:E162"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -432,14 +432,14 @@
     <row r="2">
       <c r="A2" s="1" t="inlineStr">
         <is>
-          <t>Última actualización: 17:34:04</t>
+          <t>Última actualización: 18:30:24</t>
         </is>
       </c>
     </row>
     <row r="3">
       <c r="A3" s="1" t="inlineStr">
         <is>
-          <t>Total filas: 150</t>
+          <t>Total filas: 157</t>
         </is>
       </c>
     </row>
@@ -958,7 +958,7 @@
       </c>
       <c r="C25" t="inlineStr">
         <is>
-          <t>215B_EL PATO</t>
+          <t>215C_EL PATO</t>
         </is>
       </c>
       <c r="D25" t="n">
@@ -983,7 +983,7 @@
       </c>
       <c r="C26" t="inlineStr">
         <is>
-          <t>215C_EL PATO</t>
+          <t>215B_EL PATO</t>
         </is>
       </c>
       <c r="D26" t="n">
@@ -1108,7 +1108,7 @@
       </c>
       <c r="C31" t="inlineStr">
         <is>
-          <t>16_SANTA ANA</t>
+          <t>27_EL RETIRO</t>
         </is>
       </c>
       <c r="D31" t="n">
@@ -1133,7 +1133,7 @@
       </c>
       <c r="C32" t="inlineStr">
         <is>
-          <t>27_EL RETIRO</t>
+          <t>16_SANTA ANA</t>
         </is>
       </c>
       <c r="D32" t="n">
@@ -3898,7 +3898,7 @@
     <row r="143">
       <c r="A143" t="inlineStr">
         <is>
-          <t>17:34:04</t>
+          <t>18:30:24</t>
         </is>
       </c>
       <c r="B143" t="inlineStr">
@@ -3912,7 +3912,7 @@
         </is>
       </c>
       <c r="D143" t="n">
-        <v>60</v>
+        <v>4</v>
       </c>
       <c r="E143" t="inlineStr">
         <is>
@@ -3948,7 +3948,7 @@
     <row r="145">
       <c r="A145" t="inlineStr">
         <is>
-          <t>17:34:04</t>
+          <t>18:30:24</t>
         </is>
       </c>
       <c r="B145" t="inlineStr">
@@ -3962,7 +3962,7 @@
         </is>
       </c>
       <c r="D145" t="n">
-        <v>62</v>
+        <v>6</v>
       </c>
       <c r="E145" t="inlineStr">
         <is>
@@ -3998,7 +3998,7 @@
     <row r="147">
       <c r="A147" t="inlineStr">
         <is>
-          <t>17:34:04</t>
+          <t>18:30:24</t>
         </is>
       </c>
       <c r="B147" t="inlineStr">
@@ -4012,7 +4012,7 @@
         </is>
       </c>
       <c r="D147" t="n">
-        <v>70</v>
+        <v>14</v>
       </c>
       <c r="E147" t="inlineStr">
         <is>
@@ -4023,7 +4023,7 @@
     <row r="148">
       <c r="A148" t="inlineStr">
         <is>
-          <t>17:34:04</t>
+          <t>18:30:24</t>
         </is>
       </c>
       <c r="B148" t="inlineStr">
@@ -4037,7 +4037,7 @@
         </is>
       </c>
       <c r="D148" t="n">
-        <v>80</v>
+        <v>24</v>
       </c>
       <c r="E148" t="inlineStr">
         <is>
@@ -4048,7 +4048,7 @@
     <row r="149">
       <c r="A149" t="inlineStr">
         <is>
-          <t>17:34:04</t>
+          <t>18:30:24</t>
         </is>
       </c>
       <c r="B149" t="inlineStr">
@@ -4062,7 +4062,7 @@
         </is>
       </c>
       <c r="D149" t="n">
-        <v>86</v>
+        <v>30</v>
       </c>
       <c r="E149" t="inlineStr">
         <is>
@@ -4073,12 +4073,12 @@
     <row r="150">
       <c r="A150" t="inlineStr">
         <is>
-          <t>17:34:04</t>
+          <t>18:30:24</t>
         </is>
       </c>
       <c r="B150" t="inlineStr">
         <is>
-          <t>19:05</t>
+          <t>19:04</t>
         </is>
       </c>
       <c r="C150" t="inlineStr">
@@ -4087,7 +4087,7 @@
         </is>
       </c>
       <c r="D150" t="n">
-        <v>91</v>
+        <v>34</v>
       </c>
       <c r="E150" t="inlineStr">
         <is>
@@ -4103,16 +4103,16 @@
       </c>
       <c r="B151" t="inlineStr">
         <is>
-          <t>19:12</t>
+          <t>19:05</t>
         </is>
       </c>
       <c r="C151" t="inlineStr">
         <is>
-          <t>23_HERNANDEZ</t>
+          <t>14_ABASTO</t>
         </is>
       </c>
       <c r="D151" t="n">
-        <v>98</v>
+        <v>91</v>
       </c>
       <c r="E151" t="inlineStr">
         <is>
@@ -4123,21 +4123,21 @@
     <row r="152">
       <c r="A152" t="inlineStr">
         <is>
-          <t>17:34:04</t>
+          <t>18:30:24</t>
         </is>
       </c>
       <c r="B152" t="inlineStr">
         <is>
-          <t>19:16</t>
+          <t>19:11</t>
         </is>
       </c>
       <c r="C152" t="inlineStr">
         <is>
-          <t>16_SANTA ANA</t>
+          <t>23_HERNANDEZ</t>
         </is>
       </c>
       <c r="D152" t="n">
-        <v>102</v>
+        <v>41</v>
       </c>
       <c r="E152" t="inlineStr">
         <is>
@@ -4153,16 +4153,16 @@
       </c>
       <c r="B153" t="inlineStr">
         <is>
-          <t>19:17</t>
+          <t>19:12</t>
         </is>
       </c>
       <c r="C153" t="inlineStr">
         <is>
-          <t>27_EL RETIRO</t>
+          <t>23_HERNANDEZ</t>
         </is>
       </c>
       <c r="D153" t="n">
-        <v>103</v>
+        <v>98</v>
       </c>
       <c r="E153" t="inlineStr">
         <is>
@@ -4173,21 +4173,21 @@
     <row r="154">
       <c r="A154" t="inlineStr">
         <is>
-          <t>17:34:04</t>
+          <t>18:30:24</t>
         </is>
       </c>
       <c r="B154" t="inlineStr">
         <is>
-          <t>19:24</t>
+          <t>19:16</t>
         </is>
       </c>
       <c r="C154" t="inlineStr">
         <is>
-          <t>11X44_ETCHEVERRY</t>
+          <t>16_SANTA ANA</t>
         </is>
       </c>
       <c r="D154" t="n">
-        <v>110</v>
+        <v>46</v>
       </c>
       <c r="E154" t="inlineStr">
         <is>
@@ -4198,23 +4198,198 @@
     <row r="155">
       <c r="A155" t="inlineStr">
         <is>
-          <t>17:34:04</t>
+          <t>18:30:24</t>
         </is>
       </c>
       <c r="B155" t="inlineStr">
         <is>
+          <t>19:17</t>
+        </is>
+      </c>
+      <c r="C155" t="inlineStr">
+        <is>
+          <t>27_EL RETIRO</t>
+        </is>
+      </c>
+      <c r="D155" t="n">
+        <v>47</v>
+      </c>
+      <c r="E155" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="156">
+      <c r="A156" t="inlineStr">
+        <is>
+          <t>18:30:24</t>
+        </is>
+      </c>
+      <c r="B156" t="inlineStr">
+        <is>
+          <t>19:24</t>
+        </is>
+      </c>
+      <c r="C156" t="inlineStr">
+        <is>
+          <t>11X44_ETCHEVERRY</t>
+        </is>
+      </c>
+      <c r="D156" t="n">
+        <v>54</v>
+      </c>
+      <c r="E156" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="157">
+      <c r="A157" t="inlineStr">
+        <is>
+          <t>18:30:24</t>
+        </is>
+      </c>
+      <c r="B157" t="inlineStr">
+        <is>
           <t>19:25</t>
         </is>
       </c>
-      <c r="C155" t="inlineStr">
+      <c r="C157" t="inlineStr">
         <is>
           <t>215C_EL PATO</t>
         </is>
       </c>
-      <c r="D155" t="n">
-        <v>111</v>
-      </c>
-      <c r="E155" t="inlineStr">
+      <c r="D157" t="n">
+        <v>55</v>
+      </c>
+      <c r="E157" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="158">
+      <c r="A158" t="inlineStr">
+        <is>
+          <t>18:30:24</t>
+        </is>
+      </c>
+      <c r="B158" t="inlineStr">
+        <is>
+          <t>19:49</t>
+        </is>
+      </c>
+      <c r="C158" t="inlineStr">
+        <is>
+          <t>225_GOMEZ</t>
+        </is>
+      </c>
+      <c r="D158" t="n">
+        <v>79</v>
+      </c>
+      <c r="E158" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="159">
+      <c r="A159" t="inlineStr">
+        <is>
+          <t>18:30:24</t>
+        </is>
+      </c>
+      <c r="B159" t="inlineStr">
+        <is>
+          <t>19:50</t>
+        </is>
+      </c>
+      <c r="C159" t="inlineStr">
+        <is>
+          <t>81_EL PELIGRO</t>
+        </is>
+      </c>
+      <c r="D159" t="n">
+        <v>80</v>
+      </c>
+      <c r="E159" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="160">
+      <c r="A160" t="inlineStr">
+        <is>
+          <t>18:30:24</t>
+        </is>
+      </c>
+      <c r="B160" t="inlineStr">
+        <is>
+          <t>20:07</t>
+        </is>
+      </c>
+      <c r="C160" t="inlineStr">
+        <is>
+          <t>23_HERNANDEZ</t>
+        </is>
+      </c>
+      <c r="D160" t="n">
+        <v>97</v>
+      </c>
+      <c r="E160" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="161">
+      <c r="A161" t="inlineStr">
+        <is>
+          <t>18:30:24</t>
+        </is>
+      </c>
+      <c r="B161" t="inlineStr">
+        <is>
+          <t>20:15</t>
+        </is>
+      </c>
+      <c r="C161" t="inlineStr">
+        <is>
+          <t>14_ABASTO</t>
+        </is>
+      </c>
+      <c r="D161" t="n">
+        <v>105</v>
+      </c>
+      <c r="E161" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="162">
+      <c r="A162" t="inlineStr">
+        <is>
+          <t>18:30:24</t>
+        </is>
+      </c>
+      <c r="B162" t="inlineStr">
+        <is>
+          <t>20:15</t>
+        </is>
+      </c>
+      <c r="C162" t="inlineStr">
+        <is>
+          <t>215C_EL PATO</t>
+        </is>
+      </c>
+      <c r="D162" t="n">
+        <v>105</v>
+      </c>
+      <c r="E162" t="inlineStr">
         <is>
           <t>LP1912</t>
         </is>
@@ -4231,7 +4406,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E34"/>
+  <dimension ref="A1:E35"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -4244,14 +4419,14 @@
     <row r="2">
       <c r="A2" s="1" t="inlineStr">
         <is>
-          <t>Última actualización: 17:34:04</t>
+          <t>Última actualización: 18:30:24</t>
         </is>
       </c>
     </row>
     <row r="3">
       <c r="A3" s="1" t="inlineStr">
         <is>
-          <t>Total filas: 29</t>
+          <t>Total filas: 30</t>
         </is>
       </c>
     </row>
@@ -4960,7 +5135,7 @@
     <row r="33">
       <c r="A33" t="inlineStr">
         <is>
-          <t>17:34:04</t>
+          <t>18:30:24</t>
         </is>
       </c>
       <c r="B33" t="inlineStr">
@@ -4974,7 +5149,7 @@
         </is>
       </c>
       <c r="D33" t="n">
-        <v>86</v>
+        <v>30</v>
       </c>
       <c r="E33" t="inlineStr">
         <is>
@@ -4985,7 +5160,7 @@
     <row r="34">
       <c r="A34" t="inlineStr">
         <is>
-          <t>17:34:04</t>
+          <t>18:30:24</t>
         </is>
       </c>
       <c r="B34" t="inlineStr">
@@ -4999,9 +5174,34 @@
         </is>
       </c>
       <c r="D34" t="n">
-        <v>111</v>
+        <v>55</v>
       </c>
       <c r="E34" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="35">
+      <c r="A35" t="inlineStr">
+        <is>
+          <t>18:30:24</t>
+        </is>
+      </c>
+      <c r="B35" t="inlineStr">
+        <is>
+          <t>20:15</t>
+        </is>
+      </c>
+      <c r="C35" t="inlineStr">
+        <is>
+          <t>215C_EL PATO</t>
+        </is>
+      </c>
+      <c r="D35" t="n">
+        <v>105</v>
+      </c>
+      <c r="E35" t="inlineStr">
         <is>
           <t>LP1912</t>
         </is>
@@ -5018,7 +5218,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E31"/>
+  <dimension ref="A1:E32"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -5031,14 +5231,14 @@
     <row r="2">
       <c r="A2" s="1" t="inlineStr">
         <is>
-          <t>Última actualización: 17:34:04</t>
+          <t>Última actualización: 18:30:24</t>
         </is>
       </c>
     </row>
     <row r="3">
       <c r="A3" s="1" t="inlineStr">
         <is>
-          <t>Total filas: 26</t>
+          <t>Total filas: 27</t>
         </is>
       </c>
     </row>
@@ -5672,7 +5872,7 @@
     <row r="30">
       <c r="A30" t="inlineStr">
         <is>
-          <t>17:34:04</t>
+          <t>18:30:24</t>
         </is>
       </c>
       <c r="B30" t="inlineStr">
@@ -5686,7 +5886,7 @@
         </is>
       </c>
       <c r="D30" t="n">
-        <v>71</v>
+        <v>15</v>
       </c>
       <c r="E30" t="inlineStr">
         <is>
@@ -5697,7 +5897,7 @@
     <row r="31">
       <c r="A31" t="inlineStr">
         <is>
-          <t>17:34:04</t>
+          <t>18:30:24</t>
         </is>
       </c>
       <c r="B31" t="inlineStr">
@@ -5711,11 +5911,36 @@
         </is>
       </c>
       <c r="D31" t="n">
-        <v>101</v>
+        <v>45</v>
       </c>
       <c r="E31" t="inlineStr">
         <is>
           <t>L6173</t>
+        </is>
+      </c>
+    </row>
+    <row r="32">
+      <c r="A32" t="inlineStr">
+        <is>
+          <t>18:30:24</t>
+        </is>
+      </c>
+      <c r="B32" t="inlineStr">
+        <is>
+          <t>19:47</t>
+        </is>
+      </c>
+      <c r="C32" t="inlineStr">
+        <is>
+          <t>215C_LA PLATA</t>
+        </is>
+      </c>
+      <c r="D32" t="n">
+        <v>77</v>
+      </c>
+      <c r="E32" t="inlineStr">
+        <is>
+          <t>L6203</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
📊 Horarios actualizados Línea 141 - 3038
</commit_message>
<xml_diff>
--- a/data/horarios-141-2026-05-17.xlsx
+++ b/data/horarios-141-2026-05-17.xlsx
@@ -419,7 +419,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E162"/>
+  <dimension ref="A1:E172"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -432,14 +432,14 @@
     <row r="2">
       <c r="A2" s="1" t="inlineStr">
         <is>
-          <t>Última actualización: 18:30:24</t>
+          <t>Última actualización: 19:29:32</t>
         </is>
       </c>
     </row>
     <row r="3">
       <c r="A3" s="1" t="inlineStr">
         <is>
-          <t>Total filas: 157</t>
+          <t>Total filas: 167</t>
         </is>
       </c>
     </row>
@@ -958,7 +958,7 @@
       </c>
       <c r="C25" t="inlineStr">
         <is>
-          <t>215C_EL PATO</t>
+          <t>215B_EL PATO</t>
         </is>
       </c>
       <c r="D25" t="n">
@@ -983,7 +983,7 @@
       </c>
       <c r="C26" t="inlineStr">
         <is>
-          <t>215B_EL PATO</t>
+          <t>215C_EL PATO</t>
         </is>
       </c>
       <c r="D26" t="n">
@@ -1108,7 +1108,7 @@
       </c>
       <c r="C31" t="inlineStr">
         <is>
-          <t>27_EL RETIRO</t>
+          <t>16_SANTA ANA</t>
         </is>
       </c>
       <c r="D31" t="n">
@@ -1133,7 +1133,7 @@
       </c>
       <c r="C32" t="inlineStr">
         <is>
-          <t>16_SANTA ANA</t>
+          <t>27_EL RETIRO</t>
         </is>
       </c>
       <c r="D32" t="n">
@@ -4273,21 +4273,21 @@
     <row r="158">
       <c r="A158" t="inlineStr">
         <is>
-          <t>18:30:24</t>
+          <t>19:29:32</t>
         </is>
       </c>
       <c r="B158" t="inlineStr">
         <is>
-          <t>19:49</t>
+          <t>19:29</t>
         </is>
       </c>
       <c r="C158" t="inlineStr">
         <is>
-          <t>225_GOMEZ</t>
+          <t>27_EL RETIRO</t>
         </is>
       </c>
       <c r="D158" t="n">
-        <v>79</v>
+        <v>0</v>
       </c>
       <c r="E158" t="inlineStr">
         <is>
@@ -4298,21 +4298,21 @@
     <row r="159">
       <c r="A159" t="inlineStr">
         <is>
-          <t>18:30:24</t>
+          <t>19:29:32</t>
         </is>
       </c>
       <c r="B159" t="inlineStr">
         <is>
-          <t>19:50</t>
+          <t>19:49</t>
         </is>
       </c>
       <c r="C159" t="inlineStr">
         <is>
-          <t>81_EL PELIGRO</t>
+          <t>225_GOMEZ</t>
         </is>
       </c>
       <c r="D159" t="n">
-        <v>80</v>
+        <v>20</v>
       </c>
       <c r="E159" t="inlineStr">
         <is>
@@ -4323,21 +4323,21 @@
     <row r="160">
       <c r="A160" t="inlineStr">
         <is>
-          <t>18:30:24</t>
+          <t>19:29:32</t>
         </is>
       </c>
       <c r="B160" t="inlineStr">
         <is>
-          <t>20:07</t>
+          <t>19:50</t>
         </is>
       </c>
       <c r="C160" t="inlineStr">
         <is>
-          <t>23_HERNANDEZ</t>
+          <t>81_EL PELIGRO</t>
         </is>
       </c>
       <c r="D160" t="n">
-        <v>97</v>
+        <v>21</v>
       </c>
       <c r="E160" t="inlineStr">
         <is>
@@ -4348,21 +4348,21 @@
     <row r="161">
       <c r="A161" t="inlineStr">
         <is>
-          <t>18:30:24</t>
+          <t>19:29:32</t>
         </is>
       </c>
       <c r="B161" t="inlineStr">
         <is>
-          <t>20:15</t>
+          <t>19:56</t>
         </is>
       </c>
       <c r="C161" t="inlineStr">
         <is>
-          <t>14_ABASTO</t>
+          <t>16_SANTA ANA</t>
         </is>
       </c>
       <c r="D161" t="n">
-        <v>105</v>
+        <v>27</v>
       </c>
       <c r="E161" t="inlineStr">
         <is>
@@ -4373,23 +4373,273 @@
     <row r="162">
       <c r="A162" t="inlineStr">
         <is>
+          <t>19:29:32</t>
+        </is>
+      </c>
+      <c r="B162" t="inlineStr">
+        <is>
+          <t>20:01</t>
+        </is>
+      </c>
+      <c r="C162" t="inlineStr">
+        <is>
+          <t>23_HERNANDEZ</t>
+        </is>
+      </c>
+      <c r="D162" t="n">
+        <v>32</v>
+      </c>
+      <c r="E162" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="163">
+      <c r="A163" t="inlineStr">
+        <is>
           <t>18:30:24</t>
         </is>
       </c>
-      <c r="B162" t="inlineStr">
+      <c r="B163" t="inlineStr">
+        <is>
+          <t>20:07</t>
+        </is>
+      </c>
+      <c r="C163" t="inlineStr">
+        <is>
+          <t>23_HERNANDEZ</t>
+        </is>
+      </c>
+      <c r="D163" t="n">
+        <v>97</v>
+      </c>
+      <c r="E163" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="164">
+      <c r="A164" t="inlineStr">
+        <is>
+          <t>19:29:32</t>
+        </is>
+      </c>
+      <c r="B164" t="inlineStr">
         <is>
           <t>20:15</t>
         </is>
       </c>
-      <c r="C162" t="inlineStr">
+      <c r="C164" t="inlineStr">
+        <is>
+          <t>14_ABASTO</t>
+        </is>
+      </c>
+      <c r="D164" t="n">
+        <v>46</v>
+      </c>
+      <c r="E164" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="165">
+      <c r="A165" t="inlineStr">
+        <is>
+          <t>19:29:32</t>
+        </is>
+      </c>
+      <c r="B165" t="inlineStr">
+        <is>
+          <t>20:15</t>
+        </is>
+      </c>
+      <c r="C165" t="inlineStr">
         <is>
           <t>215C_EL PATO</t>
         </is>
       </c>
-      <c r="D162" t="n">
-        <v>105</v>
-      </c>
-      <c r="E162" t="inlineStr">
+      <c r="D165" t="n">
+        <v>46</v>
+      </c>
+      <c r="E165" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="166">
+      <c r="A166" t="inlineStr">
+        <is>
+          <t>19:29:32</t>
+        </is>
+      </c>
+      <c r="B166" t="inlineStr">
+        <is>
+          <t>20:36</t>
+        </is>
+      </c>
+      <c r="C166" t="inlineStr">
+        <is>
+          <t>16_SANTA ANA</t>
+        </is>
+      </c>
+      <c r="D166" t="n">
+        <v>67</v>
+      </c>
+      <c r="E166" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="167">
+      <c r="A167" t="inlineStr">
+        <is>
+          <t>19:29:32</t>
+        </is>
+      </c>
+      <c r="B167" t="inlineStr">
+        <is>
+          <t>20:39</t>
+        </is>
+      </c>
+      <c r="C167" t="inlineStr">
+        <is>
+          <t>215B_EL PATO</t>
+        </is>
+      </c>
+      <c r="D167" t="n">
+        <v>70</v>
+      </c>
+      <c r="E167" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="168">
+      <c r="A168" t="inlineStr">
+        <is>
+          <t>19:29:32</t>
+        </is>
+      </c>
+      <c r="B168" t="inlineStr">
+        <is>
+          <t>20:42</t>
+        </is>
+      </c>
+      <c r="C168" t="inlineStr">
+        <is>
+          <t>15_ABASTO</t>
+        </is>
+      </c>
+      <c r="D168" t="n">
+        <v>73</v>
+      </c>
+      <c r="E168" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="169">
+      <c r="A169" t="inlineStr">
+        <is>
+          <t>19:29:32</t>
+        </is>
+      </c>
+      <c r="B169" t="inlineStr">
+        <is>
+          <t>20:51</t>
+        </is>
+      </c>
+      <c r="C169" t="inlineStr">
+        <is>
+          <t>23_HERNANDEZ</t>
+        </is>
+      </c>
+      <c r="D169" t="n">
+        <v>82</v>
+      </c>
+      <c r="E169" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="170">
+      <c r="A170" t="inlineStr">
+        <is>
+          <t>19:29:32</t>
+        </is>
+      </c>
+      <c r="B170" t="inlineStr">
+        <is>
+          <t>20:56</t>
+        </is>
+      </c>
+      <c r="C170" t="inlineStr">
+        <is>
+          <t>27_EL RETIRO</t>
+        </is>
+      </c>
+      <c r="D170" t="n">
+        <v>87</v>
+      </c>
+      <c r="E170" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="171">
+      <c r="A171" t="inlineStr">
+        <is>
+          <t>19:29:32</t>
+        </is>
+      </c>
+      <c r="B171" t="inlineStr">
+        <is>
+          <t>21:05</t>
+        </is>
+      </c>
+      <c r="C171" t="inlineStr">
+        <is>
+          <t>10_OLMOS</t>
+        </is>
+      </c>
+      <c r="D171" t="n">
+        <v>96</v>
+      </c>
+      <c r="E171" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="172">
+      <c r="A172" t="inlineStr">
+        <is>
+          <t>19:29:32</t>
+        </is>
+      </c>
+      <c r="B172" t="inlineStr">
+        <is>
+          <t>21:07</t>
+        </is>
+      </c>
+      <c r="C172" t="inlineStr">
+        <is>
+          <t>15_ABASTO</t>
+        </is>
+      </c>
+      <c r="D172" t="n">
+        <v>98</v>
+      </c>
+      <c r="E172" t="inlineStr">
         <is>
           <t>LP1912</t>
         </is>
@@ -4406,7 +4656,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E35"/>
+  <dimension ref="A1:E36"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -4419,14 +4669,14 @@
     <row r="2">
       <c r="A2" s="1" t="inlineStr">
         <is>
-          <t>Última actualización: 18:30:24</t>
+          <t>Última actualización: 19:29:32</t>
         </is>
       </c>
     </row>
     <row r="3">
       <c r="A3" s="1" t="inlineStr">
         <is>
-          <t>Total filas: 30</t>
+          <t>Total filas: 31</t>
         </is>
       </c>
     </row>
@@ -5185,7 +5435,7 @@
     <row r="35">
       <c r="A35" t="inlineStr">
         <is>
-          <t>18:30:24</t>
+          <t>19:29:32</t>
         </is>
       </c>
       <c r="B35" t="inlineStr">
@@ -5199,9 +5449,34 @@
         </is>
       </c>
       <c r="D35" t="n">
-        <v>105</v>
+        <v>46</v>
       </c>
       <c r="E35" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="36">
+      <c r="A36" t="inlineStr">
+        <is>
+          <t>19:29:32</t>
+        </is>
+      </c>
+      <c r="B36" t="inlineStr">
+        <is>
+          <t>20:39</t>
+        </is>
+      </c>
+      <c r="C36" t="inlineStr">
+        <is>
+          <t>215B_EL PATO</t>
+        </is>
+      </c>
+      <c r="D36" t="n">
+        <v>70</v>
+      </c>
+      <c r="E36" t="inlineStr">
         <is>
           <t>LP1912</t>
         </is>
@@ -5218,7 +5493,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E32"/>
+  <dimension ref="A1:E33"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -5231,14 +5506,14 @@
     <row r="2">
       <c r="A2" s="1" t="inlineStr">
         <is>
-          <t>Última actualización: 18:30:24</t>
+          <t>Última actualización: 19:29:32</t>
         </is>
       </c>
     </row>
     <row r="3">
       <c r="A3" s="1" t="inlineStr">
         <is>
-          <t>Total filas: 27</t>
+          <t>Total filas: 28</t>
         </is>
       </c>
     </row>
@@ -5922,7 +6197,7 @@
     <row r="32">
       <c r="A32" t="inlineStr">
         <is>
-          <t>18:30:24</t>
+          <t>19:29:32</t>
         </is>
       </c>
       <c r="B32" t="inlineStr">
@@ -5936,9 +6211,34 @@
         </is>
       </c>
       <c r="D32" t="n">
-        <v>77</v>
+        <v>18</v>
       </c>
       <c r="E32" t="inlineStr">
+        <is>
+          <t>L6203</t>
+        </is>
+      </c>
+    </row>
+    <row r="33">
+      <c r="A33" t="inlineStr">
+        <is>
+          <t>19:29:32</t>
+        </is>
+      </c>
+      <c r="B33" t="inlineStr">
+        <is>
+          <t>20:39</t>
+        </is>
+      </c>
+      <c r="C33" t="inlineStr">
+        <is>
+          <t>215C_LA PLATA</t>
+        </is>
+      </c>
+      <c r="D33" t="n">
+        <v>70</v>
+      </c>
+      <c r="E33" t="inlineStr">
         <is>
           <t>L6203</t>
         </is>

</xml_diff>

<commit_message>
📊 Horarios actualizados Línea 141 - 3039
</commit_message>
<xml_diff>
--- a/data/horarios-141-2026-05-17.xlsx
+++ b/data/horarios-141-2026-05-17.xlsx
@@ -419,7 +419,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E172"/>
+  <dimension ref="A1:E178"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -432,14 +432,14 @@
     <row r="2">
       <c r="A2" s="1" t="inlineStr">
         <is>
-          <t>Última actualización: 19:29:32</t>
+          <t>Última actualización: 20:29:27</t>
         </is>
       </c>
     </row>
     <row r="3">
       <c r="A3" s="1" t="inlineStr">
         <is>
-          <t>Total filas: 167</t>
+          <t>Total filas: 173</t>
         </is>
       </c>
     </row>
@@ -958,7 +958,7 @@
       </c>
       <c r="C25" t="inlineStr">
         <is>
-          <t>215B_EL PATO</t>
+          <t>215C_EL PATO</t>
         </is>
       </c>
       <c r="D25" t="n">
@@ -983,7 +983,7 @@
       </c>
       <c r="C26" t="inlineStr">
         <is>
-          <t>215C_EL PATO</t>
+          <t>215B_EL PATO</t>
         </is>
       </c>
       <c r="D26" t="n">
@@ -4473,7 +4473,7 @@
     <row r="166">
       <c r="A166" t="inlineStr">
         <is>
-          <t>19:29:32</t>
+          <t>20:29:27</t>
         </is>
       </c>
       <c r="B166" t="inlineStr">
@@ -4487,7 +4487,7 @@
         </is>
       </c>
       <c r="D166" t="n">
-        <v>67</v>
+        <v>7</v>
       </c>
       <c r="E166" t="inlineStr">
         <is>
@@ -4498,7 +4498,7 @@
     <row r="167">
       <c r="A167" t="inlineStr">
         <is>
-          <t>19:29:32</t>
+          <t>20:29:27</t>
         </is>
       </c>
       <c r="B167" t="inlineStr">
@@ -4512,7 +4512,7 @@
         </is>
       </c>
       <c r="D167" t="n">
-        <v>70</v>
+        <v>10</v>
       </c>
       <c r="E167" t="inlineStr">
         <is>
@@ -4523,7 +4523,7 @@
     <row r="168">
       <c r="A168" t="inlineStr">
         <is>
-          <t>19:29:32</t>
+          <t>20:29:27</t>
         </is>
       </c>
       <c r="B168" t="inlineStr">
@@ -4537,7 +4537,7 @@
         </is>
       </c>
       <c r="D168" t="n">
-        <v>73</v>
+        <v>13</v>
       </c>
       <c r="E168" t="inlineStr">
         <is>
@@ -4548,7 +4548,7 @@
     <row r="169">
       <c r="A169" t="inlineStr">
         <is>
-          <t>19:29:32</t>
+          <t>20:29:27</t>
         </is>
       </c>
       <c r="B169" t="inlineStr">
@@ -4562,7 +4562,7 @@
         </is>
       </c>
       <c r="D169" t="n">
-        <v>82</v>
+        <v>22</v>
       </c>
       <c r="E169" t="inlineStr">
         <is>
@@ -4573,7 +4573,7 @@
     <row r="170">
       <c r="A170" t="inlineStr">
         <is>
-          <t>19:29:32</t>
+          <t>20:29:27</t>
         </is>
       </c>
       <c r="B170" t="inlineStr">
@@ -4587,7 +4587,7 @@
         </is>
       </c>
       <c r="D170" t="n">
-        <v>87</v>
+        <v>27</v>
       </c>
       <c r="E170" t="inlineStr">
         <is>
@@ -4598,7 +4598,7 @@
     <row r="171">
       <c r="A171" t="inlineStr">
         <is>
-          <t>19:29:32</t>
+          <t>20:29:27</t>
         </is>
       </c>
       <c r="B171" t="inlineStr">
@@ -4612,7 +4612,7 @@
         </is>
       </c>
       <c r="D171" t="n">
-        <v>96</v>
+        <v>36</v>
       </c>
       <c r="E171" t="inlineStr">
         <is>
@@ -4623,7 +4623,7 @@
     <row r="172">
       <c r="A172" t="inlineStr">
         <is>
-          <t>19:29:32</t>
+          <t>20:29:27</t>
         </is>
       </c>
       <c r="B172" t="inlineStr">
@@ -4637,9 +4637,159 @@
         </is>
       </c>
       <c r="D172" t="n">
-        <v>98</v>
+        <v>38</v>
       </c>
       <c r="E172" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="173">
+      <c r="A173" t="inlineStr">
+        <is>
+          <t>20:29:27</t>
+        </is>
+      </c>
+      <c r="B173" t="inlineStr">
+        <is>
+          <t>21:34</t>
+        </is>
+      </c>
+      <c r="C173" t="inlineStr">
+        <is>
+          <t>11_ETCHEVERRY</t>
+        </is>
+      </c>
+      <c r="D173" t="n">
+        <v>65</v>
+      </c>
+      <c r="E173" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="174">
+      <c r="A174" t="inlineStr">
+        <is>
+          <t>20:29:27</t>
+        </is>
+      </c>
+      <c r="B174" t="inlineStr">
+        <is>
+          <t>21:36</t>
+        </is>
+      </c>
+      <c r="C174" t="inlineStr">
+        <is>
+          <t>16_SANTA ANA</t>
+        </is>
+      </c>
+      <c r="D174" t="n">
+        <v>67</v>
+      </c>
+      <c r="E174" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="175">
+      <c r="A175" t="inlineStr">
+        <is>
+          <t>20:29:27</t>
+        </is>
+      </c>
+      <c r="B175" t="inlineStr">
+        <is>
+          <t>21:37</t>
+        </is>
+      </c>
+      <c r="C175" t="inlineStr">
+        <is>
+          <t>84_COLONIA URQUIZA-ESC 49</t>
+        </is>
+      </c>
+      <c r="D175" t="n">
+        <v>68</v>
+      </c>
+      <c r="E175" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="176">
+      <c r="A176" t="inlineStr">
+        <is>
+          <t>20:29:27</t>
+        </is>
+      </c>
+      <c r="B176" t="inlineStr">
+        <is>
+          <t>21:43</t>
+        </is>
+      </c>
+      <c r="C176" t="inlineStr">
+        <is>
+          <t>23_HERNANDEZ</t>
+        </is>
+      </c>
+      <c r="D176" t="n">
+        <v>74</v>
+      </c>
+      <c r="E176" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="177">
+      <c r="A177" t="inlineStr">
+        <is>
+          <t>20:29:27</t>
+        </is>
+      </c>
+      <c r="B177" t="inlineStr">
+        <is>
+          <t>21:59</t>
+        </is>
+      </c>
+      <c r="C177" t="inlineStr">
+        <is>
+          <t>14X44_ABASTO</t>
+        </is>
+      </c>
+      <c r="D177" t="n">
+        <v>90</v>
+      </c>
+      <c r="E177" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="178">
+      <c r="A178" t="inlineStr">
+        <is>
+          <t>20:29:27</t>
+        </is>
+      </c>
+      <c r="B178" t="inlineStr">
+        <is>
+          <t>22:26</t>
+        </is>
+      </c>
+      <c r="C178" t="inlineStr">
+        <is>
+          <t>14_ABASTO</t>
+        </is>
+      </c>
+      <c r="D178" t="n">
+        <v>117</v>
+      </c>
+      <c r="E178" t="inlineStr">
         <is>
           <t>LP1912</t>
         </is>
@@ -4669,7 +4819,7 @@
     <row r="2">
       <c r="A2" s="1" t="inlineStr">
         <is>
-          <t>Última actualización: 19:29:32</t>
+          <t>Última actualización: 20:29:27</t>
         </is>
       </c>
     </row>
@@ -5460,7 +5610,7 @@
     <row r="36">
       <c r="A36" t="inlineStr">
         <is>
-          <t>19:29:32</t>
+          <t>20:29:27</t>
         </is>
       </c>
       <c r="B36" t="inlineStr">
@@ -5474,7 +5624,7 @@
         </is>
       </c>
       <c r="D36" t="n">
-        <v>70</v>
+        <v>10</v>
       </c>
       <c r="E36" t="inlineStr">
         <is>
@@ -5493,7 +5643,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E33"/>
+  <dimension ref="A1:E35"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -5506,14 +5656,14 @@
     <row r="2">
       <c r="A2" s="1" t="inlineStr">
         <is>
-          <t>Última actualización: 19:29:32</t>
+          <t>Última actualización: 20:29:27</t>
         </is>
       </c>
     </row>
     <row r="3">
       <c r="A3" s="1" t="inlineStr">
         <is>
-          <t>Total filas: 28</t>
+          <t>Total filas: 30</t>
         </is>
       </c>
     </row>
@@ -6222,7 +6372,7 @@
     <row r="33">
       <c r="A33" t="inlineStr">
         <is>
-          <t>19:29:32</t>
+          <t>20:29:27</t>
         </is>
       </c>
       <c r="B33" t="inlineStr">
@@ -6236,11 +6386,61 @@
         </is>
       </c>
       <c r="D33" t="n">
-        <v>70</v>
+        <v>10</v>
       </c>
       <c r="E33" t="inlineStr">
         <is>
           <t>L6203</t>
+        </is>
+      </c>
+    </row>
+    <row r="34">
+      <c r="A34" t="inlineStr">
+        <is>
+          <t>20:29:27</t>
+        </is>
+      </c>
+      <c r="B34" t="inlineStr">
+        <is>
+          <t>21:32</t>
+        </is>
+      </c>
+      <c r="C34" t="inlineStr">
+        <is>
+          <t>215C_LA PLATA</t>
+        </is>
+      </c>
+      <c r="D34" t="n">
+        <v>63</v>
+      </c>
+      <c r="E34" t="inlineStr">
+        <is>
+          <t>L6203</t>
+        </is>
+      </c>
+    </row>
+    <row r="35">
+      <c r="A35" t="inlineStr">
+        <is>
+          <t>20:29:27</t>
+        </is>
+      </c>
+      <c r="B35" t="inlineStr">
+        <is>
+          <t>22:09</t>
+        </is>
+      </c>
+      <c r="C35" t="inlineStr">
+        <is>
+          <t>215B_LP-P MOR-40 Y 115</t>
+        </is>
+      </c>
+      <c r="D35" t="n">
+        <v>100</v>
+      </c>
+      <c r="E35" t="inlineStr">
+        <is>
+          <t>L6173</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
📊 Horarios actualizados Línea 141 - 3040
</commit_message>
<xml_diff>
--- a/data/horarios-141-2026-05-17.xlsx
+++ b/data/horarios-141-2026-05-17.xlsx
@@ -419,7 +419,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E178"/>
+  <dimension ref="A1:E187"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -432,14 +432,14 @@
     <row r="2">
       <c r="A2" s="1" t="inlineStr">
         <is>
-          <t>Última actualización: 20:29:27</t>
+          <t>Última actualización: 22:27:04</t>
         </is>
       </c>
     </row>
     <row r="3">
       <c r="A3" s="1" t="inlineStr">
         <is>
-          <t>Total filas: 173</t>
+          <t>Total filas: 182</t>
         </is>
       </c>
     </row>
@@ -958,7 +958,7 @@
       </c>
       <c r="C25" t="inlineStr">
         <is>
-          <t>215C_EL PATO</t>
+          <t>215B_EL PATO</t>
         </is>
       </c>
       <c r="D25" t="n">
@@ -983,7 +983,7 @@
       </c>
       <c r="C26" t="inlineStr">
         <is>
-          <t>215B_EL PATO</t>
+          <t>215C_EL PATO</t>
         </is>
       </c>
       <c r="D26" t="n">
@@ -2508,7 +2508,7 @@
       </c>
       <c r="C87" t="inlineStr">
         <is>
-          <t>16_P MOR-SANTA ANA</t>
+          <t>15X38_ABASTO</t>
         </is>
       </c>
       <c r="D87" t="n">
@@ -2533,7 +2533,7 @@
       </c>
       <c r="C88" t="inlineStr">
         <is>
-          <t>15X38_ABASTO</t>
+          <t>16_P MOR-SANTA ANA</t>
         </is>
       </c>
       <c r="D88" t="n">
@@ -4790,6 +4790,231 @@
         <v>117</v>
       </c>
       <c r="E178" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="179">
+      <c r="A179" t="inlineStr">
+        <is>
+          <t>22:27:04</t>
+        </is>
+      </c>
+      <c r="B179" t="inlineStr">
+        <is>
+          <t>22:35</t>
+        </is>
+      </c>
+      <c r="C179" t="inlineStr">
+        <is>
+          <t>23_HERNANDEZ</t>
+        </is>
+      </c>
+      <c r="D179" t="n">
+        <v>8</v>
+      </c>
+      <c r="E179" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="180">
+      <c r="A180" t="inlineStr">
+        <is>
+          <t>22:27:04</t>
+        </is>
+      </c>
+      <c r="B180" t="inlineStr">
+        <is>
+          <t>22:37</t>
+        </is>
+      </c>
+      <c r="C180" t="inlineStr">
+        <is>
+          <t>215C_EL PATO</t>
+        </is>
+      </c>
+      <c r="D180" t="n">
+        <v>10</v>
+      </c>
+      <c r="E180" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="181">
+      <c r="A181" t="inlineStr">
+        <is>
+          <t>22:27:04</t>
+        </is>
+      </c>
+      <c r="B181" t="inlineStr">
+        <is>
+          <t>22:43</t>
+        </is>
+      </c>
+      <c r="C181" t="inlineStr">
+        <is>
+          <t>16_SANTA ANA</t>
+        </is>
+      </c>
+      <c r="D181" t="n">
+        <v>16</v>
+      </c>
+      <c r="E181" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="182">
+      <c r="A182" t="inlineStr">
+        <is>
+          <t>22:27:04</t>
+        </is>
+      </c>
+      <c r="B182" t="inlineStr">
+        <is>
+          <t>22:56</t>
+        </is>
+      </c>
+      <c r="C182" t="inlineStr">
+        <is>
+          <t>11X44_ETCHEVERRY</t>
+        </is>
+      </c>
+      <c r="D182" t="n">
+        <v>29</v>
+      </c>
+      <c r="E182" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="183">
+      <c r="A183" t="inlineStr">
+        <is>
+          <t>22:27:04</t>
+        </is>
+      </c>
+      <c r="B183" t="inlineStr">
+        <is>
+          <t>23:07</t>
+        </is>
+      </c>
+      <c r="C183" t="inlineStr">
+        <is>
+          <t>15_ABASTO</t>
+        </is>
+      </c>
+      <c r="D183" t="n">
+        <v>40</v>
+      </c>
+      <c r="E183" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="184">
+      <c r="A184" t="inlineStr">
+        <is>
+          <t>22:27:04</t>
+        </is>
+      </c>
+      <c r="B184" t="inlineStr">
+        <is>
+          <t>23:21</t>
+        </is>
+      </c>
+      <c r="C184" t="inlineStr">
+        <is>
+          <t>15_ABASTO</t>
+        </is>
+      </c>
+      <c r="D184" t="n">
+        <v>54</v>
+      </c>
+      <c r="E184" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="185">
+      <c r="A185" t="inlineStr">
+        <is>
+          <t>22:27:04</t>
+        </is>
+      </c>
+      <c r="B185" t="inlineStr">
+        <is>
+          <t>23:26</t>
+        </is>
+      </c>
+      <c r="C185" t="inlineStr">
+        <is>
+          <t>14_ABASTO</t>
+        </is>
+      </c>
+      <c r="D185" t="n">
+        <v>59</v>
+      </c>
+      <c r="E185" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="186">
+      <c r="A186" t="inlineStr">
+        <is>
+          <t>22:27:04</t>
+        </is>
+      </c>
+      <c r="B186" t="inlineStr">
+        <is>
+          <t>23:36</t>
+        </is>
+      </c>
+      <c r="C186" t="inlineStr">
+        <is>
+          <t>16_SANTA ANA</t>
+        </is>
+      </c>
+      <c r="D186" t="n">
+        <v>69</v>
+      </c>
+      <c r="E186" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="187">
+      <c r="A187" t="inlineStr">
+        <is>
+          <t>22:27:04</t>
+        </is>
+      </c>
+      <c r="B187" t="inlineStr">
+        <is>
+          <t>23:41</t>
+        </is>
+      </c>
+      <c r="C187" t="inlineStr">
+        <is>
+          <t>215A_EL PATO</t>
+        </is>
+      </c>
+      <c r="D187" t="n">
+        <v>74</v>
+      </c>
+      <c r="E187" t="inlineStr">
         <is>
           <t>LP1912</t>
         </is>
@@ -4806,7 +5031,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E36"/>
+  <dimension ref="A1:E38"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -4819,14 +5044,14 @@
     <row r="2">
       <c r="A2" s="1" t="inlineStr">
         <is>
-          <t>Última actualización: 20:29:27</t>
+          <t>Última actualización: 22:27:04</t>
         </is>
       </c>
     </row>
     <row r="3">
       <c r="A3" s="1" t="inlineStr">
         <is>
-          <t>Total filas: 31</t>
+          <t>Total filas: 33</t>
         </is>
       </c>
     </row>
@@ -5627,6 +5852,56 @@
         <v>10</v>
       </c>
       <c r="E36" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="37">
+      <c r="A37" t="inlineStr">
+        <is>
+          <t>22:27:04</t>
+        </is>
+      </c>
+      <c r="B37" t="inlineStr">
+        <is>
+          <t>22:37</t>
+        </is>
+      </c>
+      <c r="C37" t="inlineStr">
+        <is>
+          <t>215C_EL PATO</t>
+        </is>
+      </c>
+      <c r="D37" t="n">
+        <v>10</v>
+      </c>
+      <c r="E37" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="38">
+      <c r="A38" t="inlineStr">
+        <is>
+          <t>22:27:04</t>
+        </is>
+      </c>
+      <c r="B38" t="inlineStr">
+        <is>
+          <t>23:41</t>
+        </is>
+      </c>
+      <c r="C38" t="inlineStr">
+        <is>
+          <t>215A_EL PATO</t>
+        </is>
+      </c>
+      <c r="D38" t="n">
+        <v>74</v>
+      </c>
+      <c r="E38" t="inlineStr">
         <is>
           <t>LP1912</t>
         </is>
@@ -5656,7 +5931,7 @@
     <row r="2">
       <c r="A2" s="1" t="inlineStr">
         <is>
-          <t>Última actualización: 20:29:27</t>
+          <t>Última actualización: 22:27:04</t>
         </is>
       </c>
     </row>

</xml_diff>